<commit_message>
state: 2026-09-12 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1004,7 +1004,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr">
@@ -1012,7 +1016,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>93f9967c3ceeb4efe5e6d1c216415b8cd6807a0f8e0fd3d7fdf1903530d27cc8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1160,7 +1168,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K12" s="2" t="inlineStr"/>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="2" t="inlineStr">
@@ -1168,7 +1180,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>9c071c4826e0c6bed0f851825c5a32161944e2c0e4b11ef3f0cfc8cf2321a717</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2860,7 +2876,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr"/>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
@@ -2868,7 +2888,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N46" s="2" t="inlineStr"/>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>36cfe7e7863f9d1460b8dc4a91e8c1baec01e9664a492fb99d918b34bf2b6ea3</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4448,7 +4472,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K77" s="2" t="inlineStr"/>
       <c r="L77" s="2" t="inlineStr"/>
       <c r="M77" s="2" t="inlineStr">
@@ -4456,7 +4484,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>06d65258bb5c3c186c7c7db68031023271821689fc4fbd1ea75d865b8fd282c8</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7770,7 +7802,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7834,12 +7866,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7850,7 +7882,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>bd8c1ce600109c2433e233319fc76d333941de2357bd66d5fc70ecb75ce763a2</t>
+          <t>1dafb16e91fa0cc36d0b9c3704ad9a05b61c930c1e1bd91df670520bb5c4552c</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7934,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -7970,7 +8002,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8034,7 +8066,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8368,7 +8400,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J152" s="2" t="inlineStr"/>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr">
         <is>
@@ -8380,7 +8416,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N152" s="2" t="inlineStr"/>
+      <c r="N152" s="2" t="inlineStr">
+        <is>
+          <t>ef9fc9b9318e7fb3b77d07dc231a71dfb5a7ba4d87511ec02da4b6dd33909ada</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -8428,7 +8468,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J153" s="2" t="inlineStr"/>
+      <c r="J153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K153" s="2" t="inlineStr"/>
       <c r="L153" s="2" t="inlineStr">
         <is>
@@ -8440,7 +8484,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N153" s="2" t="inlineStr"/>
+      <c r="N153" s="2" t="inlineStr">
+        <is>
+          <t>9ffe37a558c138b12b627dad42b2b5031f97c8f9606ff73420c4d90e25a5aa62</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -8488,7 +8536,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J154" s="2" t="inlineStr"/>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr">
         <is>
@@ -8500,7 +8552,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N154" s="2" t="inlineStr"/>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>74e3b917bfc2953522782bd394b0e392149cdc683ac6a8d3eb223d095317f826</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -8608,7 +8664,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J156" s="2" t="inlineStr"/>
+      <c r="J156" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr">
         <is>
@@ -8620,7 +8680,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N156" s="2" t="inlineStr"/>
+      <c r="N156" s="2" t="inlineStr">
+        <is>
+          <t>2bb9faef957b5b4e028c37084f7c639a91ae37b499fdbedde32aac91a55d488a</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -8668,7 +8732,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J157" s="2" t="inlineStr"/>
+      <c r="J157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K157" s="2" t="inlineStr"/>
       <c r="L157" s="2" t="inlineStr">
         <is>
@@ -8680,7 +8748,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N157" s="2" t="inlineStr"/>
+      <c r="N157" s="2" t="inlineStr">
+        <is>
+          <t>61d26c9a5fc173a201c91f202de53d06297ddf5de8927e930447b1b7b12f0295</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -8728,7 +8800,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J158" s="2" t="inlineStr"/>
+      <c r="J158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr">
         <is>
@@ -8740,7 +8816,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N158" s="2" t="inlineStr"/>
+      <c r="N158" s="2" t="inlineStr">
+        <is>
+          <t>a3e05e05353a3351797d1cb622c95e6275066b2d13ceb9b48d17a9f2faac0bfc</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -10412,7 +10492,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J188" s="2" t="inlineStr"/>
+      <c r="J188" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="K188" s="2" t="inlineStr"/>
       <c r="L188" s="2" t="inlineStr">
         <is>
@@ -10424,7 +10508,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N188" s="2" t="inlineStr"/>
+      <c r="N188" s="2" t="inlineStr">
+        <is>
+          <t>3124fc1887303e571edec4a48ff382f81bc987eee7f99c2c2a097ba5bbc79ba4</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N188"/>
@@ -10699,7 +10787,11 @@
           <t>anthelioncap</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -10733,7 +10825,11 @@
           <t>kalshi</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -10767,7 +10863,11 @@
           <t>Talos-Trading</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -10801,7 +10901,11 @@
           <t>voleon</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -10841,7 +10945,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10883,7 +10987,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -10925,7 +11029,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -10967,7 +11071,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11009,7 +11113,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T13:49:47+00:00</t>
+          <t>2026-09-12T11:41:26+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11049,7 +11153,11 @@
           <t>3redpartners</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11083,7 +11191,11 @@
           <t>akunacapital</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11121,7 +11233,11 @@
           <t>aqr</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11155,7 +11271,11 @@
           <t>aquaticcapitalmanagement</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11193,7 +11313,11 @@
           <t>blackedgecapital</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11231,7 +11355,11 @@
           <t>bluecrestcapitalmanagement</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11269,7 +11397,11 @@
           <t>boerboeltrading</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11307,7 +11439,11 @@
           <t>chicagotrading</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11341,7 +11477,11 @@
           <t>drweng</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11375,7 +11515,11 @@
           <t>dvtrading</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11413,7 +11557,11 @@
           <t>engineersgate</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11451,7 +11599,11 @@
           <t>exoduspoint</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11485,7 +11637,11 @@
           <t>fiveringsllc</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11519,7 +11675,11 @@
           <t>flowtraders</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11557,7 +11717,11 @@
           <t>gelbergroup</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11591,7 +11755,11 @@
           <t>genevatrading</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11629,7 +11797,11 @@
           <t>gsacapital</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11663,7 +11835,11 @@
           <t>hyannisportresearch</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11697,7 +11873,11 @@
           <t>imc</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11731,7 +11911,11 @@
           <t>janestreet</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11769,7 +11953,11 @@
           <t>jumpcrypto</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11803,7 +11991,11 @@
           <t>jumptrading</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11841,7 +12033,11 @@
           <t>mako</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11879,7 +12075,11 @@
           <t>mangroup</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11913,7 +12113,11 @@
           <t>mavensecuritiesholdingltd</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11947,7 +12151,11 @@
           <t>oldmissioncapital</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -11981,7 +12189,11 @@
           <t>optiverprivate</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12019,7 +12231,11 @@
           <t>optiverus</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12053,7 +12269,11 @@
           <t>pdtpartners</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12091,7 +12311,11 @@
           <t>point72</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12129,7 +12353,11 @@
           <t>quadraturecapital</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12167,7 +12395,11 @@
           <t>quberesearchandtechnologies</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12205,7 +12437,11 @@
           <t>radixuniversity</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12239,7 +12475,11 @@
           <t>schonfeld</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12273,7 +12513,11 @@
           <t>sevenresearch</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12311,7 +12555,11 @@
           <t>simplextrading</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12349,7 +12597,11 @@
           <t>squarepointcapital</t>
         </is>
       </c>
-      <c r="F47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12387,7 +12639,11 @@
           <t>towerresearchcapital</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12421,7 +12677,11 @@
           <t>transmarketgroup</t>
         </is>
       </c>
-      <c r="F49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12455,7 +12715,11 @@
           <t>vaticlabs</t>
         </is>
       </c>
-      <c r="F50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12489,7 +12753,11 @@
           <t>virtu</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12527,7 +12795,11 @@
           <t>voloridgeinvestmentmanagement</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12561,7 +12833,11 @@
           <t>walleyecapital-external-students</t>
         </is>
       </c>
-      <c r="F53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12599,7 +12875,11 @@
           <t>winton</t>
         </is>
       </c>
-      <c r="F54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12633,7 +12913,11 @@
           <t>worldquant</t>
         </is>
       </c>
-      <c r="F55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12667,7 +12951,11 @@
           <t>belvederetrading</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12701,7 +12989,11 @@
           <t>valkyrietrading</t>
         </is>
       </c>
-      <c r="F57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12894,7 +13186,7 @@
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -12929,7 +13221,11 @@
           <t>https://www.albatrosslabs.io/</t>
         </is>
       </c>
-      <c r="F63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -12967,7 +13263,11 @@
           <t>https://www.aqr.com/About-Us/Our-Internship-Program</t>
         </is>
       </c>
-      <c r="F64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13005,7 +13305,11 @@
           <t>https://www.aspectcapital.com/careers/</t>
         </is>
       </c>
-      <c r="F65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13043,7 +13347,11 @@
           <t>https://www.bamfunds.com/careers/internships</t>
         </is>
       </c>
-      <c r="F66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13081,7 +13389,11 @@
           <t>https://www.bfcm.com/careers/</t>
         </is>
       </c>
-      <c r="F67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13119,7 +13431,11 @@
           <t>https://www.blueshift.am/</t>
         </is>
       </c>
-      <c r="F68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13157,7 +13473,11 @@
           <t>https://www.brevanhoward.com/students/</t>
         </is>
       </c>
-      <c r="F69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13195,7 +13515,11 @@
           <t>https://www.bridgewater.com/working-at-bridgewater/students</t>
         </is>
       </c>
-      <c r="F70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13236,7 +13560,7 @@
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
@@ -13271,7 +13595,11 @@
           <t>https://apply.workable.com/api/v1/widget/accounts/capula-investment-management-ltd</t>
         </is>
       </c>
-      <c r="F72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13309,7 +13637,11 @@
           <t>https://careers.cboe.com/us/en</t>
         </is>
       </c>
-      <c r="F73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13350,7 +13682,7 @@
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13385,7 +13717,11 @@
           <t>https://www.deshaw.com/careers</t>
         </is>
       </c>
-      <c r="F75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13423,7 +13759,11 @@
           <t>https://www.eagleseven.com/</t>
         </is>
       </c>
-      <c r="F76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13461,7 +13801,11 @@
           <t>https://www.eclipsetrading.com/careers/</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13499,7 +13843,11 @@
           <t>https://api.rippling.com/platform/api/ats/v1/board/edgehog-trading/jobs</t>
         </is>
       </c>
-      <c r="F78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13537,7 +13885,11 @@
           <t>https://www.eschatontrading.com/careers</t>
         </is>
       </c>
-      <c r="F79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13575,7 +13927,11 @@
           <t>https://www.gardacp.com/careers/</t>
         </is>
       </c>
-      <c r="F80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13616,7 +13972,7 @@
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -13651,7 +14007,11 @@
           <t>https://www.gresearch.com/careers/</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13689,7 +14049,11 @@
           <t>https://group1.com/careers/</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13727,7 +14091,11 @@
           <t>https://www.gsr.io/careers</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13768,7 +14136,7 @@
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -13803,7 +14171,11 @@
           <t>https://www.huqt.com/</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13841,7 +14213,11 @@
           <t>https://www.headlandstech.com/careers/</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13879,7 +14255,11 @@
           <t>https://hedgewestsf.org/</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13917,7 +14297,11 @@
           <t>https://www.hudsonrivertrading.com/careers/?_departments=internships</t>
         </is>
       </c>
-      <c r="F89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13955,7 +14339,11 @@
           <t>https://www.hudsonrivertrading.com/student-opportunities/</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -13993,7 +14381,11 @@
           <t>https://www.iaqf.org/upcoming-events</t>
         </is>
       </c>
-      <c r="F91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14031,7 +14423,11 @@
           <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14069,7 +14465,11 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/bridge/</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14107,7 +14507,11 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14145,7 +14549,11 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14183,7 +14591,11 @@
           <t>https://www.janestreet.com/join-jane-street/internships/</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14221,7 +14633,11 @@
           <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14259,7 +14675,11 @@
           <t>https://www.koretrading.com/front-page/careers/</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14297,7 +14717,11 @@
           <t>https://careers.lynxhedge.se/jobs.json</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14335,7 +14759,11 @@
           <t>https://www.marquettepartnersholdingsllc.com/careers</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14376,7 +14804,7 @@
       <c r="F101" s="2" t="inlineStr"/>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -14411,7 +14839,11 @@
           <t>https://battlecode.org/</t>
         </is>
       </c>
-      <c r="F102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14449,7 +14881,11 @@
           <t>https://osqf.org/</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr"/>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14487,7 +14923,11 @@
           <t>https://www.optiver.com/join-us/students/programs/futurefocus/</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14525,7 +14965,11 @@
           <t>https://readytradergo.optiver.com/</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14563,7 +15007,11 @@
           <t>https://optiver.com/working-at-optiver/career-opportunities/?level=student</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14601,7 +15049,11 @@
           <t>https://pokerbots.org/</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14639,7 +15091,11 @@
           <t>https://www.quantbot.com/careers/</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr"/>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14677,7 +15133,11 @@
           <t>https://www.rentec.com/careers</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr"/>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14715,7 +15175,11 @@
           <t>https://www.rokoscapital.com/careers</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr"/>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14753,7 +15217,11 @@
           <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr"/>
+      <c r="F111" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G111" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14791,7 +15259,11 @@
           <t>https://www.teza.com/careers/</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14829,7 +15301,11 @@
           <t>https://www.tgsmc.com/join-our-team/</t>
         </is>
       </c>
-      <c r="F113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14870,7 +15346,7 @@
       <c r="F114" s="2" t="inlineStr"/>
       <c r="G114" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H114" s="2" t="inlineStr">
@@ -14905,7 +15381,11 @@
           <t>https://www.tradebot.com/careers/students</t>
         </is>
       </c>
-      <c r="F115" s="2" t="inlineStr"/>
+      <c r="F115" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14943,7 +15423,11 @@
           <t>https://trexquant.com/careers/students</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14984,7 +15468,7 @@
       <c r="F117" s="2" t="inlineStr"/>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
@@ -15022,7 +15506,7 @@
       <c r="F118" s="2" t="inlineStr"/>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
@@ -15057,7 +15541,11 @@
           <t>https://vectortrading.com/data/roles.json</t>
         </is>
       </c>
-      <c r="F119" s="2" t="inlineStr"/>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15095,7 +15583,11 @@
           <t>https://www.verition.com/careers</t>
         </is>
       </c>
-      <c r="F120" s="2" t="inlineStr"/>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15133,7 +15625,11 @@
           <t>https://volanttrading.com/</t>
         </is>
       </c>
-      <c r="F121" s="2" t="inlineStr"/>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15171,7 +15667,11 @@
           <t>https://www.voloridge.com/join-our-team</t>
         </is>
       </c>
-      <c r="F122" s="2" t="inlineStr"/>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15209,7 +15709,11 @@
           <t>https://www.wincent.com/careers/</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15247,7 +15751,11 @@
           <t>https://www.wintermute.com/company/careers</t>
         </is>
       </c>
-      <c r="F124" s="2" t="inlineStr"/>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15285,7 +15793,11 @@
           <t>https://careers.wolve.com/postings.json</t>
         </is>
       </c>
-      <c r="F125" s="2" t="inlineStr"/>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15323,7 +15835,11 @@
           <t>https://www.xtxmarkets.com/careers/</t>
         </is>
       </c>
-      <c r="F126" s="2" t="inlineStr"/>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15361,7 +15877,11 @@
           <t>https://careers.sig.com/api/jobs</t>
         </is>
       </c>
-      <c r="F127" s="2" t="inlineStr"/>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G127" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15395,7 +15915,11 @@
           <t>https://capgroup.wd1.myworkdayjobs.com/wday/cxs/capgroup/capitalgroupcareers</t>
         </is>
       </c>
-      <c r="F128" s="2" t="inlineStr"/>
+      <c r="F128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15429,7 +15953,11 @@
           <t>https://cibc.wd3.myworkdayjobs.com/wday/cxs/cibc/campus</t>
         </is>
       </c>
-      <c r="F129" s="2" t="inlineStr"/>
+      <c r="F129" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15467,7 +15995,11 @@
           <t>https://cmegroup.wd1.myworkdayjobs.com/wday/cxs/cmegroup/cme_careers</t>
         </is>
       </c>
-      <c r="F130" s="2" t="inlineStr"/>
+      <c r="F130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15501,7 +16033,11 @@
           <t>https://dimensional.wd5.myworkdayjobs.com/wday/cxs/dimensional/dfa_careers</t>
         </is>
       </c>
-      <c r="F131" s="2" t="inlineStr"/>
+      <c r="F131" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15535,7 +16071,11 @@
           <t>https://draftkings.wd1.myworkdayjobs.com/wday/cxs/draftkings/Campus_Career_Portal</t>
         </is>
       </c>
-      <c r="F132" s="2" t="inlineStr"/>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15569,7 +16109,11 @@
           <t>https://fanniemae.wd1.myworkdayjobs.com/wday/cxs/fanniemae/FannieMaeCareers</t>
         </is>
       </c>
-      <c r="F133" s="2" t="inlineStr"/>
+      <c r="F133" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15603,7 +16147,11 @@
           <t>https://freddiemac.wd5.myworkdayjobs.com/wday/cxs/freddiemac/External</t>
         </is>
       </c>
-      <c r="F134" s="2" t="inlineStr"/>
+      <c r="F134" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15637,7 +16185,11 @@
           <t>https://spgi.wd5.myworkdayjobs.com/wday/cxs/spgi/Kensho_Careers</t>
         </is>
       </c>
-      <c r="F135" s="2" t="inlineStr"/>
+      <c r="F135" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15671,7 +16223,11 @@
           <t>https://lplfinancial.wd1.myworkdayjobs.com/wday/cxs/lplfinancial/university</t>
         </is>
       </c>
-      <c r="F136" s="2" t="inlineStr"/>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G136" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15705,7 +16261,11 @@
           <t>https://mastercard.wd1.myworkdayjobs.com/wday/cxs/mastercard/Campus</t>
         </is>
       </c>
-      <c r="F137" s="2" t="inlineStr"/>
+      <c r="F137" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15739,7 +16299,11 @@
           <t>https://ntrs.wd1.myworkdayjobs.com/wday/cxs/ntrs/northerntrust</t>
         </is>
       </c>
-      <c r="F138" s="2" t="inlineStr"/>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15777,7 +16341,11 @@
           <t>https://peak6group.wd1.myworkdayjobs.com/wday/cxs/peak6group/PEAK6</t>
         </is>
       </c>
-      <c r="F139" s="2" t="inlineStr"/>
+      <c r="F139" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15811,7 +16379,11 @@
           <t>https://pimco.wd1.myworkdayjobs.com/wday/cxs/pimco/pimco-careers</t>
         </is>
       </c>
-      <c r="F140" s="2" t="inlineStr"/>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15845,7 +16417,11 @@
           <t>https://rbc.wd3.myworkdayjobs.com/wday/cxs/rbc/RBCEARLYTALENT1</t>
         </is>
       </c>
-      <c r="F141" s="2" t="inlineStr"/>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15879,7 +16455,11 @@
           <t>https://troweprice.wd5.myworkdayjobs.com/wday/cxs/troweprice/TRowePrice</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15913,7 +16493,11 @@
           <t>https://vanguard.wd5.myworkdayjobs.com/wday/cxs/vanguard/vanguard_external</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15947,7 +16531,11 @@
           <t>https://wellington.wd5.myworkdayjobs.com/wday/cxs/wellington/Campus</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-12T11:41:26+00:00</t>
+        </is>
+      </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
           <t>0</t>

</xml_diff>

<commit_message>
state: 2026-09-13 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7866,7 +7866,7 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8734,7 +8734,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr"/>
@@ -8802,7 +8802,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10494,7 +10494,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10789,7 +10789,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10865,7 +10865,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10903,7 +10903,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10941,7 +10941,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10979,7 +10979,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11021,7 +11021,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11063,7 +11063,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11105,7 +11105,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11311,7 +11311,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11353,7 +11353,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11391,7 +11391,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11433,7 +11433,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11475,7 +11475,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11555,7 +11555,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11597,7 +11597,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11673,7 +11673,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11711,7 +11711,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11753,7 +11753,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11795,7 +11795,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11833,7 +11833,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11871,7 +11871,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11913,7 +11913,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11951,7 +11951,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -11989,7 +11989,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12031,7 +12031,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12069,7 +12069,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12107,7 +12107,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12145,7 +12145,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12183,7 +12183,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12221,7 +12221,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12301,7 +12301,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12339,7 +12339,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12381,7 +12381,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12423,7 +12423,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12461,7 +12461,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12499,7 +12499,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12537,7 +12537,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12579,7 +12579,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12617,7 +12617,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12659,7 +12659,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12701,7 +12701,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12739,7 +12739,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12781,7 +12781,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12823,7 +12823,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12861,7 +12861,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12899,7 +12899,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12941,7 +12941,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12983,7 +12983,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13025,7 +13025,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13063,7 +13063,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13101,7 +13101,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13139,7 +13139,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13177,7 +13177,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13215,7 +13215,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13257,7 +13257,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13337,7 +13337,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13375,7 +13375,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13413,7 +13413,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13451,7 +13451,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13489,7 +13489,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13721,7 +13721,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13768,7 +13768,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -13805,7 +13805,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13847,7 +13847,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13889,7 +13889,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13931,7 +13931,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13973,7 +13973,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14015,7 +14015,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14095,7 +14095,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14137,7 +14137,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14217,7 +14217,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14259,7 +14259,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14297,7 +14297,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14339,7 +14339,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14381,7 +14381,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14423,7 +14423,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14465,7 +14465,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14545,7 +14545,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14587,7 +14587,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14629,7 +14629,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14709,7 +14709,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14751,7 +14751,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14793,7 +14793,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14835,7 +14835,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14877,7 +14877,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14919,7 +14919,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -14961,7 +14961,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15003,7 +15003,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15045,7 +15045,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15087,7 +15087,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15129,7 +15129,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15171,7 +15171,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15213,7 +15213,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15255,7 +15255,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15297,7 +15297,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15377,7 +15377,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15419,7 +15419,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15461,7 +15461,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15503,7 +15503,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15545,7 +15545,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15587,7 +15587,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15671,7 +15671,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15713,7 +15713,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15755,7 +15755,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15797,7 +15797,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15839,7 +15839,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15919,7 +15919,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16079,7 +16079,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16121,7 +16121,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16163,7 +16163,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16205,7 +16205,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16247,7 +16247,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16289,7 +16289,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16331,7 +16331,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16373,7 +16373,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16415,7 +16415,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16453,7 +16453,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16491,7 +16491,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16533,7 +16533,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16571,7 +16571,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16609,7 +16609,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16647,7 +16647,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16685,7 +16685,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16723,7 +16723,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16761,7 +16761,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16799,7 +16799,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16842,7 +16842,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -16879,7 +16879,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -16917,7 +16917,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -16955,7 +16955,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -16993,7 +16993,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -17031,7 +17031,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -17069,7 +17069,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-13T13:27:13+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-14 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Programs'!$A$1:$N$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$H$158</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Applied'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7866,12 +7866,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>914754581aace9fd7a7cff7bfb787ac0e7f52f18e0194b6a8d837531643e0b9d</t>
+          <t>9f94bdf7c297d22169d8a6e0e0413c94ff4a6cd02a1b6464a87b49ba2b6c9bb9</t>
         </is>
       </c>
     </row>
@@ -7934,12 +7934,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-10T12:11:00+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7950,7 +7950,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>de71475901207962ca947d6f8f4202f2de5be54ec3c1592fc60d8211806d9b25</t>
+          <t>7aae100d64822870cb3d2a28d1948dd7d89af148e680e1b5c8f15aee2305042c</t>
         </is>
       </c>
     </row>
@@ -8002,7 +8002,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8734,10 +8734,14 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
-        </is>
-      </c>
-      <c r="K157" s="2" t="inlineStr"/>
+          <t>2026-09-14T15:23:08+00:00</t>
+        </is>
+      </c>
+      <c r="K157" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14T15:23:08+00:00</t>
+        </is>
+      </c>
       <c r="L157" s="2" t="inlineStr">
         <is>
           <t>2026-09-06</t>
@@ -8750,7 +8754,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>61d26c9a5fc173a201c91f202de53d06297ddf5de8927e930447b1b7b12f0295</t>
+          <t>354e8229c45e114d1b9a08f856918cb1d9faba977a578b3417b1c84b5f02ef8d</t>
         </is>
       </c>
     </row>
@@ -8802,7 +8806,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10494,7 +10498,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10789,7 +10793,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10827,7 +10831,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10865,7 +10869,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10903,7 +10907,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10941,7 +10945,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10979,7 +10983,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11021,7 +11025,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11063,7 +11067,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11105,7 +11109,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11147,7 +11151,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11189,7 +11193,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11231,7 +11235,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11273,7 +11277,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11311,7 +11315,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11353,7 +11357,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11391,7 +11395,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11433,7 +11437,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11475,7 +11479,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11517,7 +11521,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11555,7 +11559,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11597,7 +11601,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11635,7 +11639,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11673,7 +11677,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11711,7 +11715,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11753,7 +11757,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11795,7 +11799,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11833,7 +11837,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11871,7 +11875,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11913,7 +11917,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11951,7 +11955,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -11989,7 +11993,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12031,7 +12035,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12069,7 +12073,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12107,7 +12111,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12145,7 +12149,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12183,7 +12187,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12221,7 +12225,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12259,7 +12263,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12301,7 +12305,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12339,7 +12343,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12381,7 +12385,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12423,7 +12427,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12461,7 +12465,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12499,7 +12503,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12537,7 +12541,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12579,7 +12583,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12617,7 +12621,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12659,7 +12663,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12701,7 +12705,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12739,7 +12743,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12781,7 +12785,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12823,7 +12827,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12861,7 +12865,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12899,7 +12903,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12941,7 +12945,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12983,7 +12987,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13025,7 +13029,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13063,7 +13067,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13101,7 +13105,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13139,7 +13143,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13177,7 +13181,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13215,7 +13219,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13257,7 +13261,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13295,7 +13299,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13337,7 +13341,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13375,7 +13379,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13413,7 +13417,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13451,7 +13455,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13489,7 +13493,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13684,7 +13688,7 @@
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -13721,7 +13725,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13763,12 +13767,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T12:47:15+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -13805,7 +13809,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13847,7 +13851,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13889,7 +13893,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13931,7 +13935,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13973,7 +13977,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14015,7 +14019,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14058,7 +14062,7 @@
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -14095,7 +14099,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14137,7 +14141,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14180,7 +14184,7 @@
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -14217,7 +14221,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14259,7 +14263,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14297,7 +14301,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14339,7 +14343,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14381,7 +14385,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14423,7 +14427,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14465,7 +14469,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14508,7 +14512,7 @@
       <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -14545,7 +14549,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14587,7 +14591,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14629,7 +14633,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14672,7 +14676,7 @@
       <c r="F99" s="2" t="inlineStr"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -14709,7 +14713,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14751,7 +14755,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14793,7 +14797,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14835,7 +14839,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14877,7 +14881,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14919,7 +14923,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -14961,7 +14965,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15003,7 +15007,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15045,7 +15049,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15087,7 +15091,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15129,7 +15133,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15171,7 +15175,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15213,7 +15217,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15255,7 +15259,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15297,7 +15301,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15340,7 +15344,7 @@
       <c r="F115" s="2" t="inlineStr"/>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -15377,7 +15381,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15419,7 +15423,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15461,7 +15465,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15503,7 +15507,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15545,7 +15549,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15587,7 +15591,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15629,7 +15633,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15671,7 +15675,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15713,7 +15717,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15755,7 +15759,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15797,7 +15801,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15839,7 +15843,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15882,7 +15886,7 @@
       <c r="F128" s="2" t="inlineStr"/>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -15919,7 +15923,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -15961,7 +15965,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16004,7 +16008,7 @@
       <c r="F131" s="2" t="inlineStr"/>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -16042,7 +16046,7 @@
       <c r="F132" s="2" t="inlineStr"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -16079,7 +16083,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16121,7 +16125,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16163,7 +16167,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16205,7 +16209,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16247,7 +16251,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16289,7 +16293,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16331,7 +16335,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16373,7 +16377,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16415,7 +16419,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16453,7 +16457,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16491,7 +16495,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16533,7 +16537,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16571,7 +16575,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16609,7 +16613,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16647,7 +16651,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16685,7 +16689,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16723,7 +16727,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16761,7 +16765,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16799,7 +16803,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16837,7 +16841,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -16879,7 +16883,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -16917,7 +16921,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -16955,7 +16959,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -16993,7 +16997,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -17031,7 +17035,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -17069,7 +17073,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-13T13:59:47+00:00</t>
+          <t>2026-09-14T15:23:08+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -17223,7 +17227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H28"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17281,962 +17285,966 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Allston Trading</t>
+          <t>appian</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>allston-trading</t>
+          <t>greenhouse:appian</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://allstontrading.com</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/appian/jobs?content=true</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 172 postings, 10 US student rows</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>AlphaGrep Securities</t>
+          <t>bti36021</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>alphagrep</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>alphagrepsecurities (greenhouse)</t>
+          <t>greenhouse:bti36021</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>https://boards-api.greenhouse.io/v1/boards/bti36021/jobs?content=true</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 12 postings, 1 US student rows</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>AlphaSimplex</t>
+          <t>chicagotradingcampus</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>alphasimplex</t>
+          <t>greenhouse:chicagotradingcampus</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://www.alphasimplex.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Arb Trading Group</t>
+          <t>compeerfinancial</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>arb-trading-group</t>
+          <t>greenhouse:compeerfinancial</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://arb-tg.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Citadel (hedge fund)</t>
+          <t>cssmerge</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>citadel</t>
+          <t>greenhouse:cssmerge</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://www.citadel.com/careers/students/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Consolidated Trading</t>
+          <t>ctccampusboard</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>consolidated-trading</t>
+          <t>greenhouse:ctccampusboard</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>http://consolidatedtrading.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Cutler Group</t>
+          <t>devtechnology</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>cutler-group</t>
+          <t>greenhouse:devtechnology</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://cutlerllc.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dark Forest Technologies</t>
+          <t>eulerity</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>dark-forest-tech</t>
+          <t>greenhouse:eulerity</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://darkforesttech.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Eisler Capital</t>
+          <t>gallup</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>eisler-capital</t>
+          <t>greenhouse:gallup</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://eislercapital.com</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Emergent Trading</t>
+          <t>gardacp</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>emergent-trading</t>
+          <t>greenhouse:gardacp</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://www.emergenttrading.com/join</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Freestone Grove Partners</t>
+          <t>generalmatter</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>freestone-grove</t>
+          <t>greenhouse:generalmatter</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.gem.com/freestone-grove-partners</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs Emerging Leaders Series</t>
+          <t>hpiq</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>goldman-emerging-leaders</t>
+          <t>greenhouse:hpiq</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Kinetic Trading Partners</t>
+          <t>hudl</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>kinetic-trading-partners</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>greenhouse:hudl</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Laurion Capital</t>
+          <t>idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>laurion-capital</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>laurioncapitalmanagement (greenhouse)</t>
+          <t>greenhouse:idmeuniversityrecruiting</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Nico Trading</t>
+          <t>k2spacecorporation</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>nico-trading</t>
+          <t>greenhouse:k2spacecorporation</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://nicotrading.com</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Numerai</t>
+          <t>klaviyocampus</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>numerai</t>
+          <t>greenhouse:klaviyocampus</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://numer.ai/careers</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Quantitative Investment Management</t>
+          <t>nisc</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>qim</t>
+          <t>greenhouse:nisc</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://quantitative.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Quantbox Research</t>
+          <t>pacificfusion</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>quantbox-research</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>quantboxresearchpte (greenhouse)</t>
+          <t>greenhouse:pacificfusion</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Quantlab Financial</t>
+          <t>testnisc</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>quantlab</t>
+          <t>greenhouse:testnisc</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://www.quantlab.com/careers</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>QVR Advisors</t>
+          <t>tgsmc</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>lever</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>qvr-advisors</t>
+          <t>lever:tgsmc</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://qvradvisors.com</t>
+          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
+          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Rosetta Analytics</t>
+          <t>Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>rosetta-analytics</t>
+          <t>repo:chieler/summer-2027-swe-internships</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://rosetta-analytics.com/</t>
+          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
+          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Sensato Investors</t>
+          <t>sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>sensato-investors</t>
+          <t>repo:sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://sensatoinvestors.com</t>
+          <t>https://github.com/sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
+          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Spot Trading</t>
+          <t>vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>spot-trading</t>
+          <t>repo:vanshb03/summer2027-internships</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://spottradingllc.com</t>
+          <t>https://github.com/vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
+          <t>9045 stars, pushed 2026-08-23; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -18248,7 +18256,7 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Summerside Capital</t>
+          <t>Allston Trading</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -18258,13 +18266,17 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>summerside-capital</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
+          <t>allston-trading</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>https://allstontrading.com</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
+          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -18286,7 +18298,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Tyler Capital</t>
+          <t>AlphaGrep Securities</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -18296,17 +18308,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>tyler-capital</t>
-        </is>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.tylercapital.co.uk/</t>
+          <t>alphagrep</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>alphagrepsecurities (greenhouse)</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -18328,7 +18340,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>WH Trading</t>
+          <t>AlphaSimplex</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -18338,17 +18350,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>wh-trading</t>
+          <t>alphasimplex</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://whtrading.com/life-at-wh-trading/</t>
+          <t>https://www.alphasimplex.com/</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -18370,65 +18382,1046 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
+          <t>Arb Trading Group</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>arb-trading-group</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>https://arb-tg.com/</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Citadel (hedge fund)</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>citadel</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.citadel.com/careers/students/</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Consolidated Trading</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>consolidated-trading</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>http://consolidatedtrading.com/</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Cutler Group</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>cutler-group</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>https://cutlerllc.com/</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Dark Forest Technologies</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>dark-forest-tech</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>https://darkforesttech.com/</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Eisler Capital</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>eisler-capital</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>https://eislercapital.com</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Emergent Trading</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>emergent-trading</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>https://www.emergenttrading.com/join</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Freestone Grove Partners</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>freestone-grove</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.gem.com/freestone-grove-partners</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Goldman Sachs Emerging Leaders Series</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>goldman-emerging-leaders</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Kinetic Trading Partners</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>kinetic-trading-partners</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Laurion Capital</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>laurion-capital</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>laurioncapitalmanagement (greenhouse)</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Nico Trading</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>nico-trading</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>https://nicotrading.com</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Numerai</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>numerai</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>https://numer.ai/careers</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Quantitative Investment Management</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>qim</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>https://quantitative.com/</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Quantbox Research</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>quantbox-research</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>quantboxresearchpte (greenhouse)</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>Quantlab Financial</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>quantlab</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.quantlab.com/careers</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>QVR Advisors</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>qvr-advisors</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>https://qvradvisors.com</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Rosetta Analytics</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>rosetta-analytics</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>https://rosetta-analytics.com/</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Sensato Investors</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>sensato-investors</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>https://sensatoinvestors.com</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Spot Trading</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>spot-trading</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>https://spottradingllc.com</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Summerside Capital</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>summerside-capital</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Capital</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>tyler-capital</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tylercapital.co.uk/</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>WH Trading</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>wh-trading</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>https://whtrading.com/life-at-wh-trading/</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
           <t>XR Trading</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C51" s="2" t="inlineStr">
         <is>
           <t>firm</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>xr-trading</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>https://www.xrtrading.com/</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F51" s="2" t="inlineStr">
         <is>
           <t>Paylocity React shell: board returns 670 chars, all of it 'unsupported browser' boilerplate, zero titles. Bundle grepped - no JSON endpoint exists.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G51" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H51" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H28"/>
+  <autoFilter ref="A1:H51"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId45"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: 2026-09-15 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7866,12 +7866,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>d51d9f66f8476698fa50ad70f823fea06ed1bb0169c8665a5f2a1f4315a30a2d</t>
+          <t>cacbfe1bfa8c253bb724a3ee875c67a9087abb488e1c1d42c24c6c1e016bc977</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8002,12 +8002,12 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07T16:42:35+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="L145" s="2" t="inlineStr"/>
@@ -8018,7 +8018,7 @@
       </c>
       <c r="N145" s="2" t="inlineStr">
         <is>
-          <t>770702cb19ea8d996aed49851c54d2d3a4bc930f4c445257f7e6626ae1b193e8</t>
+          <t>1f1887cdb2115241c55873db773039a5495f8440af9d0148b518fe01ffa1fc4f</t>
         </is>
       </c>
     </row>
@@ -8066,7 +8066,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8734,7 +8734,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8806,7 +8806,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10498,7 +10498,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10793,7 +10793,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10945,7 +10945,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11025,7 +11025,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11639,7 +11639,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11677,7 +11677,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11757,7 +11757,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -11993,7 +11993,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12035,7 +12035,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12149,7 +12149,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12385,7 +12385,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12465,7 +12465,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12503,7 +12503,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12541,7 +12541,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12583,7 +12583,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12705,7 +12705,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12865,7 +12865,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13181,7 +13181,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13261,7 +13261,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13299,7 +13299,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13341,7 +13341,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13417,7 +13417,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13455,7 +13455,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13688,7 +13688,7 @@
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13772,7 +13772,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -13809,7 +13809,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13935,7 +13935,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13977,7 +13977,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14062,7 +14062,7 @@
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14141,7 +14141,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14184,7 +14184,7 @@
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -14221,7 +14221,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14263,7 +14263,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14301,7 +14301,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14343,7 +14343,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14469,7 +14469,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14512,7 +14512,7 @@
       <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14633,7 +14633,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14676,7 +14676,7 @@
       <c r="F99" s="2" t="inlineStr"/>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14797,7 +14797,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14839,7 +14839,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14923,7 +14923,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15091,7 +15091,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15133,7 +15133,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15175,7 +15175,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15217,7 +15217,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15301,7 +15301,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15344,7 +15344,7 @@
       <c r="F115" s="2" t="inlineStr"/>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15549,7 +15549,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15591,7 +15591,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15717,7 +15717,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15759,7 +15759,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15886,7 +15886,7 @@
       <c r="F128" s="2" t="inlineStr"/>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -15923,7 +15923,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -15965,7 +15965,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16008,7 +16008,7 @@
       <c r="F131" s="2" t="inlineStr"/>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -16046,7 +16046,7 @@
       <c r="F132" s="2" t="inlineStr"/>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16125,7 +16125,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16209,7 +16209,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16251,7 +16251,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16293,7 +16293,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16335,7 +16335,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16457,7 +16457,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16537,7 +16537,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16575,7 +16575,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16651,7 +16651,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16689,7 +16689,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16727,7 +16727,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -16883,7 +16883,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -16921,7 +16921,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -16959,7 +16959,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -16997,7 +16997,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -17035,7 +17035,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -17073,7 +17073,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-15T20:43:53+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -17285,7 +17285,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -17327,7 +17327,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -17369,12 +17369,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>chicagotradingcampus</t>
+          <t>compeerfinancial</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -17384,17 +17384,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:chicagotradingcampus</t>
+          <t>greenhouse:compeerfinancial</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -17411,12 +17411,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>compeerfinancial</t>
+          <t>cssmerge</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -17426,17 +17426,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:compeerfinancial</t>
+          <t>greenhouse:cssmerge</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -17453,12 +17453,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>cssmerge</t>
+          <t>devtechnology</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -17468,17 +17468,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:cssmerge</t>
+          <t>greenhouse:devtechnology</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -17495,12 +17495,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ctccampusboard</t>
+          <t>eulerity</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -17510,17 +17510,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:ctccampusboard</t>
+          <t>greenhouse:eulerity</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -17537,12 +17537,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>devtechnology</t>
+          <t>gallup</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -17552,17 +17552,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:devtechnology</t>
+          <t>greenhouse:gallup</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -17579,12 +17579,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>eulerity</t>
+          <t>generalmatter</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -17594,17 +17594,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:eulerity</t>
+          <t>greenhouse:generalmatter</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -17621,12 +17621,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>gallup</t>
+          <t>hpiq</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -17636,17 +17636,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gallup</t>
+          <t>greenhouse:hpiq</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -17663,12 +17663,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>gardacp</t>
+          <t>hudl</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -17678,17 +17678,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gardacp</t>
+          <t>greenhouse:hudl</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -17705,12 +17705,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>generalmatter</t>
+          <t>idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -17720,17 +17720,17 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:generalmatter</t>
+          <t>greenhouse:idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -17747,12 +17747,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>hpiq</t>
+          <t>k2spacecorporation</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -17762,17 +17762,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hpiq</t>
+          <t>greenhouse:k2spacecorporation</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -17789,12 +17789,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>hudl</t>
+          <t>klaviyocampus</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -17804,17 +17804,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hudl</t>
+          <t>greenhouse:klaviyocampus</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -17831,12 +17831,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>idmeuniversityrecruiting</t>
+          <t>nisc</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -17846,17 +17846,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:idmeuniversityrecruiting</t>
+          <t>greenhouse:nisc</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -17873,12 +17873,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>k2spacecorporation</t>
+          <t>pacificfusion</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -17888,17 +17888,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:k2spacecorporation</t>
+          <t>greenhouse:pacificfusion</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -17915,12 +17915,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>klaviyocampus</t>
+          <t>testnisc</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -17930,17 +17930,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:klaviyocampus</t>
+          <t>greenhouse:testnisc</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -17957,32 +17957,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>nisc</t>
+          <t>Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>greenhouse</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:nisc</t>
+          <t>repo:chieler/summer-2027-swe-internships</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
+          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
+          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -17999,32 +17999,32 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>pacificfusion</t>
+          <t>sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>greenhouse</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:pacificfusion</t>
+          <t>repo:sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
+          <t>https://github.com/sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
+          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -18046,7 +18046,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>testnisc</t>
+          <t>chicagotradingcampus</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -18056,17 +18056,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:testnisc</t>
+          <t>greenhouse:chicagotradingcampus</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -18088,27 +18088,27 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>tgsmc</t>
+          <t>ctccampusboard</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>lever</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>lever:tgsmc</t>
+          <t>greenhouse:ctccampusboard</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -18130,27 +18130,27 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Chieler/Summer-2027-SWE-Internships</t>
+          <t>gardacp</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>repo:chieler/summer-2027-swe-internships</t>
+          <t>greenhouse:gardacp</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -18172,27 +18172,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>sndsh404/summer-2027-internships</t>
+          <t>tgsmc</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>lever</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>repo:sndsh404/summer-2027-internships</t>
+          <t>lever:tgsmc</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/sndsh404/summer-2027-internships</t>
+          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
+          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-16 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4474,7 +4474,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7802,7 +7802,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7866,12 +7866,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T20:43:53+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>cacbfe1bfa8c253bb724a3ee875c67a9087abb488e1c1d42c24c6c1e016bc977</t>
+          <t>1c646d305b4c280a09f1fdcebc43895d8416592b0361b8f5e27f07ae39a0f064</t>
         </is>
       </c>
     </row>
@@ -7934,7 +7934,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8066,7 +8066,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8402,7 +8402,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8470,7 +8470,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8666,7 +8666,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8734,7 +8734,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8806,7 +8806,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10498,7 +10498,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10793,7 +10793,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10831,7 +10831,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10869,7 +10869,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10907,7 +10907,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10945,7 +10945,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10983,7 +10983,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11025,7 +11025,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11395,7 +11395,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11639,7 +11639,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11677,7 +11677,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11715,7 +11715,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11757,7 +11757,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11837,7 +11837,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11875,7 +11875,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11917,7 +11917,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11955,7 +11955,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -11993,7 +11993,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12035,7 +12035,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12073,7 +12073,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12111,7 +12111,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12149,7 +12149,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12187,7 +12187,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12305,7 +12305,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12343,7 +12343,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12385,7 +12385,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12427,7 +12427,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12465,7 +12465,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12503,7 +12503,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12541,7 +12541,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12583,7 +12583,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12621,7 +12621,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12663,7 +12663,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12705,7 +12705,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12743,7 +12743,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12785,7 +12785,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12827,7 +12827,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12865,7 +12865,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12903,7 +12903,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12945,7 +12945,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12987,7 +12987,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13029,7 +13029,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13067,7 +13067,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13143,7 +13143,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13181,7 +13181,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13219,7 +13219,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13261,7 +13261,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13299,7 +13299,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13341,7 +13341,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13379,7 +13379,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13417,7 +13417,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13455,7 +13455,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -13493,7 +13493,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13767,12 +13767,12 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:23:08+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
@@ -13809,7 +13809,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13851,7 +13851,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13935,7 +13935,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13977,7 +13977,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14019,7 +14019,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14141,7 +14141,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14221,7 +14221,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14263,7 +14263,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14301,7 +14301,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14343,7 +14343,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14385,7 +14385,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14427,7 +14427,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14469,7 +14469,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14549,7 +14549,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14591,7 +14591,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14633,7 +14633,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14713,7 +14713,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14797,7 +14797,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14839,7 +14839,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14881,7 +14881,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14923,7 +14923,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15007,7 +15007,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15049,7 +15049,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15091,7 +15091,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15133,7 +15133,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15175,7 +15175,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15217,7 +15217,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15259,7 +15259,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15301,7 +15301,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15381,7 +15381,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15423,7 +15423,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15465,7 +15465,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15507,7 +15507,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15549,7 +15549,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15591,7 +15591,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15633,7 +15633,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15675,7 +15675,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15717,7 +15717,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15759,7 +15759,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15843,7 +15843,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15923,7 +15923,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -15970,7 +15970,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -16083,7 +16083,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16125,7 +16125,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16209,7 +16209,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16251,7 +16251,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16293,7 +16293,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16335,7 +16335,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16419,7 +16419,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16457,7 +16457,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16495,7 +16495,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16537,7 +16537,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16575,7 +16575,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16613,7 +16613,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16651,7 +16651,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16689,7 +16689,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16727,7 +16727,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16765,7 +16765,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16803,7 +16803,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16841,7 +16841,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -16883,7 +16883,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -16921,7 +16921,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -16959,7 +16959,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -16997,7 +16997,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -17035,7 +17035,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -17073,7 +17073,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-16T12:40:49+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-17 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>1c646d305b4c280a09f1fdcebc43895d8416592b0361b8f5e27f07ae39a0f064</t>
+          <t>4bc75dc7332eb96e499cda2e2fbbce876e5cb85db68480f7bce7cef57098891a</t>
         </is>
       </c>
     </row>
@@ -7942,12 +7942,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T15:23:08+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>7aae100d64822870cb3d2a28d1948dd7d89af148e680e1b5c8f15aee2305042c</t>
+          <t>c138777b70d1ead474c63d20398ca1f0cdf4bcbd067670199fc8e3305e3d11f0</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,12 +8742,12 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T16:06:55+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
@@ -8762,7 +8762,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>60a880796c08ba895b63ab55bdaee867faf3afedf8135ba2a56f16e08682874a</t>
+          <t>0a65a7d54ecc562352de4dfca24a192526334f0c374fa2839c7c3dcc19d1c4f2</t>
         </is>
       </c>
     </row>
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10801,7 +10801,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10915,7 +10915,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11117,7 +11117,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11159,7 +11159,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11243,7 +11243,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11365,7 +11365,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11529,7 +11529,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11609,7 +11609,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11769,7 +11769,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12157,7 +12157,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12359,7 +12359,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12595,7 +12595,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12637,7 +12637,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12759,7 +12759,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12797,7 +12797,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12919,7 +12919,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12999,7 +12999,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13075,7 +13075,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13787,7 +13787,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13829,7 +13829,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13871,7 +13871,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13955,7 +13955,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13997,7 +13997,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14039,7 +14039,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14329,7 +14329,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14371,7 +14371,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14453,7 +14453,11 @@
           <t>https://careers-gtsx.icims.com/jobs/search?ss=1&amp;in_iframe=1</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T00:52:12+00:00</t>
+        </is>
+      </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -14493,7 +14497,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14535,7 +14539,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14577,7 +14581,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14619,7 +14623,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14661,7 +14665,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14703,7 +14707,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14745,7 +14749,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14787,7 +14791,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14829,7 +14833,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14871,7 +14875,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14913,7 +14917,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14955,7 +14959,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -14997,7 +15001,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15039,7 +15043,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15081,7 +15085,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15123,7 +15127,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15165,7 +15169,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15207,7 +15211,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15249,7 +15253,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15291,7 +15295,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15333,7 +15337,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15375,7 +15379,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15417,7 +15421,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15459,7 +15463,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15501,7 +15505,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15543,7 +15547,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15585,7 +15589,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15627,7 +15631,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15669,12 +15673,12 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T21:02:15+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
@@ -15709,7 +15713,11 @@
           <t>https://careers.twosigma.com/careers/OpenRoles/</t>
         </is>
       </c>
-      <c r="F123" s="2" t="inlineStr"/>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17T00:52:12+00:00</t>
+        </is>
+      </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15749,7 +15757,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15791,7 +15799,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15833,7 +15841,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15875,7 +15883,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15917,7 +15925,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -15959,7 +15967,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16001,7 +16009,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16043,7 +16051,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16085,7 +16093,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16123,7 +16131,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16161,7 +16169,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16203,7 +16211,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16241,7 +16249,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16279,7 +16287,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16317,7 +16325,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16355,7 +16363,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16393,7 +16401,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16431,7 +16439,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16469,7 +16477,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16507,7 +16515,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16549,7 +16557,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16587,7 +16595,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16625,7 +16633,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16663,7 +16671,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16701,7 +16709,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16739,7 +16747,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T12:40:49+00:00</t>
+          <t>2026-09-17T00:52:12+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-18 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>8f6dddcf5cda4f5703b938fb8c3902108c17e026292c8738dfee37ae8e79e423</t>
+          <t>56efcece082a87b9731033eca0397d38fcaddb4542500f4540d6fbd490df44e6</t>
         </is>
       </c>
     </row>
@@ -7942,12 +7942,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T00:52:12+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>c138777b70d1ead474c63d20398ca1f0cdf4bcbd067670199fc8e3305e3d11f0</t>
+          <t>d605a0e1ee5879383316242ff0280132a6a10ea394b4e02b6497340361b17403</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10801,7 +10801,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10839,7 +10839,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10877,7 +10877,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -10915,7 +10915,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11117,7 +11117,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11159,7 +11159,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11243,7 +11243,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11285,7 +11285,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11365,7 +11365,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11529,7 +11529,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11571,7 +11571,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11609,7 +11609,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11769,7 +11769,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12157,7 +12157,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12359,7 +12359,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12595,7 +12595,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12637,7 +12637,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12759,7 +12759,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12797,7 +12797,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -12919,7 +12919,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -12999,7 +12999,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13075,7 +13075,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13619,7 +13619,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13666,7 +13666,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13703,7 +13703,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13745,7 +13745,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13787,7 +13787,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13829,7 +13829,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13871,7 +13871,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -13913,7 +13913,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -13955,7 +13955,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -13997,7 +13997,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14039,7 +14039,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14081,7 +14081,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14245,7 +14245,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14329,7 +14329,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14371,7 +14371,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14413,7 +14413,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14455,7 +14455,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14497,7 +14497,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14539,7 +14539,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14581,7 +14581,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14623,7 +14623,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14665,7 +14665,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14707,7 +14707,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14749,7 +14749,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14791,7 +14791,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14875,7 +14875,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -14917,7 +14917,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -14959,7 +14959,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15001,7 +15001,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15085,7 +15085,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15127,7 +15127,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15169,7 +15169,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15211,7 +15211,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15253,7 +15253,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15295,7 +15295,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15337,7 +15337,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15379,7 +15379,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15421,7 +15421,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15463,7 +15463,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15505,7 +15505,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15547,7 +15547,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15589,7 +15589,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15631,7 +15631,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15673,7 +15673,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15715,7 +15715,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15757,7 +15757,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15799,7 +15799,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15841,7 +15841,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15883,7 +15883,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -15925,7 +15925,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -15967,7 +15967,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16009,7 +16009,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16051,7 +16051,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16093,7 +16093,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16169,7 +16169,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16211,7 +16211,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16249,7 +16249,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16287,7 +16287,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16325,7 +16325,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16363,7 +16363,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16401,7 +16401,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16439,7 +16439,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16477,7 +16477,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16515,7 +16515,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16557,7 +16557,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16595,7 +16595,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16633,7 +16633,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16671,7 +16671,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16709,7 +16709,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16747,7 +16747,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-18T12:19:00+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-19 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>56efcece082a87b9731033eca0397d38fcaddb4542500f4540d6fbd490df44e6</t>
+          <t>ca8cdb2d2b9ca1a4eba5e5178f49aba4de3ace3b3b05a88fa5b247f86350b6ca</t>
         </is>
       </c>
     </row>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10995,7 +10995,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11605,7 +11605,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12915,7 +12915,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12953,7 +12953,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13784,7 +13784,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13905,7 +13905,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14115,7 +14115,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14405,7 +14405,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14489,7 +14489,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14531,7 +14531,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14657,7 +14657,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14993,7 +14993,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15035,7 +15035,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15161,7 +15161,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15245,7 +15245,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       <c r="F110" s="2" t="inlineStr"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -15318,7 +15318,7 @@
       <c r="F111" s="2" t="inlineStr"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -15352,7 +15352,7 @@
       <c r="F112" s="2" t="inlineStr"/>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -15389,7 +15389,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15473,7 +15473,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15515,7 +15515,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15557,7 +15557,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15599,7 +15599,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15641,7 +15641,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15683,7 +15683,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15809,7 +15809,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15977,7 +15977,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16019,7 +16019,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16103,7 +16103,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16145,7 +16145,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16271,7 +16271,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16583,7 +16583,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16621,7 +16621,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16697,7 +16697,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16740,7 +16740,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -16777,7 +16777,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16853,7 +16853,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16891,7 +16891,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16967,7 +16967,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-19T12:01:24+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-20 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>ca8cdb2d2b9ca1a4eba5e5178f49aba4de3ace3b3b05a88fa5b247f86350b6ca</t>
+          <t>90b15d324068352a47399957f08b65cbd04e5aa6a144547f6689c0b59989aa5b</t>
         </is>
       </c>
     </row>
@@ -7942,7 +7942,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10995,7 +10995,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11605,7 +11605,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12915,7 +12915,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12953,7 +12953,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13779,12 +13779,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T12:40:36+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13905,7 +13905,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14115,7 +14115,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14405,7 +14405,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14489,7 +14489,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14531,7 +14531,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14657,7 +14657,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14993,7 +14993,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15035,7 +15035,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15161,7 +15161,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15245,7 +15245,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       <c r="F110" s="2" t="inlineStr"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -15318,7 +15318,7 @@
       <c r="F111" s="2" t="inlineStr"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -15352,7 +15352,7 @@
       <c r="F112" s="2" t="inlineStr"/>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -15389,7 +15389,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15473,7 +15473,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15515,7 +15515,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15557,7 +15557,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15599,7 +15599,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15641,7 +15641,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15683,7 +15683,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15809,7 +15809,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15977,7 +15977,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16019,7 +16019,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16103,7 +16103,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16145,7 +16145,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16271,7 +16271,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16583,7 +16583,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16621,7 +16621,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16697,7 +16697,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16735,12 +16735,12 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -16777,7 +16777,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16853,7 +16853,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16891,7 +16891,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16967,7 +16967,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-19T12:01:24+00:00</t>
+          <t>2026-09-20T12:18:51+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-21 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Programs'!$A$1:$N$190</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$H$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Applied'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>90b15d324068352a47399957f08b65cbd04e5aa6a144547f6689c0b59989aa5b</t>
+          <t>f1c69c6c475a19aa68fc1c7a194bfd8553efa4b3521c9f917b1785f1c913e0a1</t>
         </is>
       </c>
     </row>
@@ -7942,12 +7942,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T12:19:00+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>d605a0e1ee5879383316242ff0280132a6a10ea394b4e02b6497340361b17403</t>
+          <t>9b4b34980e7e1794b0658c67468a5ddf19c7220395b0394af11b794579fe2e2e</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10995,7 +10995,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11605,7 +11605,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12915,7 +12915,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12953,7 +12953,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13779,7 +13779,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13905,7 +13905,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14115,7 +14115,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14405,7 +14405,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14489,7 +14489,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14531,7 +14531,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14657,7 +14657,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14993,7 +14993,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15035,7 +15035,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15161,7 +15161,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15245,7 +15245,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15284,7 +15284,7 @@
       <c r="F110" s="2" t="inlineStr"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -15318,7 +15318,7 @@
       <c r="F111" s="2" t="inlineStr"/>
       <c r="G111" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H111" s="2" t="inlineStr">
@@ -15352,7 +15352,7 @@
       <c r="F112" s="2" t="inlineStr"/>
       <c r="G112" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H112" s="2" t="inlineStr">
@@ -15389,7 +15389,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15431,7 +15431,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15473,7 +15473,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15515,7 +15515,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15557,7 +15557,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15599,7 +15599,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15641,7 +15641,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15683,7 +15683,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15725,7 +15725,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15767,7 +15767,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15809,7 +15809,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15851,7 +15851,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15893,7 +15893,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15935,7 +15935,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15977,7 +15977,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16019,7 +16019,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16061,7 +16061,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16103,7 +16103,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16145,7 +16145,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16187,7 +16187,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16229,7 +16229,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16271,7 +16271,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16351,7 +16351,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16389,7 +16389,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16431,7 +16431,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16507,7 +16507,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16545,7 +16545,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16583,7 +16583,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16621,7 +16621,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16659,7 +16659,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16697,7 +16697,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16735,7 +16735,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16777,7 +16777,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16815,7 +16815,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16853,7 +16853,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16891,7 +16891,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -16929,7 +16929,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -16967,7 +16967,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-20T12:18:51+00:00</t>
+          <t>2026-09-21T14:00:58+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -17117,7 +17117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17180,7 +17180,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>appian</t>
+          <t>aperaaiinc</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -17190,27 +17190,27 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:appian</t>
+          <t>greenhouse:aperaaiinc</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/appian/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/aperaaiinc/jobs?content=true</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 172 postings, 10 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 9 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -17222,7 +17222,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>bti36021</t>
+          <t>appian</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -17232,17 +17232,17 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:bti36021</t>
+          <t>greenhouse:appian</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/bti36021/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/appian/jobs?content=true</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 12 postings, 1 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 172 postings, 10 US student rows</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -17264,7 +17264,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>compeerfinancial</t>
+          <t>bti36021</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -17274,17 +17274,17 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:compeerfinancial</t>
+          <t>greenhouse:bti36021</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/bti36021/jobs?content=true</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 12 postings, 1 US student rows</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -17306,7 +17306,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>cssmerge</t>
+          <t>compeerfinancial</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -17316,17 +17316,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:cssmerge</t>
+          <t>greenhouse:compeerfinancial</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -17348,7 +17348,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>devtechnology</t>
+          <t>cssmerge</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -17358,17 +17358,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:devtechnology</t>
+          <t>greenhouse:cssmerge</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -17390,7 +17390,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>eulerity</t>
+          <t>devtechnology</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -17400,17 +17400,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:eulerity</t>
+          <t>greenhouse:devtechnology</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -17432,7 +17432,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>gallup</t>
+          <t>doordashcanada</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -17442,27 +17442,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gallup</t>
+          <t>greenhouse:doordashcanada</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/doordashcanada/jobs?content=true</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 34 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -17474,7 +17474,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>generalmatter</t>
+          <t>doordashusa</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -17484,27 +17484,27 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:generalmatter</t>
+          <t>greenhouse:doordashusa</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/doordashusa/jobs?content=true</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 462 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -17516,7 +17516,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>hpiq</t>
+          <t>duolingounirecruitment</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -17526,27 +17526,27 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hpiq</t>
+          <t>greenhouse:duolingounirecruitment</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/duolingounirecruitment/jobs?content=true</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -17558,7 +17558,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>hudl</t>
+          <t>eulerity</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -17568,17 +17568,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hudl</t>
+          <t>greenhouse:eulerity</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -17600,7 +17600,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>idmeuniversityrecruiting</t>
+          <t>figma</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -17610,27 +17610,27 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:idmeuniversityrecruiting</t>
+          <t>greenhouse:figma</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/figma/jobs?content=true</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 152 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -17642,7 +17642,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>k2spacecorporation</t>
+          <t>gallup</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -17652,17 +17652,17 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:k2spacecorporation</t>
+          <t>greenhouse:gallup</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -17684,7 +17684,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>klaviyocampus</t>
+          <t>generalmatter</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -17694,17 +17694,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:klaviyocampus</t>
+          <t>greenhouse:generalmatter</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>nisc</t>
+          <t>hpiq</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -17736,17 +17736,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:nisc</t>
+          <t>greenhouse:hpiq</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -17768,7 +17768,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>pacificfusion</t>
+          <t>hudl</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -17778,17 +17778,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:pacificfusion</t>
+          <t>greenhouse:hudl</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -17810,7 +17810,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>testnisc</t>
+          <t>idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -17820,17 +17820,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:testnisc</t>
+          <t>greenhouse:idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -17852,27 +17852,27 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Chieler/Summer-2027-SWE-Internships</t>
+          <t>k2spacecorporation</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>repo:chieler/summer-2027-swe-internships</t>
+          <t>greenhouse:k2spacecorporation</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -17894,27 +17894,27 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>sndsh404/summer-2027-internships</t>
+          <t>klaviyocampus</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>repo:sndsh404/summer-2027-internships</t>
+          <t>greenhouse:klaviyocampus</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/sndsh404/summer-2027-internships</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -17931,12 +17931,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>chicagotradingcampus</t>
+          <t>nisc</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -17946,17 +17946,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:chicagotradingcampus</t>
+          <t>greenhouse:nisc</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -17973,12 +17973,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>ctccampusboard</t>
+          <t>pacificfusion</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -17988,17 +17988,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:ctccampusboard</t>
+          <t>greenhouse:pacificfusion</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -18015,12 +18015,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>gardacp</t>
+          <t>testnisc</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -18030,17 +18030,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gardacp</t>
+          <t>greenhouse:testnisc</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -18057,32 +18057,32 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>tgsmc</t>
+          <t>Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>lever</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>lever:tgsmc</t>
+          <t>repo:chieler/summer-2027-swe-internships</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
+          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
+          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -18099,12 +18099,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>vanshb03/Summer2027-Internships</t>
+          <t>sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -18114,17 +18114,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>repo:vanshb03/summer2027-internships</t>
+          <t>repo:sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/vanshb03/Summer2027-Internships</t>
+          <t>https://github.com/sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>9045 stars, pushed 2026-08-23; matched "Summer 2027 Internships"</t>
+          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -18141,210 +18141,210 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Allston Trading</t>
+          <t>chicagotradingcampus</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>allston-trading</t>
+          <t>greenhouse:chicagotradingcampus</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://allstontrading.com</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>AlphaGrep Securities</t>
+          <t>ctccampusboard</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>alphagrep</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>alphagrepsecurities (greenhouse)</t>
+          <t>greenhouse:ctccampusboard</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>AlphaSimplex</t>
+          <t>gardacp</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>alphasimplex</t>
+          <t>greenhouse:gardacp</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://www.alphasimplex.com/</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Arb Trading Group</t>
+          <t>tgsmc</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>lever</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>arb-trading-group</t>
+          <t>lever:tgsmc</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://arb-tg.com/</t>
+          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
+          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Citadel (hedge fund)</t>
+          <t>vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>citadel</t>
+          <t>repo:vanshb03/summer2027-internships</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://www.citadel.com/careers/students/</t>
+          <t>https://github.com/vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
+          <t>9045 stars, pushed 2026-08-23; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -18356,7 +18356,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Consolidated Trading</t>
+          <t>Allston Trading</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -18366,17 +18366,17 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>consolidated-trading</t>
+          <t>allston-trading</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>http://consolidatedtrading.com/</t>
+          <t>https://allstontrading.com</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
+          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -18398,7 +18398,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Cutler Group</t>
+          <t>AlphaGrep Securities</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -18408,17 +18408,17 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>cutler-group</t>
-        </is>
-      </c>
-      <c r="E31" s="3" t="inlineStr">
-        <is>
-          <t>https://cutlerllc.com/</t>
+          <t>alphagrep</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>alphagrepsecurities (greenhouse)</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
+          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -18440,7 +18440,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Dark Forest Technologies</t>
+          <t>AlphaSimplex</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -18450,17 +18450,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>dark-forest-tech</t>
+          <t>alphasimplex</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://darkforesttech.com/</t>
+          <t>https://www.alphasimplex.com/</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
+          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -18482,7 +18482,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Eisler Capital</t>
+          <t>Arb Trading Group</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -18492,17 +18492,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>eisler-capital</t>
+          <t>arb-trading-group</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>https://eislercapital.com</t>
+          <t>https://arb-tg.com/</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
+          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -18524,7 +18524,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Emergent Trading</t>
+          <t>Citadel (hedge fund)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -18534,17 +18534,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>emergent-trading</t>
+          <t>citadel</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://www.emergenttrading.com/join</t>
+          <t>https://www.citadel.com/careers/students/</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
+          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -18566,7 +18566,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Freestone Grove Partners</t>
+          <t>Consolidated Trading</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -18576,17 +18576,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>freestone-grove</t>
+          <t>consolidated-trading</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.gem.com/freestone-grove-partners</t>
+          <t>http://consolidatedtrading.com/</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
+          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -18608,7 +18608,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs Emerging Leaders Series</t>
+          <t>Cutler Group</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -18618,17 +18618,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>goldman-emerging-leaders</t>
+          <t>cutler-group</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
+          <t>https://cutlerllc.com/</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
+          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -18650,7 +18650,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Kinetic Trading Partners</t>
+          <t>Dark Forest Technologies</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -18660,13 +18660,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>kinetic-trading-partners</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr"/>
+          <t>dark-forest-tech</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>https://darkforesttech.com/</t>
+        </is>
+      </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
+          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -18688,7 +18692,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Laurion Capital</t>
+          <t>Eisler Capital</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -18698,17 +18702,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>laurion-capital</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>laurioncapitalmanagement (greenhouse)</t>
+          <t>eisler-capital</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>https://eislercapital.com</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
+          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -18730,7 +18734,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Nico Trading</t>
+          <t>Emergent Trading</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -18740,17 +18744,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>nico-trading</t>
+          <t>emergent-trading</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://nicotrading.com</t>
+          <t>https://www.emergenttrading.com/join</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
+          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -18772,7 +18776,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Numerai</t>
+          <t>Freestone Grove Partners</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -18782,17 +18786,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>numerai</t>
+          <t>freestone-grove</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://numer.ai/careers</t>
+          <t>https://jobs.gem.com/freestone-grove-partners</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
+          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -18814,7 +18818,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Quantitative Investment Management</t>
+          <t>Goldman Sachs Emerging Leaders Series</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -18824,17 +18828,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>qim</t>
+          <t>goldman-emerging-leaders</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://quantitative.com/</t>
+          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
+          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -18856,7 +18860,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Quantbox Research</t>
+          <t>Kinetic Trading Partners</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -18866,17 +18870,13 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>quantbox-research</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>quantboxresearchpte (greenhouse)</t>
-        </is>
-      </c>
+          <t>kinetic-trading-partners</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
+          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -18898,7 +18898,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Quantlab Financial</t>
+          <t>Laurion Capital</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -18908,17 +18908,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>quantlab</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>https://www.quantlab.com/careers</t>
+          <t>laurion-capital</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>laurioncapitalmanagement (greenhouse)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
+          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -18940,7 +18940,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>QVR Advisors</t>
+          <t>Nico Trading</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -18950,17 +18950,17 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>qvr-advisors</t>
+          <t>nico-trading</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>https://qvradvisors.com</t>
+          <t>https://nicotrading.com</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
+          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -18982,7 +18982,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Rosetta Analytics</t>
+          <t>Numerai</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -18992,17 +18992,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>rosetta-analytics</t>
+          <t>numerai</t>
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>https://rosetta-analytics.com/</t>
+          <t>https://numer.ai/careers</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
+          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -19024,7 +19024,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Sensato Investors</t>
+          <t>Quantitative Investment Management</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -19034,17 +19034,17 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>sensato-investors</t>
+          <t>qim</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://sensatoinvestors.com</t>
+          <t>https://quantitative.com/</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
+          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -19066,7 +19066,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Spot Trading</t>
+          <t>Quantbox Research</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -19076,17 +19076,17 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>spot-trading</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>https://spottradingllc.com</t>
+          <t>quantbox-research</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>quantboxresearchpte (greenhouse)</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
+          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -19108,7 +19108,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Summerside Capital</t>
+          <t>Quantlab Financial</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -19118,13 +19118,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>summerside-capital</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr"/>
+          <t>quantlab</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.quantlab.com/careers</t>
+        </is>
+      </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
+          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -19146,7 +19150,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Tyler Capital</t>
+          <t>QVR Advisors</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -19156,17 +19160,17 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>tyler-capital</t>
+          <t>qvr-advisors</t>
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>https://www.tylercapital.co.uk/</t>
+          <t>https://qvradvisors.com</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -19188,7 +19192,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>WH Trading</t>
+          <t>Rosetta Analytics</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -19198,17 +19202,17 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>wh-trading</t>
+          <t>rosetta-analytics</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://whtrading.com/life-at-wh-trading/</t>
+          <t>https://rosetta-analytics.com/</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -19230,42 +19234,248 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
+          <t>Sensato Investors</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>sensato-investors</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>https://sensatoinvestors.com</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Spot Trading</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>spot-trading</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>https://spottradingllc.com</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Summerside Capital</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>summerside-capital</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Tyler Capital</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>tyler-capital</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tylercapital.co.uk/</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>WH Trading</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>wh-trading</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>https://whtrading.com/life-at-wh-trading/</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
           <t>XR Trading</t>
         </is>
       </c>
-      <c r="C51" s="2" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>firm</t>
         </is>
       </c>
-      <c r="D51" s="2" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>xr-trading</t>
         </is>
       </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>https://www.xrtrading.com/</t>
         </is>
       </c>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Paylocity React shell: board returns 670 chars, all of it 'unsupported browser' boilerplate, zero titles. Bundle grepped - no JSON endpoint exists.</t>
         </is>
       </c>
-      <c r="G51" s="2" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
+      <c r="H56" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H51"/>
+  <autoFilter ref="A1:H56"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -19291,27 +19501,32 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: 2026-09-22 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr"/>
@@ -4482,7 +4482,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7810,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7874,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7890,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>f1c69c6c475a19aa68fc1c7a194bfd8553efa4b3521c9f917b1785f1c913e0a1</t>
+          <t>7c177cf55b24ea1cfcfef30c9acbe7b9219b6ea5c191c0e78820e7d94f81a0e3</t>
         </is>
       </c>
     </row>
@@ -7942,12 +7942,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -7958,7 +7958,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>9b4b34980e7e1794b0658c67468a5ddf19c7220395b0394af11b794579fe2e2e</t>
+          <t>5211633896d1f19a2c25272d82debf587fe742b7b9611d3239d20246ed9b2213</t>
         </is>
       </c>
     </row>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8074,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8410,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8674,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8742,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8814,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10506,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10915,7 +10915,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10953,7 +10953,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10991,7 +10991,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11029,7 +11029,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11067,7 +11067,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11105,7 +11105,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11147,7 +11147,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11189,7 +11189,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11231,7 +11231,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11273,7 +11273,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11399,7 +11399,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11437,7 +11437,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11517,7 +11517,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11559,7 +11559,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11601,7 +11601,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11643,7 +11643,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11723,7 +11723,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11761,7 +11761,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11841,7 +11841,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11921,7 +11921,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11959,7 +11959,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12001,7 +12001,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12039,7 +12039,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12081,7 +12081,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12119,7 +12119,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12157,7 +12157,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12195,7 +12195,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12233,7 +12233,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12271,7 +12271,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12309,7 +12309,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12351,7 +12351,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12389,7 +12389,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12431,7 +12431,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12473,7 +12473,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12511,7 +12511,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12587,7 +12587,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12629,7 +12629,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12667,7 +12667,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12709,7 +12709,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12751,7 +12751,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12789,7 +12789,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12831,7 +12831,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12873,7 +12873,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12911,7 +12911,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12949,7 +12949,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12991,7 +12991,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13033,7 +13033,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13075,7 +13075,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13113,7 +13113,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13151,7 +13151,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13189,7 +13189,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13227,7 +13227,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13265,7 +13265,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13307,7 +13307,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13345,7 +13345,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13387,7 +13387,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13425,7 +13425,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13463,7 +13463,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13501,7 +13501,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13539,7 +13539,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13733,7 +13733,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13775,7 +13775,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -13817,7 +13817,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13859,7 +13859,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13901,7 +13901,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13943,7 +13943,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13985,7 +13985,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14027,7 +14027,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14069,7 +14069,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14111,7 +14111,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14153,7 +14153,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14195,7 +14195,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14233,7 +14233,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14275,7 +14275,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14317,7 +14317,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14359,7 +14359,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14401,7 +14401,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14485,7 +14485,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14527,7 +14527,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14569,7 +14569,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14611,7 +14611,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14653,7 +14653,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14695,7 +14695,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14737,7 +14737,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14779,7 +14779,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14821,7 +14821,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14863,7 +14863,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14905,7 +14905,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14947,7 +14947,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14989,7 +14989,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15031,7 +15031,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15073,7 +15073,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15115,7 +15115,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15157,7 +15157,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15199,7 +15199,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15241,7 +15241,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15283,7 +15283,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15325,7 +15325,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15367,7 +15367,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15409,7 +15409,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15451,7 +15451,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15493,7 +15493,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15535,7 +15535,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15577,7 +15577,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15617,7 +15617,11 @@
           <t>https://solayer.org/careers</t>
         </is>
       </c>
-      <c r="F118" s="2" t="inlineStr"/>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22T12:39:39+00:00</t>
+        </is>
+      </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -15657,7 +15661,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15699,7 +15703,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15741,7 +15745,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15783,7 +15787,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15825,7 +15829,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15867,7 +15871,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15909,7 +15913,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15951,7 +15955,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15993,7 +15997,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16035,7 +16039,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16077,7 +16081,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16119,7 +16123,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16161,7 +16165,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16203,7 +16207,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16245,7 +16249,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16283,7 +16287,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16321,7 +16325,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16363,7 +16367,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16401,7 +16405,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16439,7 +16443,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16477,7 +16481,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16515,7 +16519,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16553,7 +16557,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16591,7 +16595,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16629,7 +16633,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16667,7 +16671,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16709,7 +16713,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16747,7 +16751,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16785,7 +16789,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16823,7 +16827,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16861,7 +16865,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16899,7 +16903,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:00:58+00:00</t>
+          <t>2026-09-22T12:39:39+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-23 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2873,15 +2873,19 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr"/>
+          <t>2026-09-23T12:49:57+00:00</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23T12:49:57+00:00</t>
+        </is>
+      </c>
       <c r="L46" s="2" t="inlineStr"/>
       <c r="M46" s="2" t="inlineStr">
         <is>
@@ -2890,7 +2894,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>36cfe7e7863f9d1460b8dc4a91e8c1baec01e9664a492fb99d918b34bf2b6ea3</t>
+          <t>2959d548616852711e1dc9a8dabc9bed791fca8d77122e8792af1c662e96519b</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4486,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7810,7 +7814,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7874,12 +7878,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7890,7 +7894,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>7c177cf55b24ea1cfcfef30c9acbe7b9219b6ea5c191c0e78820e7d94f81a0e3</t>
+          <t>d874699a98a98c1eb6c7ef79f07d060a6e16093391ef7df0168b3c8947dd3762</t>
         </is>
       </c>
     </row>
@@ -7942,7 +7946,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8010,7 +8014,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8074,7 +8078,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8410,7 +8414,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8478,7 +8482,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8546,7 +8550,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8674,7 +8678,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8742,7 +8746,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8814,7 +8818,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10506,7 +10510,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10915,7 +10919,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10953,7 +10957,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10991,7 +10995,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11029,7 +11033,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11067,7 +11071,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11105,7 +11109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11147,7 +11151,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11189,7 +11193,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11231,7 +11235,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11273,7 +11277,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11315,7 +11319,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11357,7 +11361,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11399,7 +11403,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11437,7 +11441,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11479,7 +11483,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11517,7 +11521,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11559,7 +11563,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11601,7 +11605,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11643,7 +11647,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11685,7 +11689,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11723,7 +11727,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11761,7 +11765,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11799,7 +11803,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11841,7 +11845,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11883,7 +11887,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11921,7 +11925,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11959,7 +11963,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12001,7 +12005,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12039,7 +12043,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12081,7 +12085,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12119,7 +12123,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12157,7 +12161,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12195,7 +12199,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12233,7 +12237,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12271,7 +12275,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12309,7 +12313,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12351,7 +12355,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12389,7 +12393,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12431,7 +12435,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12473,7 +12477,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12511,7 +12515,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12549,7 +12553,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12587,7 +12591,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12629,7 +12633,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12667,7 +12671,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12709,7 +12713,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12751,7 +12755,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12789,7 +12793,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12831,7 +12835,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12873,7 +12877,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12911,7 +12915,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12949,7 +12953,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12991,7 +12995,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13033,7 +13037,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13075,7 +13079,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13113,7 +13117,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13151,7 +13155,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13189,7 +13193,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13227,7 +13231,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13265,7 +13269,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13307,7 +13311,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13345,7 +13349,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13387,7 +13391,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13425,7 +13429,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13463,7 +13467,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13501,7 +13505,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13539,7 +13543,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13733,7 +13737,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13780,7 +13784,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13817,7 +13821,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13859,7 +13863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13901,7 +13905,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13943,7 +13947,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13985,7 +13989,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14027,7 +14031,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14069,7 +14073,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14111,7 +14115,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14153,7 +14157,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14195,7 +14199,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14233,7 +14237,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14275,7 +14279,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14317,7 +14321,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14359,7 +14363,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14401,7 +14405,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14443,7 +14447,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14485,7 +14489,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14527,7 +14531,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14569,7 +14573,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14611,7 +14615,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14653,7 +14657,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14695,7 +14699,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14737,7 +14741,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14779,7 +14783,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14821,7 +14825,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14863,7 +14867,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14905,7 +14909,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14947,7 +14951,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14989,7 +14993,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15031,7 +15035,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15073,7 +15077,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15115,7 +15119,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15157,7 +15161,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15199,7 +15203,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15241,7 +15245,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15283,7 +15287,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15325,7 +15329,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15367,7 +15371,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15409,7 +15413,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15451,7 +15455,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15493,7 +15497,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15535,7 +15539,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15577,7 +15581,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15619,7 +15623,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15661,7 +15665,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15703,7 +15707,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15745,7 +15749,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15787,7 +15791,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15829,7 +15833,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15871,7 +15875,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15913,7 +15917,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15955,7 +15959,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -15997,7 +16001,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16039,7 +16043,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16081,7 +16085,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16123,7 +16127,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16165,7 +16169,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16207,7 +16211,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16249,7 +16253,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16287,7 +16291,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16325,7 +16329,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16367,7 +16371,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16405,7 +16409,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16443,7 +16447,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16481,7 +16485,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16519,7 +16523,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16557,7 +16561,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16595,7 +16599,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16633,7 +16637,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16671,7 +16675,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16713,7 +16717,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16751,7 +16755,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16789,7 +16793,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16827,7 +16831,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16865,7 +16869,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16903,7 +16907,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-23T12:49:57+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-24 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7878,12 +7878,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>d874699a98a98c1eb6c7ef79f07d060a6e16093391ef7df0168b3c8947dd3762</t>
+          <t>f54812d8301383ddec3b01e830249087e4ff30b95a4a40528d71c41c593cfb07</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr"/>
@@ -8550,7 +8550,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8746,7 +8746,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8818,7 +8818,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10510,7 +10510,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10919,7 +10919,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10957,7 +10957,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10995,7 +10995,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11033,7 +11033,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11071,7 +11071,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11109,7 +11109,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11151,7 +11151,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11193,7 +11193,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11235,7 +11235,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11277,7 +11277,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11319,7 +11319,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11361,7 +11361,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11403,7 +11403,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11483,7 +11483,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11521,7 +11521,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11563,7 +11563,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11605,7 +11605,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11647,7 +11647,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11689,7 +11689,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11727,7 +11727,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11765,7 +11765,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11803,7 +11803,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11845,7 +11845,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11887,7 +11887,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11925,7 +11925,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11963,7 +11963,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12005,7 +12005,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12043,7 +12043,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12085,7 +12085,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12123,7 +12123,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12161,7 +12161,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12199,7 +12199,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12275,7 +12275,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12313,7 +12313,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12355,7 +12355,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12393,7 +12393,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12435,7 +12435,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12477,7 +12477,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12515,7 +12515,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12591,7 +12591,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12633,7 +12633,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12671,7 +12671,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12713,7 +12713,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12755,7 +12755,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12793,7 +12793,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12835,7 +12835,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12877,7 +12877,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12915,7 +12915,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12953,7 +12953,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12995,7 +12995,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13037,7 +13037,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13079,7 +13079,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13155,7 +13155,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13193,7 +13193,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13231,7 +13231,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13269,7 +13269,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13311,7 +13311,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13349,7 +13349,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13391,7 +13391,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13467,7 +13467,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13505,7 +13505,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13543,7 +13543,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13737,7 +13737,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13784,7 +13784,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13863,7 +13863,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13905,7 +13905,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13947,7 +13947,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13989,7 +13989,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14031,7 +14031,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14073,7 +14073,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14115,7 +14115,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14157,7 +14157,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14199,7 +14199,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14237,7 +14237,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14279,7 +14279,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14321,7 +14321,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14363,7 +14363,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14405,7 +14405,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14447,7 +14447,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14489,7 +14489,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14531,7 +14531,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14573,7 +14573,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14615,7 +14615,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14657,7 +14657,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14699,7 +14699,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14741,7 +14741,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -14825,7 +14825,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14867,7 +14867,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14909,7 +14909,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14951,7 +14951,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14993,7 +14993,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15035,7 +15035,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15077,7 +15077,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15161,7 +15161,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15203,7 +15203,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15245,7 +15245,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15287,7 +15287,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15329,7 +15329,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15371,7 +15371,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15413,7 +15413,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15455,7 +15455,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15497,7 +15497,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15539,7 +15539,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15581,7 +15581,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15623,7 +15623,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15665,7 +15665,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15707,7 +15707,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15754,7 +15754,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -15791,7 +15791,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15833,7 +15833,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15875,7 +15875,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15917,7 +15917,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15959,7 +15959,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -16001,7 +16001,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16043,7 +16043,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16085,7 +16085,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16127,7 +16127,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16169,7 +16169,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16211,7 +16211,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16253,7 +16253,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16291,7 +16291,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16371,7 +16371,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16409,7 +16409,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16447,7 +16447,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16485,7 +16485,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16523,7 +16523,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16561,7 +16561,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16599,7 +16599,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16637,7 +16637,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16675,7 +16675,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16717,7 +16717,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16755,7 +16755,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16793,7 +16793,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16831,7 +16831,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16869,7 +16869,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16907,7 +16907,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-24T12:48:38+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-25 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7878,12 +7878,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>f54812d8301383ddec3b01e830249087e4ff30b95a4a40528d71c41c593cfb07</t>
+          <t>9d50868a4f375af4073f1702fa95c5beab51ce17ecb88c6afbda4f6caaea8e5d</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8482,10 +8482,14 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
-        </is>
-      </c>
-      <c r="K153" s="2" t="inlineStr"/>
+          <t>2026-09-25T12:50:11+00:00</t>
+        </is>
+      </c>
+      <c r="K153" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25T12:50:11+00:00</t>
+        </is>
+      </c>
       <c r="L153" s="2" t="inlineStr">
         <is>
           <t>2026-09-06</t>
@@ -8498,7 +8502,7 @@
       </c>
       <c r="N153" s="2" t="inlineStr">
         <is>
-          <t>9ffe37a558c138b12b627dad42b2b5031f97c8f9606ff73420c4d90e25a5aa62</t>
+          <t>6719b2608fc54b0cd475a3bec8eddd667a0640a47d368c62655d2344e22e2a66</t>
         </is>
       </c>
     </row>
@@ -8550,7 +8554,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8678,7 +8682,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8746,7 +8750,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8818,7 +8822,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10510,7 +10514,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10919,7 +10923,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10957,7 +10961,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10995,7 +10999,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11033,7 +11037,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11071,7 +11075,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11109,7 +11113,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11151,7 +11155,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11193,7 +11197,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11235,7 +11239,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11277,7 +11281,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11319,7 +11323,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11361,7 +11365,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11403,7 +11407,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11441,7 +11445,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11483,7 +11487,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11521,7 +11525,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11563,7 +11567,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11605,7 +11609,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11647,7 +11651,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11689,7 +11693,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11727,7 +11731,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11765,7 +11769,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11803,7 +11807,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11845,7 +11849,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11887,7 +11891,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11925,7 +11929,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11963,7 +11967,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12005,7 +12009,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12043,7 +12047,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12085,7 +12089,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12123,7 +12127,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12161,7 +12165,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12199,7 +12203,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12237,7 +12241,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12275,7 +12279,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12313,7 +12317,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12355,7 +12359,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12393,7 +12397,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12435,7 +12439,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12477,7 +12481,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12515,7 +12519,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12553,7 +12557,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12591,7 +12595,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12633,7 +12637,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12671,7 +12675,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12713,7 +12717,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12755,7 +12759,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12793,7 +12797,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12835,7 +12839,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12877,7 +12881,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12915,7 +12919,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12953,7 +12957,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12995,7 +12999,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13037,7 +13041,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13079,7 +13083,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13117,7 +13121,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13155,7 +13159,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13193,7 +13197,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13231,7 +13235,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13269,7 +13273,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13311,7 +13315,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13349,7 +13353,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13391,7 +13395,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13429,7 +13433,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13467,7 +13471,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13505,7 +13509,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13543,7 +13547,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13737,7 +13741,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13779,12 +13783,12 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -13821,7 +13825,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13863,7 +13867,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13905,7 +13909,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13947,7 +13951,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13989,7 +13993,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14031,7 +14035,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14073,7 +14077,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14115,7 +14119,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14157,7 +14161,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14199,7 +14203,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14237,7 +14241,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14279,7 +14283,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14321,7 +14325,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14363,7 +14367,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14405,7 +14409,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14447,7 +14451,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14489,7 +14493,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14531,7 +14535,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14573,7 +14577,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14615,7 +14619,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14657,7 +14661,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14699,7 +14703,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14746,7 +14750,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -14788,7 +14792,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -14825,7 +14829,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14867,7 +14871,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14909,7 +14913,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14951,7 +14955,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14993,7 +14997,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15035,7 +15039,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15077,7 +15081,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15119,7 +15123,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15161,7 +15165,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15203,7 +15207,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15245,7 +15249,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15287,7 +15291,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15329,7 +15333,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15371,7 +15375,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15413,7 +15417,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15455,7 +15459,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15497,7 +15501,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15539,7 +15543,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15581,7 +15585,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15623,7 +15627,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15665,7 +15669,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15707,7 +15711,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15749,12 +15753,12 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T12:49:57+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -15791,7 +15795,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15833,7 +15837,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15875,7 +15879,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15917,7 +15921,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15959,7 +15963,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -16001,7 +16005,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16043,7 +16047,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16085,7 +16089,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16127,7 +16131,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16169,7 +16173,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16211,7 +16215,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16253,7 +16257,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16291,7 +16295,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16329,7 +16333,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16371,7 +16375,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16409,7 +16413,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16447,7 +16451,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16485,7 +16489,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16523,7 +16527,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16561,7 +16565,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16599,7 +16603,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16637,7 +16641,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16675,7 +16679,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16717,7 +16721,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16755,7 +16759,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16793,7 +16797,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16831,7 +16835,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16869,7 +16873,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16907,7 +16911,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T12:48:38+00:00</t>
+          <t>2026-09-25T12:50:11+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-26 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2878,7 +2878,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -4486,7 +4486,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -7814,7 +7814,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -7878,12 +7878,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -7894,7 +7894,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>9d50868a4f375af4073f1702fa95c5beab51ce17ecb88c6afbda4f6caaea8e5d</t>
+          <t>25d9060444d819c24c18ac01280aa99235cc539bc0d5501e340e0abdaa16ad27</t>
         </is>
       </c>
     </row>
@@ -7946,7 +7946,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8014,7 +8014,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8078,7 +8078,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8414,7 +8414,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8482,7 +8482,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8554,7 +8554,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8682,7 +8682,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8750,7 +8750,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8822,7 +8822,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10514,7 +10514,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -10961,7 +10961,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -10999,7 +10999,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -11037,7 +11037,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -11075,7 +11075,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -11113,7 +11113,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -11155,7 +11155,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -11197,7 +11197,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -11239,7 +11239,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -11281,7 +11281,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -11365,7 +11365,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -11407,7 +11407,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -11445,7 +11445,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -11525,7 +11525,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -11567,7 +11567,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -11609,7 +11609,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -11651,7 +11651,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -11693,7 +11693,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -11731,7 +11731,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -11769,7 +11769,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -11807,7 +11807,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -11849,7 +11849,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -11891,7 +11891,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -11967,7 +11967,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -12047,7 +12047,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -12089,7 +12089,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -12127,7 +12127,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -12165,7 +12165,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -12203,7 +12203,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -12241,7 +12241,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -12279,7 +12279,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -12317,7 +12317,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -12359,7 +12359,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -12397,7 +12397,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -12439,7 +12439,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -12481,7 +12481,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -12519,7 +12519,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -12557,7 +12557,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -12595,7 +12595,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -12637,7 +12637,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -12675,7 +12675,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -12717,7 +12717,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -12759,7 +12759,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -12797,7 +12797,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -12839,7 +12839,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -12881,7 +12881,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -12919,7 +12919,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -12957,7 +12957,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -12999,7 +12999,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -13041,7 +13041,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -13083,7 +13083,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -13121,7 +13121,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -13159,7 +13159,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -13197,7 +13197,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -13235,7 +13235,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -13315,7 +13315,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -13353,7 +13353,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -13395,7 +13395,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -13471,7 +13471,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -13509,7 +13509,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -13547,7 +13547,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -13783,7 +13783,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -13825,7 +13825,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -13867,7 +13867,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -13909,7 +13909,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -13951,7 +13951,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -13993,7 +13993,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -14035,7 +14035,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -14077,7 +14077,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -14119,7 +14119,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -14161,7 +14161,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -14203,7 +14203,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -14283,7 +14283,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -14325,7 +14325,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -14367,7 +14367,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -14409,7 +14409,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -14451,7 +14451,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -14493,7 +14493,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -14535,7 +14535,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -14577,7 +14577,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -14619,7 +14619,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -14661,7 +14661,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -14703,7 +14703,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -14750,7 +14750,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -14792,7 +14792,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -14829,7 +14829,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -14871,7 +14871,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -14913,7 +14913,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -14955,7 +14955,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -14997,7 +14997,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -15039,7 +15039,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -15081,7 +15081,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -15123,7 +15123,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -15165,7 +15165,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -15207,7 +15207,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -15249,7 +15249,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -15291,7 +15291,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -15333,7 +15333,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -15375,7 +15375,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -15417,7 +15417,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -15459,7 +15459,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -15501,7 +15501,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -15543,7 +15543,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -15585,7 +15585,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -15627,7 +15627,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -15669,7 +15669,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -15753,7 +15753,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -15795,7 +15795,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -15837,7 +15837,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -15879,7 +15879,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -15921,7 +15921,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -15963,7 +15963,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -16005,7 +16005,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -16047,7 +16047,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -16089,7 +16089,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -16131,7 +16131,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -16173,7 +16173,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -16215,7 +16215,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -16257,7 +16257,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -16295,7 +16295,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -16333,7 +16333,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -16375,7 +16375,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -16413,7 +16413,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -16451,7 +16451,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -16489,7 +16489,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -16527,7 +16527,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -16565,7 +16565,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -16603,7 +16603,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -16641,7 +16641,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -16679,7 +16679,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -16721,7 +16721,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -16759,7 +16759,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -16797,7 +16797,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -16835,7 +16835,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -16873,7 +16873,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -16911,7 +16911,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:50:11+00:00</t>
+          <t>2026-09-26T12:17:03+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-28 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -16,7 +16,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'All Programs'!$A$1:$N$213</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Sources'!$A$1:$H$192</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Applied'!$A$1:$C$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Discovered'!$A$1:$H$58</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -3804,7 +3804,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N63" s="2" t="inlineStr"/>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>a6d079ec7f9100088d25f39f43f86faf2667be43dd7f05f21fd7b900739a3760</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -4102,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4166,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4230,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4294,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
@@ -4358,7 +4362,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4422,7 +4426,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4590,7 +4594,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5114,7 +5118,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6498,10 +6502,14 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
-        </is>
-      </c>
-      <c r="K114" s="2" t="inlineStr"/>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L114" s="2" t="inlineStr"/>
       <c r="M114" s="2" t="inlineStr">
         <is>
@@ -6510,7 +6518,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>c73cabb199b26e430f8dee053f572be42d8f6665df50643fb64e8ca6bf064772</t>
+          <t>62d32530d603b027f9449498244ff9de23502a87dc8d606d86478637471e5684</t>
         </is>
       </c>
     </row>
@@ -6666,7 +6674,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6730,7 +6738,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7970,7 +7978,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8034,12 +8042,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8050,7 +8058,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>52802246bbef831b31b7e9d9be931e4e3fa5f7ffe9138e5e40daa184a7e65486</t>
+          <t>4f009f794507f781652d228af6a53f321291f2e3ce5f378536471ea3d600b2e5</t>
         </is>
       </c>
     </row>
@@ -8102,12 +8110,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T12:39:39+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8118,7 +8126,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>5211633896d1f19a2c25272d82debf587fe742b7b9611d3239d20246ed9b2213</t>
+          <t>25f3e22ab690e5dc0b3394bca1518de4dc0a25382e535bd2abdd744ff813ee90</t>
         </is>
       </c>
     </row>
@@ -8170,7 +8178,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8234,7 +8242,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8570,7 +8578,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8638,7 +8646,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8710,7 +8718,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8838,7 +8846,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8906,7 +8914,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8978,7 +8986,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10670,7 +10678,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10850,7 +10858,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10918,7 +10926,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr"/>
@@ -10986,10 +10994,14 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
-        </is>
-      </c>
-      <c r="K193" s="2" t="inlineStr"/>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L193" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11002,7 +11014,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>508589d77b4091cb91503fd2e8f89c487efe1700ee453cdab3fd578c2506a127</t>
+          <t>8d5be6c2e2d53d3c482b997109b4d440a4cb9f42b421c59e9660932a23a483b9</t>
         </is>
       </c>
     </row>
@@ -11054,7 +11066,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr"/>
@@ -11122,10 +11134,14 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
-        </is>
-      </c>
-      <c r="K195" s="2" t="inlineStr"/>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L195" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11138,7 +11154,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>24b7e680af6978f17b5eebaf4a17959124498c2ab61679421666e71ecc2c4b3f</t>
+          <t>4a082bd8ae515f500fdf636e7d9d1b17188a776a9936aee26a03d7a531030ddc</t>
         </is>
       </c>
     </row>
@@ -11190,7 +11206,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr"/>
@@ -11258,7 +11274,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr"/>
@@ -11326,7 +11342,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11394,7 +11410,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11462,7 +11478,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11530,7 +11546,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr"/>
@@ -11598,7 +11614,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11666,7 +11682,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11734,7 +11750,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr"/>
@@ -11802,7 +11818,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11870,7 +11886,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K206" s="2" t="inlineStr"/>
@@ -11934,10 +11950,14 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
-        </is>
-      </c>
-      <c r="K207" s="2" t="inlineStr"/>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L207" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11950,7 +11970,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>91d5fb062194e170ca2e9688a9586bacd8e1202b3cbcbe53555801441f8118e9</t>
+          <t>8f5ce11e6e144e5fcab44fb1da76c9a2231fa37f5ec7c670d3e7d7ee137c39fc</t>
         </is>
       </c>
     </row>
@@ -12002,7 +12022,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12070,10 +12090,14 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
-        </is>
-      </c>
-      <c r="K209" s="2" t="inlineStr"/>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="L209" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -12086,7 +12110,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12138,7 +12162,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12626,7 +12650,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -12664,7 +12688,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -12702,7 +12726,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -12740,7 +12764,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -12778,7 +12802,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -12816,7 +12840,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -12858,7 +12882,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -12900,7 +12924,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -12942,7 +12966,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -12984,7 +13008,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -13026,7 +13050,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -13068,7 +13092,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -13110,7 +13134,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -13152,7 +13176,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13194,7 +13218,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -13232,7 +13256,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -13274,7 +13298,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -13312,7 +13336,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -13354,7 +13378,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13396,7 +13420,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -13438,7 +13462,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -13480,7 +13504,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -13522,7 +13546,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -13560,7 +13584,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -13598,7 +13622,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -13636,7 +13660,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -13678,7 +13702,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -13720,7 +13744,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -13758,7 +13782,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -13796,7 +13820,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -13838,7 +13862,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -13876,7 +13900,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -13918,7 +13942,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -13956,7 +13980,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -13994,7 +14018,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -14032,7 +14056,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -14070,7 +14094,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -14108,7 +14132,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -14146,7 +14170,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -14188,7 +14212,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -14226,7 +14250,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -14268,7 +14292,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -14310,7 +14334,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -14352,7 +14376,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -14390,7 +14414,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -14428,7 +14452,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -14466,7 +14490,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -14508,7 +14532,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -14546,7 +14570,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -14588,7 +14612,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -14630,7 +14654,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -14668,7 +14692,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -14710,7 +14734,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -14752,7 +14776,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -14790,7 +14814,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -14832,7 +14856,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -14870,7 +14894,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -14912,7 +14936,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -14954,7 +14978,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -14996,7 +15020,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -15034,7 +15058,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -15072,7 +15096,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -15110,7 +15134,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -15148,7 +15172,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -15186,7 +15210,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -15228,7 +15252,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -15266,7 +15290,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -15308,7 +15332,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -15346,7 +15370,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -15388,7 +15412,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -15426,7 +15450,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -15464,7 +15488,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -15502,7 +15526,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -15696,7 +15720,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15743,7 +15767,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -15780,7 +15804,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15822,7 +15846,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15864,7 +15888,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15906,7 +15930,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15948,7 +15972,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -15990,7 +16014,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16032,7 +16056,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16074,7 +16098,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -16116,7 +16140,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -16158,7 +16182,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -16200,7 +16224,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -16242,7 +16266,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -16284,7 +16308,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -16326,7 +16350,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -16368,7 +16392,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -16410,7 +16434,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -16452,7 +16476,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -16494,7 +16518,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -16536,7 +16560,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -16578,7 +16602,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -16616,7 +16640,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -16658,7 +16682,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -16700,7 +16724,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -16742,7 +16766,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -16784,7 +16808,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -16826,7 +16850,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -16868,7 +16892,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -16910,7 +16934,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -16952,7 +16976,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -16994,7 +17018,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -17036,7 +17060,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -17078,7 +17102,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -17120,7 +17144,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -17162,7 +17186,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -17209,7 +17233,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -17251,7 +17275,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -17288,7 +17312,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -17330,7 +17354,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -17372,7 +17396,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -17414,7 +17438,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -17456,7 +17480,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -17498,7 +17522,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -17540,7 +17564,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -17582,7 +17606,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -17624,7 +17648,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -17666,7 +17690,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -17708,7 +17732,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -17750,7 +17774,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -17792,7 +17816,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -17834,7 +17858,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -17876,7 +17900,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -17918,7 +17942,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -17960,7 +17984,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -18002,7 +18026,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -18044,7 +18068,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -18086,7 +18110,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -18128,7 +18152,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -18170,7 +18194,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -18212,7 +18236,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -18254,7 +18278,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -18296,7 +18320,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -18338,7 +18362,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -18380,7 +18404,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -18422,7 +18446,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -18464,7 +18488,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -18506,7 +18530,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -18548,7 +18572,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -18590,7 +18614,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -18632,7 +18656,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -18674,7 +18698,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -18717,7 +18741,7 @@
       <c r="F151" s="2" t="inlineStr"/>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -18754,7 +18778,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -18796,7 +18820,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -18838,7 +18862,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -18880,7 +18904,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -18922,7 +18946,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -18964,7 +18988,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -19006,7 +19030,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -19048,7 +19072,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -19090,7 +19114,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -19132,7 +19156,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -19174,7 +19198,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -19216,7 +19240,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -19258,7 +19282,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -19300,7 +19324,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -19342,7 +19366,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -19384,7 +19408,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -19424,10 +19448,14 @@
           <t>https://www.worldquant.com/brain/iqc/</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr"/>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28T15:25:45+00:00</t>
+        </is>
+      </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -19464,7 +19492,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -19506,7 +19534,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -19548,7 +19576,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -19590,7 +19618,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -19628,7 +19656,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -19670,7 +19698,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -19708,7 +19736,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -19750,7 +19778,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -19792,7 +19820,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -19830,7 +19858,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -19868,7 +19896,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -19906,7 +19934,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -19944,7 +19972,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -19982,7 +20010,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -20020,7 +20048,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -20058,7 +20086,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -20096,7 +20124,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -20138,7 +20166,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -20180,7 +20208,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -20218,7 +20246,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -20256,7 +20284,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -20294,7 +20322,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -20332,7 +20360,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -20370,7 +20398,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-09-28T15:25:45+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -20554,7 +20582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20701,7 +20729,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>bti36021</t>
+          <t>astranis</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -20711,27 +20739,27 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:bti36021</t>
+          <t>greenhouse:astranis</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/bti36021/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/astranis/jobs?content=true</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 12 postings, 1 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 164 postings, 86 US student rows</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -20743,7 +20771,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>compeerfinancial</t>
+          <t>bti36021</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -20753,17 +20781,17 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:compeerfinancial</t>
+          <t>greenhouse:bti36021</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/bti36021/jobs?content=true</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 12 postings, 1 US student rows</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -20785,7 +20813,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>cssmerge</t>
+          <t>compeerfinancial</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -20795,17 +20823,17 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:cssmerge</t>
+          <t>greenhouse:compeerfinancial</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/compeerfinancial/jobs?content=true</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 67 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -20827,7 +20855,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>devtechnology</t>
+          <t>cssmerge</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -20837,17 +20865,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:devtechnology</t>
+          <t>greenhouse:cssmerge</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/cssmerge/jobs?content=true</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 245 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -20869,7 +20897,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>doordashcanada</t>
+          <t>devtechnology</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -20879,27 +20907,27 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:doordashcanada</t>
+          <t>greenhouse:devtechnology</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/doordashcanada/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/devtechnology/jobs?content=true</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 34 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 26 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -20911,7 +20939,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>doordashusa</t>
+          <t>doordashcanada</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -20921,17 +20949,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:doordashusa</t>
+          <t>greenhouse:doordashcanada</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/doordashusa/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/doordashcanada/jobs?content=true</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 462 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 34 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -20953,7 +20981,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>duolingounirecruitment</t>
+          <t>doordashusa</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -20963,17 +20991,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:duolingounirecruitment</t>
+          <t>greenhouse:doordashusa</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/duolingounirecruitment/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/doordashusa/jobs?content=true</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 3 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 462 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -20995,7 +21023,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>eulerity</t>
+          <t>duolingounirecruitment</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -21005,27 +21033,27 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:eulerity</t>
+          <t>greenhouse:duolingounirecruitment</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/duolingounirecruitment/jobs?content=true</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -21037,7 +21065,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>figma</t>
+          <t>eulerity</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -21047,27 +21075,27 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:figma</t>
+          <t>greenhouse:eulerity</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/figma/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/eulerity/jobs?content=true</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 152 postings, 6 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 17 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -21079,7 +21107,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>gallup</t>
+          <t>figma</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -21089,27 +21117,27 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gallup</t>
+          <t>greenhouse:figma</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/figma/jobs?content=true</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 152 postings, 6 US student rows</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
@@ -21121,7 +21149,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>generalmatter</t>
+          <t>gallup</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -21131,17 +21159,17 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:generalmatter</t>
+          <t>greenhouse:gallup</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gallup/jobs?content=true</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 54 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -21163,7 +21191,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>hpiq</t>
+          <t>generalmatter</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -21173,17 +21201,17 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hpiq</t>
+          <t>greenhouse:generalmatter</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/generalmatter/jobs?content=true</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 132 postings, 24 US student rows</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -21205,7 +21233,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>hudl</t>
+          <t>hpiq</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -21215,17 +21243,17 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:hudl</t>
+          <t>greenhouse:hpiq</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hpiq/jobs?content=true</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 32 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -21247,7 +21275,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>idmeuniversityrecruiting</t>
+          <t>hudl</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -21257,17 +21285,17 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:idmeuniversityrecruiting</t>
+          <t>greenhouse:hudl</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/hudl/jobs?content=true</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 31 postings, 3 US student rows</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -21289,7 +21317,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>k2spacecorporation</t>
+          <t>idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -21299,17 +21327,17 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:k2spacecorporation</t>
+          <t>greenhouse:idmeuniversityrecruiting</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/idmeuniversityrecruiting/jobs?content=true</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 7 postings, 7 US student rows</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -21331,7 +21359,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>klaviyocampus</t>
+          <t>k2spacecorporation</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -21341,17 +21369,17 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:klaviyocampus</t>
+          <t>greenhouse:k2spacecorporation</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/k2spacecorporation/jobs?content=true</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 219 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -21373,7 +21401,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>nisc</t>
+          <t>klaviyocampus</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -21383,17 +21411,17 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:nisc</t>
+          <t>greenhouse:klaviyocampus</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/klaviyocampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 3 postings, 2 US student rows</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -21415,7 +21443,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>pacificfusion</t>
+          <t>nisc</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -21425,17 +21453,17 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:pacificfusion</t>
+          <t>greenhouse:nisc</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/nisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 39 postings, 8 US student rows</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -21457,7 +21485,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>testnisc</t>
+          <t>pacificfusion</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -21467,17 +21495,17 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:testnisc</t>
+          <t>greenhouse:pacificfusion</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/pacificfusion/jobs?content=true</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 5 US student rows</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -21499,27 +21527,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Chieler/Summer-2027-SWE-Internships</t>
+          <t>testnisc</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>repo:chieler/summer-2027-swe-internships</t>
+          <t>greenhouse:testnisc</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/testnisc/jobs?content=true</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 37 postings, 9 US student rows</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -21541,7 +21569,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>sndsh404/summer-2027-internships</t>
+          <t>Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -21551,17 +21579,17 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>repo:sndsh404/summer-2027-internships</t>
+          <t>repo:chieler/summer-2027-swe-internships</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/sndsh404/summer-2027-internships</t>
+          <t>https://github.com/Chieler/Summer-2027-SWE-Internships</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
+          <t>26 stars, pushed 2026-09-13; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -21578,32 +21606,32 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>discarded-low-priority</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>chicagotradingcampus</t>
+          <t>sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>greenhouse</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:chicagotradingcampus</t>
+          <t>repo:sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
+          <t>https://github.com/sndsh404/summer-2027-internships</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
+          <t>934 stars, pushed 2026-08-03; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -21625,7 +21653,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ctccampusboard</t>
+          <t>chicagotradingcampus</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -21635,17 +21663,17 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:ctccampusboard</t>
+          <t>greenhouse:chicagotradingcampus</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/chicagotradingcampus/jobs?content=true</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 8 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -21667,7 +21695,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>gardacp</t>
+          <t>ctccampusboard</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -21677,17 +21705,17 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>greenhouse:gardacp</t>
+          <t>greenhouse:ctccampusboard</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/ctccampusboard/jobs?content=true</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 6 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -21709,37 +21737,37 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>tgsmc</t>
+          <t>drwuniversityjobs</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>lever</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>lever:tgsmc</t>
+          <t>greenhouse:drwuniversityjobs</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/drwuniversityjobs/jobs?content=true</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 2 postings, 1 US student rows</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
     </row>
@@ -21751,27 +21779,27 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>vanshb03/Summer2027-Internships</t>
+          <t>gardacp</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>repo</t>
+          <t>greenhouse</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>repo:vanshb03/summer2027-internships</t>
+          <t>greenhouse:gardacp</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>https://github.com/vanshb03/Summer2027-Internships</t>
+          <t>https://boards-api.greenhouse.io/v1/boards/gardacp/jobs?content=true</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>9045 stars, pushed 2026-08-23; matched "Summer 2027 Internships"</t>
+          <t>linked from simplify-2027.tsv; not in sources.csv; API returns 14 postings, 4 US student rows</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -21788,84 +21816,84 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Allston Trading</t>
+          <t>tgsmc</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>lever</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>allston-trading</t>
+          <t>lever:tgsmc</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>https://allstontrading.com</t>
+          <t>https://api.lever.co/v0/postings/tgsmc?mode=json</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
+          <t>found in the HTML of tgs-join-our-team, which is watched as page_text; not in sources.csv; API returns 0 postings, 0 US student rows</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>rejected</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>AlphaGrep Securities</t>
+          <t>vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>firm</t>
+          <t>repo</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>alphagrep</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>alphagrepsecurities (greenhouse)</t>
+          <t>repo:vanshb03/summer2027-internships</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>https://github.com/vanshb03/Summer2027-Internships</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
+          <t>9045 stars, pushed 2026-08-23; matched "Summer 2027 Internships"</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -21877,7 +21905,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>AlphaSimplex</t>
+          <t>Allston Trading</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -21887,17 +21915,17 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>alphasimplex</t>
+          <t>allston-trading</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>https://www.alphasimplex.com/</t>
+          <t>https://allstontrading.com</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
+          <t>DNS resolves, ports 443 and 80 closed. Acquired by DV Trading Dec 2021; DV's board is already watched as dvtrading-greenhouse.</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -21919,7 +21947,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Arb Trading Group</t>
+          <t>AlphaGrep Securities</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -21929,17 +21957,17 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>arb-trading-group</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>https://arb-tg.com/</t>
+          <t>alphagrep</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>alphagrepsecurities (greenhouse)</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
+          <t>16 jobs including a 2027 Campus Program, but every location is India/China/Singapore - zero US rows now or historically.</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -21961,7 +21989,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Citadel (hedge fund)</t>
+          <t>AlphaSimplex</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -21971,17 +21999,17 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>citadel</t>
+          <t>alphasimplex</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>https://www.citadel.com/careers/students/</t>
+          <t>https://www.alphasimplex.com/</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
+          <t>Acquired by Virtus (closed Apr 2023). The Workday board that answers is all-Virtus sales/advisory, not quant.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -22003,7 +22031,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Consolidated Trading</t>
+          <t>Arb Trading Group</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -22013,17 +22041,17 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>consolidated-trading</t>
+          <t>arb-trading-group</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>http://consolidatedtrading.com/</t>
+          <t>https://arb-tg.com/</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
+          <t>4,775-char Webflow site, every careers path 404. arbtrading.com is a catch-all serving the same page for all 22 paths - a trap that would look healthy.</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -22045,7 +22073,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Cutler Group</t>
+          <t>Citadel (hedge fund)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -22055,17 +22083,17 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>cutler-group</t>
+          <t>citadel</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>https://cutlerllc.com/</t>
+          <t>https://www.citadel.com/careers/students/</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
+          <t>403 Cloudflare intermittently (1 of 3 fetches over 12 samples); homepage always 403. An intermittent block is worse than a hard one - it would fire spurious source failures. method=manual is correct.</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -22087,7 +22115,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Dark Forest Technologies</t>
+          <t>Consolidated Trading</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -22097,17 +22125,17 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>dark-forest-tech</t>
+          <t>consolidated-trading</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>https://darkforesttech.com/</t>
+          <t>http://consolidatedtrading.com/</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
+          <t>1,086 chars with no careers content, all careers paths 404, HTTPS handshake fails.</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -22129,7 +22157,7 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Eisler Capital</t>
+          <t>Cutler Group</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -22139,17 +22167,17 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>eisler-capital</t>
+          <t>cutler-group</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>https://eislercapital.com</t>
+          <t>https://cutlerllc.com/</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
+          <t>224 chars, under the floor; WP REST shows two pages total. NOTE cutlergroup.com is a Canadian bathroom-vanity manufacturer - wrong company.</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -22171,7 +22199,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Emergent Trading</t>
+          <t>Dark Forest Technologies</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -22181,17 +22209,17 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>emergent-trading</t>
+          <t>dark-forest-tech</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>https://www.emergenttrading.com/join</t>
+          <t>https://darkforesttech.com/</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
+          <t>231 chars, under the floor. A single GitHub Pages placeholder; recruiting@darkforesttech.com only.</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -22213,7 +22241,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Freestone Grove Partners</t>
+          <t>Eisler Capital</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -22223,17 +22251,17 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>freestone-grove</t>
+          <t>eisler-capital</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.gem.com/freestone-grove-partners</t>
+          <t>https://eislercapital.com</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
+          <t>DEFUNCT: no A record; www CNAMEs to a torn-down CloudFront distribution. Flagship wound down 31 Dec 2025.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -22255,7 +22283,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs Emerging Leaders Series</t>
+          <t>Emergent Trading</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -22265,17 +22293,17 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>goldman-emerging-leaders</t>
+          <t>emergent-trading</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
+          <t>https://www.emergenttrading.com/join</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
+          <t>Ember.js shell: /join is the real careers route and returns 0 chars. App and vendor bundles grepped, no ATS and no fetch target.</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -22297,7 +22325,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Kinetic Trading Partners</t>
+          <t>Freestone Grove Partners</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -22307,13 +22335,17 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>kinetic-trading-partners</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr"/>
+          <t>freestone-grove</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.gem.com/freestone-grove-partners</t>
+        </is>
+      </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
+          <t>Gem JS shell, 32 chars. Board verified real but empty: the GraphQL POST returns jobPostings: []. Worth re-probing later.</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -22335,7 +22367,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Laurion Capital</t>
+          <t>Goldman Sachs Emerging Leaders Series</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -22345,17 +22377,17 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>laurion-capital</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>laurioncapitalmanagement (greenhouse)</t>
+          <t>goldman-emerging-leaders</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.goldmansachs.com/careers/students/programs-and-internships/americas/emerging-leaders-series</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
+          <t>403 Akamai. higher.gs.com/roles returns 200 but 29 chars (JS shell). Programme is live for 2026 but only reachable at edition-specific Avature URLs that expire.</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -22377,7 +22409,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Nico Trading</t>
+          <t>Kinetic Trading Partners</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -22387,17 +22419,13 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>nico-trading</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>https://nicotrading.com</t>
-        </is>
-      </c>
+          <t>kinetic-trading-partners</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
+          <t>Zero LinkedIn results, absent from every quant directory checked. The name collides with Kinetic Partners Management LP, Kinetix Trading Solutions and retail prop-firm affiliate sites.</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -22419,7 +22447,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Numerai</t>
+          <t>Laurion Capital</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -22429,17 +22457,17 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>numerai</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>https://numer.ai/careers</t>
+          <t>laurion-capital</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>laurioncapitalmanagement (greenhouse)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
+          <t>Slug resolves but the board has 0 postings. A permanently empty board can only ever look healthy-and-quiet, so it is not added - same call as optiver/marshallwace in Phase 2.</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -22461,7 +22489,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Quantitative Investment Management</t>
+          <t>Nico Trading</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -22471,17 +22499,17 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>qim</t>
+          <t>nico-trading</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>https://quantitative.com/</t>
+          <t>https://nicotrading.com</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
+          <t>114-byte GoDaddy parking redirect, 0 chars. Firm operating but web-dark.</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -22503,7 +22531,7 @@
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Quantbox Research</t>
+          <t>Numerai</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -22513,17 +22541,17 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>quantbox-research</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>quantboxresearchpte (greenhouse)</t>
+          <t>numerai</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>https://numer.ai/careers</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
+          <t>404. No first-party careers page; Wellfound 403s us and Built In serves nav boilerplate with zero titles.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -22545,7 +22573,7 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Quantlab Financial</t>
+          <t>Quantitative Investment Management</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -22555,17 +22583,17 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>quantlab</t>
+          <t>qim</t>
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>https://www.quantlab.com/careers</t>
+          <t>https://quantitative.com/</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
+          <t>Every path 404 while robots.txt returns 200 - the site is genuinely unpublished, not blocking us. Firm is still an active RIA.</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -22587,7 +22615,7 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>QVR Advisors</t>
+          <t>Quantbox Research</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -22597,17 +22625,17 @@
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>qvr-advisors</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>https://qvradvisors.com</t>
+          <t>quantbox-research</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>quantboxresearchpte (greenhouse)</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
+          <t>7 jobs, junior roles are Amsterdam/Singapore only.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -22629,7 +22657,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Rosetta Analytics</t>
+          <t>Quantlab Financial</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -22639,17 +22667,17 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>rosetta-analytics</t>
+          <t>quantlab</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>https://rosetta-analytics.com/</t>
+          <t>https://www.quantlab.com/careers</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
+          <t>403 S3 AccessDenied, 26 chars. Its Jobvite board returns 200 with 237 chars (empty, under the 500 floor) and redirects back into the block.</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -22671,7 +22699,7 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Sensato Investors</t>
+          <t>QVR Advisors</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -22681,17 +22709,17 @@
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>sensato-investors</t>
+          <t>qvr-advisors</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>https://sensatoinvestors.com</t>
+          <t>https://qvradvisors.com</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
+          <t>DEFUNCT: homepage rewritten to past tense ('was formerly a boutique SEC-registered investment advisor'). Closing after ~30% losses Jan-Apr 2026.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -22713,7 +22741,7 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Spot Trading</t>
+          <t>Rosetta Analytics</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -22723,17 +22751,17 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>spot-trading</t>
+          <t>rosetta-analytics</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>https://spottradingllc.com</t>
+          <t>https://rosetta-analytics.com/</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
+          <t>DEFUNCT: 114 bytes, 0 chars, JS redirect to a parking lander. Closed March 2025.</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -22755,7 +22783,7 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Summerside Capital</t>
+          <t>Sensato Investors</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -22765,13 +22793,17 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>summerside-capital</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr"/>
+          <t>sensato-investors</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>https://sensatoinvestors.com</t>
+        </is>
+      </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
+          <t>HTTPS TLS internal error; over http, 27KB of HTML yields 44 chars. No careers link anywhere.</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -22793,7 +22825,7 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Tyler Capital</t>
+          <t>Spot Trading</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -22803,17 +22835,17 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>tyler-capital</t>
+          <t>spot-trading</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>https://www.tylercapital.co.uk/</t>
+          <t>https://spottradingllc.com</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+          <t>DEFUNCT: 'Coming Soon' placeholder, 40 chars. Firm closed 28 Feb 2018.</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -22835,7 +22867,7 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>WH Trading</t>
+          <t>Summerside Capital</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -22845,17 +22877,13 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>wh-trading</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>https://whtrading.com/life-at-wh-trading/</t>
-        </is>
-      </c>
+          <t>summerside-capital</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr"/>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+          <t>No A record on five domain variants. No trading firm of this name appears to exist.</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -22877,42 +22905,126 @@
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
+          <t>Tyler Capital</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>tyler-capital</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tylercapital.co.uk/</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>Watchable (2,093 chars) but states explicitly: 'we don't run an internship or graduate recruitment program'. UK-only. Not worth a row.</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>WH Trading</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>firm</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>wh-trading</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>https://whtrading.com/life-at-wh-trading/</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>Page is 2,320 chars but lists no roles; /careers and /jobs 404. Hiring via opportunities@whtrading.com only.</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
           <t>XR Trading</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>firm</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>xr-trading</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>https://www.xrtrading.com/</t>
         </is>
       </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
         <is>
           <t>Paylocity React shell: board returns 670 chars, all of it 'unsupported browser' boilerplate, zero titles. Bundle grepped - no JSON endpoint exists.</t>
         </is>
       </c>
-      <c r="G56" s="2" t="inlineStr">
+      <c r="G58" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="H58" s="2" t="inlineStr">
         <is>
           <t>2026-09-11</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H56"/>
+  <autoFilter ref="A1:H58"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
@@ -22943,8 +23055,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId34"/>
@@ -22953,17 +23065,19 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId52"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
state: 2026-09-29 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8042,12 +8042,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>4f009f794507f781652d228af6a53f321291f2e3ce5f378536471ea3d600b2e5</t>
+          <t>fae966e585e0cfc03b511c9b0ddbaf66b38bf2019562119a82de3bfac8f9696f</t>
         </is>
       </c>
     </row>
@@ -8110,12 +8110,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>25f3e22ab690e5dc0b3394bca1518de4dc0a25382e535bd2abdd744ff813ee90</t>
+          <t>035e6db5adfcc3203bbde0cad2342afeaadf660bc36c79c535e32e070f27e849</t>
         </is>
       </c>
     </row>
@@ -8178,7 +8178,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8242,7 +8242,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8578,7 +8578,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8646,7 +8646,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8914,7 +8914,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10678,7 +10678,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10926,7 +10926,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr"/>
@@ -10994,12 +10994,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>8d5be6c2e2d53d3c482b997109b4d440a4cb9f42b421c59e9660932a23a483b9</t>
+          <t>b41f6ade7438c1edf733e205a9a0f4779780ddebc887fa6f67305765f3fe7e66</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr"/>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11206,10 +11206,14 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
-        </is>
-      </c>
-      <c r="K196" s="2" t="inlineStr"/>
+          <t>2026-09-29T14:07:58+00:00</t>
+        </is>
+      </c>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29T14:07:58+00:00</t>
+        </is>
+      </c>
       <c r="L196" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11222,7 +11226,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>63485420a1d693d73c277ad75bc4354af21ef4b7c6986bae53385c03009f1e8a</t>
+          <t>de7b874fd5a83c4536690d1ad528cd9d62752306bbc232ae50be8766906fd725</t>
         </is>
       </c>
     </row>
@@ -11274,7 +11278,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr"/>
@@ -11342,7 +11346,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11410,7 +11414,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11478,7 +11482,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11546,7 +11550,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr"/>
@@ -11614,7 +11618,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11682,7 +11686,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11750,7 +11754,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr"/>
@@ -11818,7 +11822,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11886,7 +11890,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K206" s="2" t="inlineStr"/>
@@ -11950,12 +11954,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11970,7 +11974,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>8f5ce11e6e144e5fcab44fb1da76c9a2231fa37f5ec7c670d3e7d7ee137c39fc</t>
+          <t>8bbb4508176879484ace92088f23c8a074716a937a534c74d58986992a48a01d</t>
         </is>
       </c>
     </row>
@@ -12022,7 +12026,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12090,7 +12094,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12162,7 +12166,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12650,7 +12654,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -12688,7 +12692,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -12726,7 +12730,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -12764,7 +12768,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -12802,7 +12806,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -12840,7 +12844,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -12882,7 +12886,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -12924,7 +12928,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -12966,7 +12970,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -13008,7 +13012,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -13050,7 +13054,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -13092,7 +13096,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -13134,7 +13138,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -13176,7 +13180,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13218,7 +13222,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -13256,7 +13260,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -13298,7 +13302,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -13336,7 +13340,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -13378,7 +13382,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13420,7 +13424,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -13462,7 +13466,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -13504,7 +13508,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -13546,7 +13550,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -13584,7 +13588,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -13622,7 +13626,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -13660,7 +13664,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -13702,7 +13706,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -13744,7 +13748,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -13782,7 +13786,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -13820,7 +13824,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -13862,7 +13866,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -13900,7 +13904,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -13942,7 +13946,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -13980,7 +13984,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -14018,7 +14022,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -14056,7 +14060,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -14094,7 +14098,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -14132,7 +14136,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -14170,7 +14174,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -14212,7 +14216,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -14250,7 +14254,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -14292,7 +14296,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -14334,7 +14338,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -14376,7 +14380,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -14414,7 +14418,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -14452,7 +14456,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -14490,7 +14494,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -14532,7 +14536,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -14570,7 +14574,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -14612,7 +14616,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -14654,7 +14658,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -14692,7 +14696,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -14734,7 +14738,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -14776,7 +14780,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -14814,7 +14818,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -14856,7 +14860,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -14894,7 +14898,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -14936,7 +14940,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -14978,7 +14982,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -15020,7 +15024,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -15058,7 +15062,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -15096,7 +15100,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -15134,7 +15138,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -15172,7 +15176,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -15210,7 +15214,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -15252,7 +15256,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -15290,7 +15294,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -15332,7 +15336,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -15370,7 +15374,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -15412,7 +15416,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -15450,7 +15454,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -15488,7 +15492,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -15526,7 +15530,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -15720,7 +15724,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15762,12 +15766,12 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-09-26T12:17:03+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -15804,7 +15808,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15846,7 +15850,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15888,7 +15892,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15930,7 +15934,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15972,7 +15976,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16014,7 +16018,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16056,7 +16060,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16098,7 +16102,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -16140,7 +16144,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -16182,7 +16186,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -16224,7 +16228,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -16266,7 +16270,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -16308,7 +16312,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -16350,7 +16354,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -16392,7 +16396,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -16434,7 +16438,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -16476,7 +16480,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -16518,7 +16522,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -16560,7 +16564,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -16602,7 +16606,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -16640,7 +16644,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -16682,7 +16686,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -16724,7 +16728,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -16766,7 +16770,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -16808,7 +16812,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -16850,7 +16854,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -16892,7 +16896,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -16934,7 +16938,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -16976,7 +16980,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -17018,7 +17022,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -17060,7 +17064,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -17102,7 +17106,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -17144,7 +17148,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -17186,7 +17190,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -17233,7 +17237,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -17275,7 +17279,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -17312,7 +17316,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -17354,7 +17358,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -17396,7 +17400,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -17438,7 +17442,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -17480,7 +17484,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -17522,7 +17526,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -17564,7 +17568,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -17606,7 +17610,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -17648,7 +17652,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -17690,7 +17694,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -17732,7 +17736,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -17774,7 +17778,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -17816,7 +17820,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -17858,7 +17862,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -17900,7 +17904,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -17942,7 +17946,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -17984,7 +17988,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -18026,7 +18030,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -18068,7 +18072,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -18110,7 +18114,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -18152,7 +18156,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -18194,7 +18198,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -18236,7 +18240,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -18278,7 +18282,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -18320,7 +18324,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -18362,7 +18366,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -18404,7 +18408,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -18446,7 +18450,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -18488,7 +18492,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -18530,7 +18534,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -18572,7 +18576,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -18614,7 +18618,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -18656,7 +18660,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -18698,7 +18702,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -18741,7 +18745,7 @@
       <c r="F151" s="2" t="inlineStr"/>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -18778,7 +18782,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -18820,7 +18824,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -18862,7 +18866,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -18904,7 +18908,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -18946,7 +18950,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -18988,7 +18992,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -19030,7 +19034,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -19072,7 +19076,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -19114,7 +19118,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -19156,7 +19160,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -19198,7 +19202,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -19240,7 +19244,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -19282,7 +19286,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -19324,7 +19328,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -19366,7 +19370,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -19408,7 +19412,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -19455,7 +19459,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -19492,7 +19496,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -19534,7 +19538,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -19576,7 +19580,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -19618,7 +19622,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -19656,7 +19660,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -19698,7 +19702,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -19736,7 +19740,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -19778,7 +19782,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -19820,7 +19824,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -19858,7 +19862,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -19896,7 +19900,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -19934,7 +19938,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -19972,7 +19976,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -20010,7 +20014,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -20048,7 +20052,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -20086,7 +20090,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -20124,7 +20128,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -20166,7 +20170,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -20208,7 +20212,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -20246,7 +20250,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -20284,7 +20288,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -20322,7 +20326,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -20360,7 +20364,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -20398,7 +20402,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-29T14:07:58+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-09-30 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8042,12 +8042,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>fae966e585e0cfc03b511c9b0ddbaf66b38bf2019562119a82de3bfac8f9696f</t>
+          <t>c4938f052d21ad86e6e914c6617f9c9eac4c172b49af8d73ba56e155189542e2</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8110,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8242,7 +8242,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8578,7 +8578,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8646,7 +8646,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8914,7 +8914,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10678,7 +10678,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10926,7 +10926,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr"/>
@@ -10994,12 +10994,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11014,7 +11014,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>b41f6ade7438c1edf733e205a9a0f4779780ddebc887fa6f67305765f3fe7e66</t>
+          <t>c9179eee7c2097bc14698f27863e7d34f3348e1d94ec0795ff47e3d5ab436e77</t>
         </is>
       </c>
     </row>
@@ -11066,7 +11066,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr"/>
@@ -11134,12 +11134,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11154,7 +11154,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>4a082bd8ae515f500fdf636e7d9d1b17188a776a9936aee26a03d7a531030ddc</t>
+          <t>f167aa848901d0363e8144b4e47d45f95149d16f975ec408ea04835e0c642ed9</t>
         </is>
       </c>
     </row>
@@ -11206,7 +11206,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11278,7 +11278,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr"/>
@@ -11346,7 +11346,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11414,7 +11414,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11482,7 +11482,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr"/>
@@ -11618,7 +11618,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11686,7 +11686,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11754,10 +11754,14 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
-        </is>
-      </c>
-      <c r="K204" s="2" t="inlineStr"/>
+          <t>2026-09-30T13:45:29+00:00</t>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30T13:45:29+00:00</t>
+        </is>
+      </c>
       <c r="L204" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11770,7 +11774,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>5cfd18060b4b9d51508a27ad7ae69e86d8234409eae29b9687f6ad71ac3ac4dc</t>
+          <t>d577854726860cefa8b7bc5191fbef689f636ecf12b7ec70b4be78748becacf0</t>
         </is>
       </c>
     </row>
@@ -11822,7 +11826,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11890,7 +11894,7 @@
       </c>
       <c r="J206" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K206" s="2" t="inlineStr"/>
@@ -11954,12 +11958,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11974,7 +11978,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>8bbb4508176879484ace92088f23c8a074716a937a534c74d58986992a48a01d</t>
+          <t>16fc244bf83875312381ece0dcc56b27d08a673a002c038732648cd73fc6a36d</t>
         </is>
       </c>
     </row>
@@ -12026,7 +12030,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12094,12 +12098,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12114,7 +12118,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12166,7 +12170,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12654,7 +12658,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -12692,7 +12696,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -12730,7 +12734,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -12768,7 +12772,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -12806,7 +12810,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -12844,7 +12848,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -12886,7 +12890,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -12928,7 +12932,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -12970,7 +12974,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -13012,7 +13016,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -13054,7 +13058,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -13096,7 +13100,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -13138,7 +13142,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -13180,7 +13184,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -13222,7 +13226,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -13260,7 +13264,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -13302,7 +13306,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -13340,7 +13344,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -13382,7 +13386,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -13424,7 +13428,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -13466,7 +13470,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -13508,7 +13512,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -13550,7 +13554,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -13588,7 +13592,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -13626,7 +13630,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -13664,7 +13668,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -13706,7 +13710,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -13748,7 +13752,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -13786,7 +13790,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -13824,7 +13828,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -13866,7 +13870,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -13904,7 +13908,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -13946,7 +13950,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -13984,7 +13988,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -14022,7 +14026,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -14060,7 +14064,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -14098,7 +14102,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -14136,7 +14140,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -14174,7 +14178,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -14216,7 +14220,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -14254,7 +14258,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -14296,7 +14300,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -14338,7 +14342,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -14380,7 +14384,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -14418,7 +14422,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -14456,7 +14460,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -14494,7 +14498,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -14536,7 +14540,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -14574,7 +14578,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -14616,7 +14620,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -14658,7 +14662,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -14696,7 +14700,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -14738,7 +14742,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -14780,7 +14784,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -14818,7 +14822,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -14860,7 +14864,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -14898,7 +14902,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -14940,7 +14944,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -14982,7 +14986,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -15024,7 +15028,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -15062,7 +15066,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -15100,7 +15104,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -15138,7 +15142,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -15176,7 +15180,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -15214,7 +15218,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -15256,7 +15260,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -15294,7 +15298,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -15336,7 +15340,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -15374,7 +15378,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -15416,7 +15420,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -15454,7 +15458,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -15492,7 +15496,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -15530,7 +15534,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -15724,7 +15728,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15771,7 +15775,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -15808,7 +15812,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -15850,7 +15854,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -15892,7 +15896,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -15934,7 +15938,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -15976,7 +15980,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -16018,7 +16022,7 @@
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
@@ -16060,7 +16064,7 @@
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
@@ -16102,7 +16106,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -16144,7 +16148,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -16186,7 +16190,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -16228,7 +16232,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -16270,7 +16274,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -16312,7 +16316,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -16354,7 +16358,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -16396,7 +16400,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -16438,7 +16442,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -16480,7 +16484,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -16522,7 +16526,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -16564,7 +16568,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -16606,7 +16610,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -16644,7 +16648,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -16686,7 +16690,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -16728,7 +16732,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -16770,7 +16774,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -16812,7 +16816,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -16854,7 +16858,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -16896,7 +16900,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -16938,7 +16942,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -16980,7 +16984,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -17022,7 +17026,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -17064,7 +17068,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -17106,7 +17110,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -17148,7 +17152,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -17190,7 +17194,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -17316,7 +17320,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -17358,7 +17362,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -17400,7 +17404,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -17442,7 +17446,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -17484,7 +17488,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -17526,7 +17530,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -17568,7 +17572,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -17610,7 +17614,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -17652,7 +17656,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -17694,7 +17698,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -17736,7 +17740,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -17778,7 +17782,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -17820,7 +17824,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -17862,7 +17866,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -17904,7 +17908,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -17951,7 +17955,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -17988,7 +17992,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -18030,7 +18034,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -18072,7 +18076,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -18114,7 +18118,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -18156,7 +18160,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -18198,7 +18202,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -18240,7 +18244,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -18282,7 +18286,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -18324,7 +18328,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -18366,7 +18370,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -18408,7 +18412,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -18450,7 +18454,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -18492,7 +18496,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -18534,7 +18538,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -18576,7 +18580,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -18618,7 +18622,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -18660,7 +18664,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -18702,7 +18706,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -18745,7 +18749,7 @@
       <c r="F151" s="2" t="inlineStr"/>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -18782,7 +18786,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -18824,7 +18828,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -18866,7 +18870,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -18908,7 +18912,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -18950,7 +18954,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -18992,7 +18996,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -19034,7 +19038,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -19076,7 +19080,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -19118,7 +19122,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -19160,7 +19164,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -19202,7 +19206,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -19244,7 +19248,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -19286,7 +19290,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -19328,7 +19332,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -19370,7 +19374,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -19412,7 +19416,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -19459,7 +19463,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -19496,7 +19500,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -19538,7 +19542,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -19580,7 +19584,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -19622,7 +19626,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -19660,7 +19664,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -19702,7 +19706,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -19740,7 +19744,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -19782,7 +19786,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -19824,7 +19828,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -19862,7 +19866,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -19900,7 +19904,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -19938,7 +19942,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -19976,7 +19980,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -20014,7 +20018,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -20052,7 +20056,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -20090,7 +20094,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -20128,7 +20132,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -20170,7 +20174,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -20212,7 +20216,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -20250,7 +20254,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -20288,7 +20292,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -20326,7 +20330,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -20364,7 +20368,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -20402,7 +20406,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-09-30T13:45:29+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-02 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
@@ -4362,7 +4362,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4594,7 +4594,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5118,7 +5118,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6502,7 +6502,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6738,7 +6738,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7978,7 +7978,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8042,12 +8042,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8058,7 +8058,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>dff0c7c0bbb6f4bf7c8fdbf6b1baec94132426f3c46eb1437a0339d88156aa84</t>
+          <t>12204ca88ff760dc59ca7d91f157bfcee0414ad3fd70413f3816f5a3f638814d</t>
         </is>
       </c>
     </row>
@@ -8110,12 +8110,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:07:58+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8126,7 +8126,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>035e6db5adfcc3203bbde0cad2342afeaadf660bc36c79c535e32e070f27e849</t>
+          <t>d1f24ab708bf4d606c9a7bbb1f931306acec8cb0b789fa38d0e7a7aa720e39c9</t>
         </is>
       </c>
     </row>
@@ -8178,7 +8178,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8242,7 +8242,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8578,7 +8578,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8646,7 +8646,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8718,7 +8718,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8914,7 +8914,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8986,7 +8986,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10678,7 +10678,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10858,7 +10858,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10926,10 +10926,14 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
-        </is>
-      </c>
-      <c r="K192" s="2" t="inlineStr"/>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="L192" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -10942,7 +10946,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>b47c36bb2ee2b26c77ec5e4475bc254d384f2555a03745a7b8debadef1201c13</t>
+          <t>5849cd1f0a1d2fe399642c5beec06f20d5e3f29b3f5e385731ecd95949e16c1b</t>
         </is>
       </c>
     </row>
@@ -10994,12 +10998,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11014,7 +11018,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>a974a17d2768e967bc41e922d91e23b318492f84bf6273effbde03bbaaf48d3e</t>
+          <t>2fc3dafc5a8417b44d45d208d520e5ab44cfe453d9effdc3ae173276bdf0df24</t>
         </is>
       </c>
     </row>
@@ -11066,10 +11070,14 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
-        </is>
-      </c>
-      <c r="K194" s="2" t="inlineStr"/>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="L194" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11082,7 +11090,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>b7114977696626f0648f0bbef9b71726ec25d14bd0cd081d842b252261f21c13</t>
+          <t>f00adf1650b8a3f3d78c292b33ab4795d2ec0a3bd00b337b6c0aba02b968746a</t>
         </is>
       </c>
     </row>
@@ -11134,12 +11142,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11154,7 +11162,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>6db7b80e8640b187ecfce9c50aa930edd04e5695bd4a4ab53780a427c16b05c1</t>
+          <t>382f0ff884f2d69d57f4142c29df168e91f7f8e9281a13931c4f7bddd01b2397</t>
         </is>
       </c>
     </row>
@@ -11206,7 +11214,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11278,7 +11286,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11350,7 +11358,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11418,7 +11426,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11486,7 +11494,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11554,12 +11562,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11574,7 +11582,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>7b79376c8769e78af04e0c3c89748d9a9d87b534b2be7a1efac768df40fbb1b2</t>
+          <t>a03e1de236c1d2d887b92cce731219d887ebfa90a794e0d18449db8cc530766c</t>
         </is>
       </c>
     </row>
@@ -11626,7 +11634,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11694,7 +11702,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11762,7 +11770,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11834,7 +11842,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11966,12 +11974,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11986,7 +11994,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>8f5ce11e6e144e5fcab44fb1da76c9a2231fa37f5ec7c670d3e7d7ee137c39fc</t>
+          <t>5aceabd06c3fe1967cc589d3922433a13239ee6b23b36cd705d29c7943beae66</t>
         </is>
       </c>
     </row>
@@ -12038,7 +12046,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12106,12 +12114,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T13:45:29+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12126,7 +12134,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12186,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12474,7 +12482,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12722,7 +12730,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12790,7 +12798,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12858,7 +12866,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr"/>
@@ -17532,7 +17540,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J304" s="2" t="inlineStr"/>
+      <c r="J304" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K304" s="2" t="inlineStr"/>
       <c r="L304" s="2" t="inlineStr">
         <is>
@@ -17544,7 +17556,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N304" s="2" t="inlineStr"/>
+      <c r="N304" s="2" t="inlineStr">
+        <is>
+          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="2" t="inlineStr">
@@ -17592,7 +17608,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J305" s="2" t="inlineStr"/>
+      <c r="J305" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K305" s="2" t="inlineStr"/>
       <c r="L305" s="2" t="inlineStr">
         <is>
@@ -17652,7 +17672,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J306" s="2" t="inlineStr"/>
+      <c r="J306" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K306" s="2" t="inlineStr"/>
       <c r="L306" s="2" t="inlineStr">
         <is>
@@ -17664,7 +17688,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N306" s="2" t="inlineStr"/>
+      <c r="N306" s="2" t="inlineStr">
+        <is>
+          <t>c96cbecf17320ed640804a102893b8853b7ccd7d27a0445c6629132a813161fe</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -17712,7 +17740,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J307" s="2" t="inlineStr"/>
+      <c r="J307" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K307" s="2" t="inlineStr"/>
       <c r="L307" s="2" t="inlineStr">
         <is>
@@ -17724,7 +17756,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N307" s="2" t="inlineStr"/>
+      <c r="N307" s="2" t="inlineStr">
+        <is>
+          <t>e61d095bc724d0bffcfa9af426fb3ca60cfbc77fe20384dac0032427b660a6a2</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" s="2" t="inlineStr">
@@ -17772,7 +17808,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J308" s="2" t="inlineStr"/>
+      <c r="J308" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K308" s="2" t="inlineStr"/>
       <c r="L308" s="2" t="inlineStr">
         <is>
@@ -17784,7 +17824,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N308" s="2" t="inlineStr"/>
+      <c r="N308" s="2" t="inlineStr">
+        <is>
+          <t>e6a8b62feae47671a9eace8e68f600fefd7d691d28f3c37a339ef0ed04e5d36d</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="2" t="inlineStr">
@@ -17832,7 +17876,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J309" s="2" t="inlineStr"/>
+      <c r="J309" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K309" s="2" t="inlineStr"/>
       <c r="L309" s="2" t="inlineStr">
         <is>
@@ -17844,7 +17892,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N309" s="2" t="inlineStr"/>
+      <c r="N309" s="2" t="inlineStr">
+        <is>
+          <t>860097cc82f28741a94b12fe159db53cca93f0811188483f5608452c37cad3d2</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -17948,7 +18000,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J311" s="2" t="inlineStr"/>
+      <c r="J311" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K311" s="2" t="inlineStr"/>
       <c r="L311" s="2" t="inlineStr">
         <is>
@@ -17960,7 +18016,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N311" s="2" t="inlineStr"/>
+      <c r="N311" s="2" t="inlineStr">
+        <is>
+          <t>2cc4387e1d0ba1ba0bcffa6325bd94482d49d376063b49394fb833f1d6c8d974</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="2" t="inlineStr">
@@ -18008,7 +18068,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J312" s="2" t="inlineStr"/>
+      <c r="J312" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K312" s="2" t="inlineStr"/>
       <c r="L312" s="2" t="inlineStr">
         <is>
@@ -18236,7 +18300,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J316" s="2" t="inlineStr"/>
+      <c r="J316" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K316" s="2" t="inlineStr"/>
       <c r="L316" s="2" t="inlineStr">
         <is>
@@ -18296,7 +18364,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J317" s="2" t="inlineStr"/>
+      <c r="J317" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K317" s="2" t="inlineStr"/>
       <c r="L317" s="2" t="inlineStr">
         <is>
@@ -18356,7 +18428,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J318" s="2" t="inlineStr"/>
+      <c r="J318" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K318" s="2" t="inlineStr"/>
       <c r="L318" s="2" t="inlineStr">
         <is>
@@ -18368,7 +18444,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N318" s="2" t="inlineStr"/>
+      <c r="N318" s="2" t="inlineStr">
+        <is>
+          <t>2e93fb5b9a7551a7ee64edea2c118684e0785c754ece9d96bf585b04dfe59d8f</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -18416,7 +18496,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J319" s="2" t="inlineStr"/>
+      <c r="J319" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K319" s="2" t="inlineStr"/>
       <c r="L319" s="2" t="inlineStr">
         <is>
@@ -18428,7 +18512,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N319" s="2" t="inlineStr"/>
+      <c r="N319" s="2" t="inlineStr">
+        <is>
+          <t>f156c5a1eb2a730f052e5bdde879df206b4d79cf988c70df5cb096ad4063a1ad</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -18476,7 +18564,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J320" s="2" t="inlineStr"/>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K320" s="2" t="inlineStr"/>
       <c r="L320" s="2" t="inlineStr">
         <is>
@@ -18488,7 +18580,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N320" s="2" t="inlineStr"/>
+      <c r="N320" s="2" t="inlineStr">
+        <is>
+          <t>91f69cbea24426b1ebf3ce81ea78eb3ae94fda3cc7036100c76a86d44f547f64</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="2" t="inlineStr">
@@ -18536,7 +18632,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J321" s="2" t="inlineStr"/>
+      <c r="J321" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K321" s="2" t="inlineStr"/>
       <c r="L321" s="2" t="inlineStr">
         <is>
@@ -18548,7 +18648,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N321" s="2" t="inlineStr"/>
+      <c r="N321" s="2" t="inlineStr">
+        <is>
+          <t>b0af1d82d20b10ed08964884480dbe54861f8f4c7c2970d35bedda6ddd6c0e94</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="2" t="inlineStr">
@@ -18596,7 +18700,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J322" s="2" t="inlineStr"/>
+      <c r="J322" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K322" s="2" t="inlineStr"/>
       <c r="L322" s="2" t="inlineStr">
         <is>
@@ -18608,7 +18716,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N322" s="2" t="inlineStr"/>
+      <c r="N322" s="2" t="inlineStr">
+        <is>
+          <t>48648157d6c78f32ee9973b2361efae253aacc860035a45ea5084b71937f0ff7</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="2" t="inlineStr">
@@ -18656,7 +18768,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J323" s="2" t="inlineStr"/>
+      <c r="J323" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="K323" s="2" t="inlineStr"/>
       <c r="L323" s="2" t="inlineStr">
         <is>
@@ -18668,7 +18784,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N323" s="2" t="inlineStr"/>
+      <c r="N323" s="2" t="inlineStr">
+        <is>
+          <t>0d6c21704f64a7b47ca16027c2ef4ac10712fbb03c884d3acf995836e5285533</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N323"/>
@@ -19080,7 +19200,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19118,7 +19238,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19160,7 +19280,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19198,7 +19318,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19236,7 +19356,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19274,7 +19394,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19312,7 +19432,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19352,7 +19472,11 @@
           <t>ashby.txt</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -19388,7 +19512,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19428,7 +19552,11 @@
           <t>aprameyak/2027-tech-jobs</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -19466,7 +19594,11 @@
           <t>dreamworkhq/Open-Tech-Internships-2027</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -19506,7 +19638,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19546,7 +19678,11 @@
           <t>mehek-builds/Summer2027-Internships</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -19586,7 +19722,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19628,7 +19764,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19670,7 +19806,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19712,7 +19848,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19754,7 +19890,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19796,7 +19932,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -19838,7 +19974,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -19880,7 +20016,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -19922,7 +20058,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -19960,7 +20096,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20002,7 +20138,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20040,7 +20176,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20082,7 +20218,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20124,7 +20260,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20166,7 +20302,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20208,7 +20344,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20250,7 +20386,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20288,7 +20424,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20326,7 +20462,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20364,7 +20500,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20406,7 +20542,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20448,7 +20584,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20486,7 +20622,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20524,7 +20660,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20566,7 +20702,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20604,7 +20740,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20646,7 +20782,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20684,7 +20820,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20722,7 +20858,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20764,7 +20900,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20802,7 +20938,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -20840,7 +20976,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -20878,7 +21014,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -20920,7 +21056,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -20958,7 +21094,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21000,7 +21136,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21042,7 +21178,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21084,7 +21220,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21126,7 +21262,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21164,7 +21300,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21202,7 +21338,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21240,7 +21376,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21282,7 +21418,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21320,7 +21456,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21362,7 +21498,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21404,7 +21540,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21442,7 +21578,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21484,7 +21620,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21526,7 +21662,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21564,7 +21700,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21606,7 +21742,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21644,7 +21780,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21686,7 +21822,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21728,7 +21864,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21770,7 +21906,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21808,7 +21944,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -21846,7 +21982,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -21884,7 +22020,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -21922,7 +22058,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -21960,7 +22096,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22002,7 +22138,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22040,7 +22176,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22082,7 +22218,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22120,7 +22256,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22162,7 +22298,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22200,7 +22336,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22240,7 +22376,11 @@
           <t>greenhouse.txt</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -22276,7 +22416,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22314,7 +22454,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22354,7 +22494,11 @@
           <t>lever.txt</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -22582,7 +22726,11 @@
           <t>REU Site</t>
         </is>
       </c>
-      <c r="F90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -22622,7 +22770,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22664,7 +22812,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22704,7 +22852,11 @@
           <t>https://allenai.org/internships</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -22744,7 +22896,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22786,7 +22938,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -22828,7 +22980,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -22871,7 +23023,7 @@
       <c r="F97" s="2" t="inlineStr"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -22908,7 +23060,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -22950,7 +23102,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -22992,7 +23144,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -23034,7 +23186,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23076,7 +23228,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23118,7 +23270,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23160,7 +23312,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23200,7 +23352,11 @@
           <t>https://builtin.com/jobs/data-analytics/internship</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr"/>
+      <c r="F105" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23238,7 +23394,11 @@
           <t>https://builtin.com/jobs/dev-engineering/internship</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr"/>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23276,7 +23436,11 @@
           <t>https://builtin.com/jobs/finance/internship</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr"/>
+      <c r="F107" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23317,7 +23481,7 @@
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -23354,7 +23518,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23396,7 +23560,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23438,7 +23602,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23480,7 +23644,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23520,7 +23684,11 @@
           <t>https://riss.ri.cmu.edu/</t>
         </is>
       </c>
-      <c r="F113" s="2" t="inlineStr"/>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23560,7 +23728,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23602,7 +23770,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23644,7 +23812,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23686,7 +23854,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23728,7 +23896,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23770,7 +23938,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -23812,7 +23980,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -23854,7 +24022,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -23896,7 +24064,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -23938,7 +24106,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -23980,7 +24148,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24018,7 +24186,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24060,7 +24228,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24102,7 +24270,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24144,7 +24312,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24186,7 +24354,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24228,7 +24396,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24270,7 +24438,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24312,7 +24480,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24354,7 +24522,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24396,7 +24564,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24438,7 +24606,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24480,7 +24648,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24522,7 +24690,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24564,7 +24732,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -24606,7 +24774,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24648,7 +24816,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24690,7 +24858,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24732,7 +24900,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24772,7 +24940,11 @@
           <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24812,7 +24984,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -24854,7 +25026,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -24896,7 +25068,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -24938,7 +25110,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -24980,7 +25152,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25022,7 +25194,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25062,7 +25234,11 @@
           <t>https://www.jhuapl.edu/careers/internships</t>
         </is>
       </c>
-      <c r="F150" s="2" t="inlineStr"/>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25102,7 +25278,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25144,7 +25320,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25186,7 +25362,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25229,7 +25405,7 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -25266,7 +25442,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25306,7 +25482,11 @@
           <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
         </is>
       </c>
-      <c r="F156" s="2" t="inlineStr"/>
+      <c r="F156" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25346,7 +25526,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25388,7 +25568,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25430,7 +25610,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25472,7 +25652,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25514,7 +25694,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25556,7 +25736,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25596,7 +25776,11 @@
           <t>https://www.ll.mit.edu/careers/student-opportunities</t>
         </is>
       </c>
-      <c r="F163" s="2" t="inlineStr"/>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G163" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25636,7 +25820,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25678,7 +25862,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25718,7 +25902,11 @@
           <t>https://www.intelligencecareers.gov/nsa/students</t>
         </is>
       </c>
-      <c r="F166" s="2" t="inlineStr"/>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25758,7 +25946,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -25800,7 +25988,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -25842,7 +26030,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -25884,7 +26072,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -25924,7 +26112,11 @@
           <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
         </is>
       </c>
-      <c r="F171" s="2" t="inlineStr"/>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25964,7 +26156,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26006,7 +26198,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26048,7 +26240,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26088,7 +26280,11 @@
           <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
         </is>
       </c>
-      <c r="F175" s="2" t="inlineStr"/>
+      <c r="F175" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T14:00:53+00:00</t>
+        </is>
+      </c>
       <c r="G175" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26128,7 +26324,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26170,7 +26366,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26212,7 +26408,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26254,7 +26450,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26296,7 +26492,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26338,7 +26534,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26380,7 +26576,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26422,7 +26618,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26464,7 +26660,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26506,7 +26702,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26548,7 +26744,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26590,7 +26786,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26632,7 +26828,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26674,7 +26870,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26717,7 +26913,7 @@
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -26754,7 +26950,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -26796,7 +26992,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -26838,7 +27034,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -26880,7 +27076,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -26922,7 +27118,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -26964,7 +27160,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27006,7 +27202,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27048,7 +27244,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27090,7 +27286,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27128,7 +27324,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27170,7 +27366,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27208,7 +27404,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27250,7 +27446,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27292,7 +27488,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27330,7 +27526,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27368,7 +27564,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27406,7 +27602,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27444,7 +27640,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27482,7 +27678,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27520,7 +27716,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27558,7 +27754,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27596,7 +27792,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27638,7 +27834,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27680,7 +27876,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27718,7 +27914,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27756,7 +27952,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -27794,7 +27990,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -27832,7 +28028,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -27870,7 +28066,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-02T14:00:53+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-03 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,10 +4298,14 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L72" s="2" t="inlineStr"/>
       <c r="M72" s="2" t="inlineStr">
         <is>
@@ -4310,7 +4314,7 @@
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>02fb00b81b8ab70a6cc77d2496306f2cb4098cd9700b2b7d8b3f6a2b5d0776ef</t>
+          <t>72fa80328b9c4686227f4a986a19832ecf252d194f978f745948259f94b79a35</t>
         </is>
       </c>
     </row>
@@ -4362,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4426,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4594,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5118,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6502,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6674,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6738,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7978,7 +7982,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8042,12 +8046,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8058,7 +8062,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>12204ca88ff760dc59ca7d91f157bfcee0414ad3fd70413f3816f5a3f638814d</t>
+          <t>f2db90db914c14635ea9f1f6c7bd7e5fc5a9739b8b7b35d8467c1d56f4f7cacc</t>
         </is>
       </c>
     </row>
@@ -8110,12 +8114,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8126,7 +8130,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>d1f24ab708bf4d606c9a7bbb1f931306acec8cb0b789fa38d0e7a7aa720e39c9</t>
+          <t>ace0bff5405602c2b4b34ff8bceb6a79377e683019e0f40f66dc5d2381e7c3dc</t>
         </is>
       </c>
     </row>
@@ -8178,7 +8182,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8242,7 +8246,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8578,7 +8582,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8646,7 +8650,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8718,7 +8722,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8846,7 +8850,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8914,7 +8918,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8986,7 +8990,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10678,7 +10682,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10858,7 +10862,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10926,7 +10930,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -10998,12 +11002,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11018,7 +11022,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>2fc3dafc5a8417b44d45d208d520e5ab44cfe453d9effdc3ae173276bdf0df24</t>
+          <t>1e627458f1a0b6608587445d37ecb2b997a405962bf4695b100df799058ea10d</t>
         </is>
       </c>
     </row>
@@ -11070,7 +11074,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11142,12 +11146,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11162,7 +11166,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>382f0ff884f2d69d57f4142c29df168e91f7f8e9281a13931c4f7bddd01b2397</t>
+          <t>a8b980148d1fcb9de0056775159c842e4819f3d418f9f9769dcc51de408ba5e1</t>
         </is>
       </c>
     </row>
@@ -11214,7 +11218,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11286,7 +11290,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11358,7 +11362,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11426,7 +11430,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11494,7 +11498,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11562,7 +11566,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11634,7 +11638,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11702,7 +11706,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11765,17 +11769,17 @@
       </c>
       <c r="I204" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T13:45:29+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -11790,7 +11794,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>d577854726860cefa8b7bc5191fbef689f636ecf12b7ec70b4be78748becacf0</t>
+          <t>fe075697d40a7f9db49816d88ebd93f9cfab60e0a572e64769ad7d5aed73a088</t>
         </is>
       </c>
     </row>
@@ -11842,7 +11846,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11974,12 +11978,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11994,7 +11998,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>5aceabd06c3fe1967cc589d3922433a13239ee6b23b36cd705d29c7943beae66</t>
+          <t>833809f7222e45a7cbd4ee2ea73bd90b0716d7e2bef03208131645768aa07489</t>
         </is>
       </c>
     </row>
@@ -12046,7 +12050,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12114,12 +12118,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12134,7 +12138,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12186,7 +12190,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12482,7 +12486,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12730,7 +12734,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12798,7 +12802,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12866,10 +12870,14 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K221" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L221" s="2" t="inlineStr">
         <is>
           <t>2026-09-30</t>
@@ -12882,7 +12890,7 @@
       </c>
       <c r="N221" s="2" t="inlineStr">
         <is>
-          <t>0e1b61c71a2c613c885acb030ea3435ed5b078d1b40039db57dc9627161f90d5</t>
+          <t>90a85363c454b0894939ab271ef928998ece74001cf74e1c6ccfa44ff72cfc6c</t>
         </is>
       </c>
     </row>
@@ -17542,10 +17550,14 @@
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K304" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K304" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L304" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -17558,7 +17570,7 @@
       </c>
       <c r="N304" s="2" t="inlineStr">
         <is>
-          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
+          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
         </is>
       </c>
     </row>
@@ -17610,7 +17622,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr"/>
@@ -17674,7 +17686,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr"/>
@@ -17742,7 +17754,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr"/>
@@ -17810,7 +17822,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr"/>
@@ -17878,7 +17890,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr"/>
@@ -18002,7 +18014,7 @@
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr"/>
@@ -18070,7 +18082,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr"/>
@@ -18302,7 +18314,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18366,7 +18378,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18430,7 +18442,7 @@
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K318" s="2" t="inlineStr"/>
@@ -18498,7 +18510,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18566,7 +18578,7 @@
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="K320" s="2" t="inlineStr"/>
@@ -18634,10 +18646,14 @@
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K321" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K321" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L321" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18650,7 +18666,7 @@
       </c>
       <c r="N321" s="2" t="inlineStr">
         <is>
-          <t>b0af1d82d20b10ed08964884480dbe54861f8f4c7c2970d35bedda6ddd6c0e94</t>
+          <t>933101db3dfa9c9b136935ae5c0369e51954e0b6e8d17128fa07bab9c5a416d0</t>
         </is>
       </c>
     </row>
@@ -18702,10 +18718,14 @@
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K322" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K322" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L322" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18718,7 +18738,7 @@
       </c>
       <c r="N322" s="2" t="inlineStr">
         <is>
-          <t>48648157d6c78f32ee9973b2361efae253aacc860035a45ea5084b71937f0ff7</t>
+          <t>165c478a2b03fbbf3ab802883170010c6578aa773b45f59d6bb62db5c54c89c1</t>
         </is>
       </c>
     </row>
@@ -18770,10 +18790,14 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
-        </is>
-      </c>
-      <c r="K323" s="2" t="inlineStr"/>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
+      <c r="K323" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:42:39+00:00</t>
+        </is>
+      </c>
       <c r="L323" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18786,7 +18810,7 @@
       </c>
       <c r="N323" s="2" t="inlineStr">
         <is>
-          <t>0d6c21704f64a7b47ca16027c2ef4ac10712fbb03c884d3acf995836e5285533</t>
+          <t>ba86226392bfc98df6eeb51f0fe16527f412b502525455c7c54564a43e870d90</t>
         </is>
       </c>
     </row>
@@ -19200,7 +19224,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19238,7 +19262,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19280,7 +19304,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19318,7 +19342,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19356,7 +19380,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19394,7 +19418,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19432,7 +19456,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19474,7 +19498,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19512,7 +19536,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19554,7 +19578,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -19596,7 +19620,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -19638,7 +19662,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19680,7 +19704,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -19722,7 +19746,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19764,7 +19788,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19806,7 +19830,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19848,7 +19872,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19890,7 +19914,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19932,7 +19956,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -19974,7 +19998,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -20016,7 +20040,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -20058,7 +20082,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -20096,7 +20120,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20138,7 +20162,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20176,7 +20200,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20218,7 +20242,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20260,7 +20284,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20302,7 +20326,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20344,7 +20368,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20386,7 +20410,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20424,7 +20448,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20462,7 +20486,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20500,7 +20524,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20542,7 +20566,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20584,7 +20608,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20622,7 +20646,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20660,7 +20684,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20702,7 +20726,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20740,7 +20764,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20782,7 +20806,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20820,7 +20844,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20858,7 +20882,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20900,7 +20924,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20938,7 +20962,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -20976,7 +21000,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -21014,7 +21038,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -21056,7 +21080,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -21094,7 +21118,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21136,7 +21160,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21178,7 +21202,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21220,7 +21244,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21262,7 +21286,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21300,7 +21324,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21338,7 +21362,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21376,7 +21400,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21418,7 +21442,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21456,7 +21480,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21498,7 +21522,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21540,7 +21564,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21578,7 +21602,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21620,7 +21644,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21662,7 +21686,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21700,7 +21724,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21742,7 +21766,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21780,7 +21804,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21822,7 +21846,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21864,7 +21888,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21906,7 +21930,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21944,7 +21968,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -21982,7 +22006,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -22020,7 +22044,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -22058,7 +22082,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -22096,7 +22120,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22138,7 +22162,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22176,7 +22200,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22218,7 +22242,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22256,7 +22280,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22298,7 +22322,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22336,7 +22360,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22378,7 +22402,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -22416,7 +22440,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22454,7 +22478,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22496,7 +22520,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -22728,7 +22752,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -22770,7 +22794,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22812,7 +22836,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22854,7 +22878,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -22896,7 +22920,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22938,7 +22962,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -22980,7 +23004,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -23023,7 +23047,7 @@
       <c r="F97" s="2" t="inlineStr"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -23060,7 +23084,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -23102,7 +23126,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -23144,7 +23168,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -23186,7 +23210,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23228,7 +23252,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23270,7 +23294,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23312,7 +23336,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23354,7 +23378,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -23396,7 +23420,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -23438,7 +23462,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -23481,7 +23505,7 @@
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -23518,7 +23542,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23560,7 +23584,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23602,7 +23626,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23644,7 +23668,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23686,7 +23710,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -23728,7 +23752,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23770,7 +23794,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23812,7 +23836,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23854,7 +23878,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23896,7 +23920,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23938,7 +23962,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -23980,7 +24004,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -24022,7 +24046,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -24064,7 +24088,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -24106,7 +24130,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -24148,7 +24172,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24186,7 +24210,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24228,7 +24252,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24270,7 +24294,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24312,7 +24336,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24354,7 +24378,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24396,7 +24420,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24438,7 +24462,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24480,7 +24504,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24522,7 +24546,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24564,7 +24588,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24606,7 +24630,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24648,7 +24672,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24690,7 +24714,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24732,7 +24756,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -24774,7 +24798,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24816,7 +24840,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24858,7 +24882,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24900,7 +24924,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24942,7 +24966,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -24984,7 +25008,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -25026,7 +25050,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -25068,7 +25092,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -25110,7 +25134,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -25152,7 +25176,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25194,7 +25218,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25236,7 +25260,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -25278,7 +25302,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25320,7 +25344,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25362,7 +25386,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25405,7 +25429,7 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -25442,7 +25466,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25484,7 +25508,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -25526,7 +25550,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25568,7 +25592,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25610,7 +25634,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25652,7 +25676,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25694,7 +25718,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25736,7 +25760,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25778,7 +25802,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -25820,7 +25844,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25862,7 +25886,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25904,7 +25928,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -25946,7 +25970,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -25988,7 +26012,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -26030,7 +26054,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -26072,7 +26096,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -26114,7 +26138,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -26156,7 +26180,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26198,7 +26222,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26240,7 +26264,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26282,7 +26306,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -26324,7 +26348,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26366,7 +26390,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26408,7 +26432,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26450,7 +26474,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26492,7 +26516,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26534,7 +26558,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26576,7 +26600,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26618,7 +26642,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26660,7 +26684,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26702,7 +26726,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26744,7 +26768,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26786,7 +26810,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26828,7 +26852,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26870,7 +26894,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26913,7 +26937,7 @@
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -26950,7 +26974,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -26992,7 +27016,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -27034,7 +27058,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -27076,7 +27100,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -27118,7 +27142,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -27160,7 +27184,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27202,7 +27226,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27244,7 +27268,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27286,7 +27310,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27324,7 +27348,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27366,7 +27390,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27404,7 +27428,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27446,7 +27470,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27488,7 +27512,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27526,7 +27550,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27564,7 +27588,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27602,7 +27626,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27640,7 +27664,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27678,7 +27702,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27716,7 +27740,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27754,7 +27778,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27792,7 +27816,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27834,7 +27858,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27876,7 +27900,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27914,7 +27938,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27952,7 +27976,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -27990,7 +28014,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -28028,7 +28052,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -28066,7 +28090,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-03T12:42:39+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-04 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,12 +2890,12 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27T13:03:11+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>36cfe7e7863f9d1460b8dc4a91e8c1baec01e9664a492fb99d918b34bf2b6ea3</t>
+          <t>2959d548616852711e1dc9a8dabc9bed791fca8d77122e8792af1c662e96519b</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8046,12 +8046,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>f2db90db914c14635ea9f1f6c7bd7e5fc5a9739b8b7b35d8467c1d56f4f7cacc</t>
+          <t>41bb8bddc00411ec1c97dd67a6057a53d9114db48fa7268ccaf2b9b6133e0223</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8650,7 +8650,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10682,7 +10682,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10930,7 +10930,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11002,12 +11002,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>1e627458f1a0b6608587445d37ecb2b997a405962bf4695b100df799058ea10d</t>
+          <t>89c578400ba3bbd8545dcc1761229fe90ce83c988fc7bd1c993e27061014b3b6</t>
         </is>
       </c>
     </row>
@@ -11074,7 +11074,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11146,7 +11146,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11218,7 +11218,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11566,12 +11566,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>a03e1de236c1d2d887b92cce731219d887ebfa90a794e0d18449db8cc530766c</t>
+          <t>6897297a57ed16fb0c0473afa7e019e8ca71cbf8bac0148ab06d9f59bcb52ac5</t>
         </is>
       </c>
     </row>
@@ -11638,7 +11638,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11706,7 +11706,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11774,7 +11774,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11846,7 +11846,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11978,12 +11978,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>833809f7222e45a7cbd4ee2ea73bd90b0716d7e2bef03208131645768aa07489</t>
+          <t>91d5fb062194e170ca2e9688a9586bacd8e1202b3cbcbe53555801441f8118e9</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12050,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12118,7 +12118,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12190,7 +12190,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12486,7 +12486,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12734,7 +12734,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
@@ -17622,7 +17622,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr"/>
@@ -17686,7 +17686,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr"/>
@@ -17754,7 +17754,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr"/>
@@ -17822,7 +17822,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr"/>
@@ -17890,7 +17890,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr"/>
@@ -18014,7 +18014,7 @@
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr"/>
@@ -18082,7 +18082,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr"/>
@@ -18314,7 +18314,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18378,7 +18378,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18442,7 +18442,7 @@
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K318" s="2" t="inlineStr"/>
@@ -18510,7 +18510,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18578,7 +18578,7 @@
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K320" s="2" t="inlineStr"/>
@@ -18646,12 +18646,12 @@
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L321" s="2" t="inlineStr">
@@ -18666,7 +18666,7 @@
       </c>
       <c r="N321" s="2" t="inlineStr">
         <is>
-          <t>933101db3dfa9c9b136935ae5c0369e51954e0b6e8d17128fa07bab9c5a416d0</t>
+          <t>ef10472491bb1e77525eddbe0ad0a1059c4905a72e74fa5b8afb24b6b6708f3d</t>
         </is>
       </c>
     </row>
@@ -18718,12 +18718,12 @@
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
@@ -18738,7 +18738,7 @@
       </c>
       <c r="N322" s="2" t="inlineStr">
         <is>
-          <t>165c478a2b03fbbf3ab802883170010c6578aa773b45f59d6bb62db5c54c89c1</t>
+          <t>1c4f4963d4b82f6a879f315fe62b3559a4306e3e5475181075a0244ce2f57f43</t>
         </is>
       </c>
     </row>
@@ -18790,12 +18790,12 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
@@ -18810,7 +18810,7 @@
       </c>
       <c r="N323" s="2" t="inlineStr">
         <is>
-          <t>ba86226392bfc98df6eeb51f0fe16527f412b502525455c7c54564a43e870d90</t>
+          <t>1df3ebd86bf5cced6e039a523378089385b83c6c2ec96d5ed1bf23fb44e97062</t>
         </is>
       </c>
     </row>
@@ -19224,7 +19224,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19304,7 +19304,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19342,7 +19342,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19380,7 +19380,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19418,7 +19418,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19498,7 +19498,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19536,7 +19536,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -19620,7 +19620,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19704,7 +19704,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -19746,7 +19746,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19788,7 +19788,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19830,7 +19830,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19914,7 +19914,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19956,7 +19956,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -19998,7 +19998,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -20082,7 +20082,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -20120,7 +20120,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20162,7 +20162,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20200,7 +20200,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20284,7 +20284,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20326,7 +20326,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20368,7 +20368,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20410,7 +20410,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20448,7 +20448,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20486,7 +20486,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20524,7 +20524,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20566,7 +20566,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20608,7 +20608,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20646,7 +20646,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20684,7 +20684,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20726,7 +20726,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20764,7 +20764,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20806,7 +20806,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20844,7 +20844,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20882,7 +20882,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20924,7 +20924,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20962,7 +20962,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -21000,7 +21000,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -21038,7 +21038,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -21080,7 +21080,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -21118,7 +21118,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21160,7 +21160,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21202,7 +21202,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21244,7 +21244,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21324,7 +21324,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21362,7 +21362,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21400,7 +21400,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21442,7 +21442,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21480,7 +21480,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21522,7 +21522,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21564,7 +21564,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21602,7 +21602,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21644,7 +21644,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21686,7 +21686,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21724,7 +21724,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21766,7 +21766,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21846,7 +21846,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21888,7 +21888,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21930,7 +21930,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21968,7 +21968,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -22006,7 +22006,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -22082,7 +22082,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -22120,7 +22120,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22162,7 +22162,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22200,7 +22200,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22242,7 +22242,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22280,7 +22280,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22360,7 +22360,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22402,7 +22402,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22478,7 +22478,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22520,7 +22520,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -22752,7 +22752,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -22794,7 +22794,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22878,7 +22878,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -22920,7 +22920,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -23047,7 +23047,7 @@
       <c r="F97" s="2" t="inlineStr"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -23084,7 +23084,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -23126,7 +23126,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -23168,7 +23168,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23252,7 +23252,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23294,7 +23294,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23336,7 +23336,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23378,7 +23378,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -23420,7 +23420,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -23462,7 +23462,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -23505,7 +23505,7 @@
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -23542,7 +23542,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23584,7 +23584,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23626,7 +23626,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23668,7 +23668,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23710,7 +23710,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -23752,7 +23752,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23794,7 +23794,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23836,7 +23836,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23878,7 +23878,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23962,7 +23962,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -24004,7 +24004,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -24046,7 +24046,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -24088,7 +24088,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -24130,7 +24130,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -24172,7 +24172,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24252,7 +24252,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24294,7 +24294,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24336,7 +24336,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24378,7 +24378,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24462,7 +24462,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24504,7 +24504,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24546,7 +24546,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24630,7 +24630,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24672,7 +24672,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24756,7 +24756,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -24798,7 +24798,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24840,7 +24840,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24882,7 +24882,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -25050,7 +25050,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -25134,7 +25134,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25218,7 +25218,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25260,7 +25260,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25386,7 +25386,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25429,7 +25429,7 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -25466,7 +25466,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25508,7 +25508,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25592,7 +25592,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25634,7 +25634,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25676,7 +25676,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25718,7 +25718,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25760,7 +25760,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25802,7 +25802,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -25844,7 +25844,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25886,7 +25886,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25928,7 +25928,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -25970,7 +25970,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -26012,7 +26012,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -26054,7 +26054,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -26096,7 +26096,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -26138,7 +26138,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -26180,7 +26180,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26222,7 +26222,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26264,7 +26264,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26306,7 +26306,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26390,7 +26390,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26432,7 +26432,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26474,7 +26474,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26516,7 +26516,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26558,7 +26558,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26600,7 +26600,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26642,7 +26642,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26684,7 +26684,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26726,7 +26726,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26768,7 +26768,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26810,7 +26810,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26852,7 +26852,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26894,7 +26894,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26937,7 +26937,7 @@
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -26974,7 +26974,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -27016,7 +27016,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -27058,7 +27058,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -27100,7 +27100,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -27142,7 +27142,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -27184,7 +27184,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27226,7 +27226,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27268,7 +27268,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27310,7 +27310,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27348,7 +27348,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27390,7 +27390,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27428,7 +27428,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27470,7 +27470,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27512,7 +27512,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27550,7 +27550,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27588,7 +27588,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27626,7 +27626,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27702,7 +27702,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27778,7 +27778,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27816,7 +27816,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27858,7 +27858,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27900,7 +27900,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27938,7 +27938,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27976,7 +27976,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -28014,7 +28014,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -28052,7 +28052,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -28090,7 +28090,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-04T13:23:24+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-06 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,12 +6506,12 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>2026-09-28T15:25:45+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L114" s="2" t="inlineStr"/>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>62d32530d603b027f9449498244ff9de23502a87dc8d606d86478637471e5684</t>
+          <t>6b57b6d45119bce4b9c57e0b98d5f324efd8b16950e41e2d4023b2da03de8a0e</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8046,12 +8046,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>e9a6db2f1663a429f716ede6b119a280060111f374313463f7a73591164a42fc</t>
+          <t>f12403b7a1cc63984c43f841bf2865772461e58cbef99b4f532c4d2fc7041e18</t>
         </is>
       </c>
     </row>
@@ -8114,12 +8114,12 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr"/>
@@ -8130,7 +8130,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>adf162ed7b842000a90a035785f195d2b79c09c5c96f4eaa8067ee7465165418</t>
+          <t>9825a4080be5b83710d18831e519177abf270fe4990d866e180fe916c7b547c3</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8182,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8650,7 +8650,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10682,7 +10682,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10930,7 +10930,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11002,12 +11002,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>c102e7fe26decfa874ac383a4a1d7bd005d937e1462d782735a7771e2d177423</t>
+          <t>faecac775446d161bc25628d75c0dbf3e28c74d9f3eb7b2898e96efc5917f7f8</t>
         </is>
       </c>
     </row>
@@ -11074,12 +11074,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>e79075eec0bf49747b960b963efedecb66fe299c4e23250c66e370bbe9e4591d</t>
+          <t>bb894f5a3ae71936a627f4a8762561f8cd4dc803f03a08a6821da68bdbf8ae74</t>
         </is>
       </c>
     </row>
@@ -11146,12 +11146,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>2d4a8326a9c94a27ef5040114b78890944853bf26476e0a6701bffa8e238c683</t>
+          <t>968164f9b0add901aad6c07bcb2af93c281fa5d1ba806f4a79916b71bd17a4c0</t>
         </is>
       </c>
     </row>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11566,12 +11566,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T13:23:24+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>6897297a57ed16fb0c0473afa7e019e8ca71cbf8bac0148ab06d9f59bcb52ac5</t>
+          <t>02241835dc3d885000d0df63df6e8a26c22cb9e4b7a142ce6242caf7f9a4772d</t>
         </is>
       </c>
     </row>
@@ -11638,7 +11638,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11706,7 +11706,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11774,12 +11774,12 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -11794,7 +11794,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>fe075697d40a7f9db49816d88ebd93f9cfab60e0a572e64769ad7d5aed73a088</t>
+          <t>dc81c5532c7c0b6c9b507b2421ff5c1044154fa78817e439049417a443153446</t>
         </is>
       </c>
     </row>
@@ -11846,7 +11846,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11978,12 +11978,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>3b39fc00e1dab0946952c77cb893dfbe48fe3d66ba35fbf362b3083d4fff62f8</t>
+          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12050,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12118,12 +12118,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-03T12:42:39+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
+          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
         </is>
       </c>
     </row>
@@ -12190,7 +12190,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12486,7 +12486,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12734,7 +12734,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
@@ -17622,7 +17622,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr"/>
@@ -17686,7 +17686,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr"/>
@@ -17754,7 +17754,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr"/>
@@ -17822,7 +17822,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr"/>
@@ -17890,7 +17890,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr"/>
@@ -18014,7 +18014,7 @@
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr"/>
@@ -18082,7 +18082,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr"/>
@@ -18314,7 +18314,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18378,7 +18378,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18442,7 +18442,7 @@
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K318" s="2" t="inlineStr"/>
@@ -18510,7 +18510,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18578,7 +18578,7 @@
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K320" s="2" t="inlineStr"/>
@@ -18646,12 +18646,12 @@
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L321" s="2" t="inlineStr">
@@ -18666,7 +18666,7 @@
       </c>
       <c r="N321" s="2" t="inlineStr">
         <is>
-          <t>b8a5a3e3360ef50d728fcc16b8ed870564f5c926e72f77ef55e37ac04492866c</t>
+          <t>b1f042feb790c64770217fb4ba4cae804d796d7405a7db660bb10b923a7bc25b</t>
         </is>
       </c>
     </row>
@@ -18718,12 +18718,12 @@
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
@@ -18738,7 +18738,7 @@
       </c>
       <c r="N322" s="2" t="inlineStr">
         <is>
-          <t>bcd668f4856ef65ceb01d88aeb79e3e8f06cae8af6d5a7b898cdec101f20be86</t>
+          <t>d3cfe4d23d5c86175f3b3a6f8a41b2c13f93b826c0148365b64cf70006bf1bcf</t>
         </is>
       </c>
     </row>
@@ -18790,12 +18790,12 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
@@ -18810,7 +18810,7 @@
       </c>
       <c r="N323" s="2" t="inlineStr">
         <is>
-          <t>a10ae534249fc9e112f21952181faa35baae55b8948c00b31651c3107d4df655</t>
+          <t>88e53baea21cab237960e37590e0e0fa0fabf8a0bd0cd38ac3cbe2072e501d82</t>
         </is>
       </c>
     </row>
@@ -19224,7 +19224,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19262,7 +19262,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19304,7 +19304,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19342,7 +19342,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19380,7 +19380,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19418,7 +19418,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19456,7 +19456,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19498,7 +19498,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19536,7 +19536,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19583,7 +19583,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -19620,7 +19620,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -19662,7 +19662,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19704,7 +19704,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -19746,7 +19746,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19788,7 +19788,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19830,7 +19830,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19914,7 +19914,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19956,7 +19956,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -19998,7 +19998,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -20040,7 +20040,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -20082,7 +20082,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -20120,7 +20120,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20162,7 +20162,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20200,7 +20200,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20242,7 +20242,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20284,7 +20284,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20326,7 +20326,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20368,7 +20368,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20410,7 +20410,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20448,7 +20448,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20486,7 +20486,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20524,7 +20524,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20566,7 +20566,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20608,7 +20608,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20646,7 +20646,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20684,7 +20684,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20726,7 +20726,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20764,7 +20764,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20806,7 +20806,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20844,7 +20844,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20882,7 +20882,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20924,7 +20924,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20962,7 +20962,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -21000,7 +21000,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -21038,7 +21038,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -21080,7 +21080,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -21118,7 +21118,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21160,7 +21160,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21202,7 +21202,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21244,7 +21244,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21286,7 +21286,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21324,7 +21324,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21362,7 +21362,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21400,7 +21400,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21442,7 +21442,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21480,7 +21480,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21522,7 +21522,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21564,7 +21564,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21602,7 +21602,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21644,7 +21644,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21686,7 +21686,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21724,7 +21724,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21766,7 +21766,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21804,7 +21804,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21846,7 +21846,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21888,7 +21888,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21930,7 +21930,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21968,7 +21968,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -22006,7 +22006,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -22044,7 +22044,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -22082,7 +22082,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -22120,7 +22120,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22162,7 +22162,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22200,7 +22200,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22242,7 +22242,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22280,7 +22280,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22322,7 +22322,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22360,7 +22360,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22402,7 +22402,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -22440,7 +22440,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22478,7 +22478,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22520,7 +22520,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -22752,7 +22752,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -22794,7 +22794,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22836,7 +22836,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22878,7 +22878,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -22920,7 +22920,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22962,7 +22962,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -23004,7 +23004,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -23047,7 +23047,7 @@
       <c r="F97" s="2" t="inlineStr"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -23084,7 +23084,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -23126,7 +23126,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -23168,7 +23168,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -23210,7 +23210,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23252,7 +23252,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23294,7 +23294,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23336,7 +23336,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23378,7 +23378,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -23420,7 +23420,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -23462,7 +23462,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -23505,7 +23505,7 @@
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -23542,7 +23542,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23584,7 +23584,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23626,7 +23626,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23668,7 +23668,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23710,7 +23710,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -23752,7 +23752,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23794,7 +23794,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23836,7 +23836,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23878,7 +23878,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23920,7 +23920,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23962,7 +23962,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -24004,7 +24004,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -24046,7 +24046,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -24088,7 +24088,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -24130,7 +24130,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -24172,7 +24172,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24210,7 +24210,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24252,7 +24252,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24294,7 +24294,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24336,7 +24336,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24378,7 +24378,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24420,7 +24420,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24462,7 +24462,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24504,7 +24504,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24546,7 +24546,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24630,7 +24630,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24672,7 +24672,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24756,7 +24756,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -24798,7 +24798,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24840,7 +24840,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24882,7 +24882,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24924,7 +24924,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24966,7 +24966,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -25008,7 +25008,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -25050,7 +25050,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -25092,7 +25092,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -25134,7 +25134,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -25176,7 +25176,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25218,7 +25218,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25260,7 +25260,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25344,7 +25344,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25386,7 +25386,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25429,7 +25429,7 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -25466,7 +25466,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25508,7 +25508,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25592,7 +25592,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25634,7 +25634,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25676,7 +25676,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25718,7 +25718,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25760,7 +25760,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25802,7 +25802,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -25844,7 +25844,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25886,7 +25886,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25928,7 +25928,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -25970,7 +25970,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -26012,7 +26012,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -26054,7 +26054,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -26096,7 +26096,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -26138,7 +26138,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -26180,7 +26180,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26222,7 +26222,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26264,7 +26264,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26306,7 +26306,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -26348,7 +26348,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26390,7 +26390,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26432,7 +26432,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26474,7 +26474,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26516,7 +26516,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26558,7 +26558,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26600,7 +26600,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26642,7 +26642,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26684,7 +26684,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26726,7 +26726,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26768,7 +26768,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26810,7 +26810,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26852,7 +26852,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26894,7 +26894,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26937,7 +26937,7 @@
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -26974,7 +26974,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -27016,7 +27016,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -27058,7 +27058,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -27100,7 +27100,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -27142,7 +27142,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -27184,7 +27184,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27226,7 +27226,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27268,7 +27268,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27310,7 +27310,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27348,7 +27348,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27390,7 +27390,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27428,7 +27428,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27470,7 +27470,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27512,7 +27512,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27550,7 +27550,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27588,7 +27588,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27626,7 +27626,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27664,7 +27664,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27702,7 +27702,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27740,7 +27740,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27778,7 +27778,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27816,7 +27816,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27858,7 +27858,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27900,7 +27900,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27938,7 +27938,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27976,7 +27976,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -28014,7 +28014,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -28052,7 +28052,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -28090,7 +28090,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-07 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,12 +2890,12 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-04T13:23:24+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>
@@ -2906,7 +2906,7 @@
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>2959d548616852711e1dc9a8dabc9bed791fca8d77122e8792af1c662e96519b</t>
+          <t>36cfe7e7863f9d1460b8dc4a91e8c1baec01e9664a492fb99d918b34bf2b6ea3</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8046,12 +8046,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>f12403b7a1cc63984c43f841bf2865772461e58cbef99b4f532c4d2fc7041e18</t>
+          <t>16a4ff0e9a0990e1da9315a22305f12f2528e33c90ad55449361f8b329cdd2f2</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8650,7 +8650,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10682,7 +10682,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10930,7 +10930,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11002,12 +11002,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>faecac775446d161bc25628d75c0dbf3e28c74d9f3eb7b2898e96efc5917f7f8</t>
+          <t>2d2099bc333d09757dc4bf16560e448d692e36bde3968c862e53d488b982504d</t>
         </is>
       </c>
     </row>
@@ -11074,7 +11074,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11146,12 +11146,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>968164f9b0add901aad6c07bcb2af93c281fa5d1ba806f4a79916b71bd17a4c0</t>
+          <t>a564f254ee375aa2d736f798efe0b02a808b4733e318c21fca0e974ce470c5ec</t>
         </is>
       </c>
     </row>
@@ -11218,7 +11218,7 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
@@ -11290,7 +11290,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11566,12 +11566,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>02241835dc3d885000d0df63df6e8a26c22cb9e4b7a142ce6242caf7f9a4772d</t>
+          <t>a1f7a561fc8f794ccb444ef66e1031b1c2ae4aa658b30650696e2bc7ec2c7b1e</t>
         </is>
       </c>
     </row>
@@ -11638,7 +11638,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11706,7 +11706,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr"/>
@@ -11774,12 +11774,12 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -11794,7 +11794,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>dc81c5532c7c0b6c9b507b2421ff5c1044154fa78817e439049417a443153446</t>
+          <t>fe407a1f970cb6774a68730ac78b1812bb948b211b14501b52cdc9c3a22dbccf</t>
         </is>
       </c>
     </row>
@@ -11846,7 +11846,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11978,12 +11978,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11998,7 +11998,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
+          <t>0398a8b2f44e87e35cebc2bc39be0125946115179470248ee01cc1b367a10e6a</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12050,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12118,12 +12118,12 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L209" s="2" t="inlineStr">
@@ -12138,7 +12138,7 @@
       </c>
       <c r="N209" s="2" t="inlineStr">
         <is>
-          <t>2b48cfa758cf26f1d5088203c6833faf49ccc262a35081cbeac530c44ab1f8c3</t>
+          <t>9dc659d5a1fe3b03e2ee07ac61ff49350faf5a66cf12f7e0d9c141c6ecc1c17d</t>
         </is>
       </c>
     </row>
@@ -12190,7 +12190,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12486,7 +12486,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12734,7 +12734,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12802,7 +12802,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12870,7 +12870,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -17545,17 +17545,17 @@
       </c>
       <c r="I304" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L304" s="2" t="inlineStr">
@@ -17570,7 +17570,7 @@
       </c>
       <c r="N304" s="2" t="inlineStr">
         <is>
-          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
+          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
         </is>
       </c>
     </row>
@@ -17622,7 +17622,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr"/>
@@ -17686,10 +17686,14 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
-        </is>
-      </c>
-      <c r="K306" s="2" t="inlineStr"/>
+          <t>2026-10-07T14:42:32+00:00</t>
+        </is>
+      </c>
+      <c r="K306" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07T14:42:32+00:00</t>
+        </is>
+      </c>
       <c r="L306" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -17702,7 +17706,7 @@
       </c>
       <c r="N306" s="2" t="inlineStr">
         <is>
-          <t>c96cbecf17320ed640804a102893b8853b7ccd7d27a0445c6629132a813161fe</t>
+          <t>337c3d5c81cd7fdc69c92fddb83f5908e33136b373106e1b5e1c03e302dc5adb</t>
         </is>
       </c>
     </row>
@@ -17754,7 +17758,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr"/>
@@ -17822,7 +17826,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr"/>
@@ -17890,7 +17894,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr"/>
@@ -18014,7 +18018,7 @@
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr"/>
@@ -18082,7 +18086,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr"/>
@@ -18314,7 +18318,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18378,7 +18382,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18442,7 +18446,7 @@
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K318" s="2" t="inlineStr"/>
@@ -18510,7 +18514,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18578,7 +18582,7 @@
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K320" s="2" t="inlineStr"/>
@@ -18646,12 +18650,12 @@
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L321" s="2" t="inlineStr">
@@ -18666,7 +18670,7 @@
       </c>
       <c r="N321" s="2" t="inlineStr">
         <is>
-          <t>b1f042feb790c64770217fb4ba4cae804d796d7405a7db660bb10b923a7bc25b</t>
+          <t>1eee3f863b2760f35f4fc5caead5f08a4d767cab3af7e02a10d9909950eae00e</t>
         </is>
       </c>
     </row>
@@ -18718,12 +18722,12 @@
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
@@ -18738,7 +18742,7 @@
       </c>
       <c r="N322" s="2" t="inlineStr">
         <is>
-          <t>d3cfe4d23d5c86175f3b3a6f8a41b2c13f93b826c0148365b64cf70006bf1bcf</t>
+          <t>f65ab4a0614cb236d1659b60b5f9c62d230989a6c1f4046bc5a6beb58a3b202f</t>
         </is>
       </c>
     </row>
@@ -18790,12 +18794,12 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
@@ -18810,7 +18814,7 @@
       </c>
       <c r="N323" s="2" t="inlineStr">
         <is>
-          <t>88e53baea21cab237960e37590e0e0fa0fabf8a0bd0cd38ac3cbe2072e501d82</t>
+          <t>a5292dfeb2b4ed0478c525575d6049eabe86c183078f49012976a9352c0139ab</t>
         </is>
       </c>
     </row>
@@ -19224,7 +19228,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19262,7 +19266,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19304,7 +19308,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19342,7 +19346,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19380,7 +19384,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19418,7 +19422,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19456,7 +19460,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19498,7 +19502,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19536,7 +19540,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19583,7 +19587,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -19620,7 +19624,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -19662,7 +19666,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19704,7 +19708,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -19746,7 +19750,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19788,7 +19792,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19830,7 +19834,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19872,7 +19876,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19914,7 +19918,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19956,7 +19960,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -19998,7 +20002,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -20040,7 +20044,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -20082,7 +20086,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -20120,7 +20124,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20162,7 +20166,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20200,7 +20204,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20242,7 +20246,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20284,7 +20288,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20326,7 +20330,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20368,7 +20372,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20410,7 +20414,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20448,7 +20452,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20486,7 +20490,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20524,7 +20528,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20566,7 +20570,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20608,7 +20612,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20646,7 +20650,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20684,7 +20688,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20726,7 +20730,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20764,7 +20768,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20806,7 +20810,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20844,7 +20848,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20882,7 +20886,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20924,7 +20928,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20962,7 +20966,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -21000,7 +21004,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -21038,7 +21042,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -21080,7 +21084,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -21118,7 +21122,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21160,7 +21164,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21202,7 +21206,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21244,7 +21248,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21286,7 +21290,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21324,7 +21328,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21362,7 +21366,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21400,7 +21404,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21442,7 +21446,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21480,7 +21484,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21522,7 +21526,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21564,7 +21568,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21602,7 +21606,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21644,7 +21648,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21686,7 +21690,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21724,7 +21728,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21766,7 +21770,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21804,7 +21808,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21846,7 +21850,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21888,7 +21892,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21930,7 +21934,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21968,7 +21972,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -22006,7 +22010,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -22044,7 +22048,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -22082,7 +22086,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -22120,7 +22124,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22162,7 +22166,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22200,7 +22204,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22242,7 +22246,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22280,7 +22284,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22322,7 +22326,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22360,7 +22364,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22402,7 +22406,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -22440,7 +22444,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22478,7 +22482,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22520,7 +22524,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -22752,7 +22756,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -22794,7 +22798,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22836,7 +22840,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22878,7 +22882,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -22920,7 +22924,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22962,7 +22966,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -23004,7 +23008,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -23047,7 +23051,7 @@
       <c r="F97" s="2" t="inlineStr"/>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -23084,7 +23088,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -23126,7 +23130,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -23168,7 +23172,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -23210,7 +23214,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23252,7 +23256,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23294,7 +23298,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23336,7 +23340,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23378,7 +23382,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -23420,7 +23424,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -23462,7 +23466,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -23505,7 +23509,7 @@
       <c r="F108" s="2" t="inlineStr"/>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -23542,7 +23546,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23584,7 +23588,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23626,7 +23630,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23668,7 +23672,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23710,7 +23714,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -23752,7 +23756,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23794,7 +23798,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23836,7 +23840,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23878,7 +23882,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23920,7 +23924,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23962,7 +23966,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -24004,7 +24008,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -24046,7 +24050,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -24088,7 +24092,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -24130,7 +24134,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -24172,7 +24176,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24210,7 +24214,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24252,7 +24256,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24294,7 +24298,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24336,7 +24340,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24378,7 +24382,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24420,7 +24424,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24462,7 +24466,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24504,7 +24508,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24546,7 +24550,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24588,7 +24592,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24630,7 +24634,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24672,7 +24676,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24714,7 +24718,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24761,7 +24765,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -24798,7 +24802,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24840,7 +24844,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24882,7 +24886,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24924,7 +24928,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24966,7 +24970,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -25008,7 +25012,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -25050,7 +25054,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -25092,7 +25096,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -25134,7 +25138,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -25176,7 +25180,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25218,7 +25222,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25260,7 +25264,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -25302,7 +25306,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25344,7 +25348,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25386,7 +25390,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25429,7 +25433,7 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -25466,7 +25470,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25508,7 +25512,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -25550,7 +25554,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25592,7 +25596,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25634,7 +25638,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25676,7 +25680,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25718,7 +25722,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25760,7 +25764,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25802,7 +25806,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -25844,7 +25848,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25886,7 +25890,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25928,7 +25932,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -25970,7 +25974,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -26012,7 +26016,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -26054,7 +26058,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -26096,7 +26100,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -26138,7 +26142,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -26180,7 +26184,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26222,7 +26226,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26264,7 +26268,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26306,7 +26310,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -26348,7 +26352,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26390,7 +26394,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26432,7 +26436,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26474,7 +26478,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26516,7 +26520,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26558,7 +26562,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26600,7 +26604,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26642,7 +26646,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26684,7 +26688,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26726,7 +26730,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26768,7 +26772,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26810,7 +26814,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26852,7 +26856,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26894,7 +26898,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26937,7 +26941,7 @@
       <c r="F190" s="2" t="inlineStr"/>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -26974,7 +26978,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -27016,7 +27020,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -27058,7 +27062,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -27100,7 +27104,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -27142,7 +27146,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -27184,7 +27188,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27226,7 +27230,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27268,7 +27272,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27310,7 +27314,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27348,7 +27352,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27390,7 +27394,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27428,7 +27432,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27470,7 +27474,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27512,7 +27516,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27550,7 +27554,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27588,7 +27592,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27626,7 +27630,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27664,7 +27668,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27702,7 +27706,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27740,7 +27744,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27778,7 +27782,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27816,7 +27820,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27858,7 +27862,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27900,7 +27904,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27938,7 +27942,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27976,7 +27980,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -28014,7 +28018,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -28052,7 +28056,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -28090,7 +28094,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-08 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -7982,7 +7982,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8046,12 +8046,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8062,7 +8062,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>16a4ff0e9a0990e1da9315a22305f12f2528e33c90ad55449361f8b329cdd2f2</t>
+          <t>bfdd2e277c2c12081d4935c0396b97768545901235ccd3b5d52a70b6c940ff94</t>
         </is>
       </c>
     </row>
@@ -8114,7 +8114,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8182,7 +8182,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8246,7 +8246,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8650,7 +8650,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8722,7 +8722,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8850,7 +8850,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
@@ -8990,7 +8990,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10682,7 +10682,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10862,7 +10862,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10930,7 +10930,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11002,12 +11002,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11022,7 +11022,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>2d2099bc333d09757dc4bf16560e448d692e36bde3968c862e53d488b982504d</t>
+          <t>55aa3c3b411138dba0e0c12558b43e7e4e74fecce5f11007874d8206b922daa3</t>
         </is>
       </c>
     </row>
@@ -11074,12 +11074,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11094,7 +11094,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>bb894f5a3ae71936a627f4a8762561f8cd4dc803f03a08a6821da68bdbf8ae74</t>
+          <t>c52b57cce9eb161c21a787804f715604ea4b9b4451a07f4c154df106687dae71</t>
         </is>
       </c>
     </row>
@@ -11146,12 +11146,12 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L195" s="2" t="inlineStr">
@@ -11166,7 +11166,7 @@
       </c>
       <c r="N195" s="2" t="inlineStr">
         <is>
-          <t>a564f254ee375aa2d736f798efe0b02a808b4733e318c21fca0e974ce470c5ec</t>
+          <t>31621a2b6fefbe0c71c3012ec1bb8a03440e9275391996e332e7d65886dce713</t>
         </is>
       </c>
     </row>
@@ -11218,12 +11218,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:34:49+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11238,7 +11238,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>3c80905d1d6277e50be0a05b7d5620b2f1737012cd6187cf946d71d1a7bc8dcb</t>
+          <t>4a26ade2f69607e364c3af2b4ec186ffb3cf4ae890c4df9033aee06cab95819d</t>
         </is>
       </c>
     </row>
@@ -11290,7 +11290,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11362,7 +11362,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11430,7 +11430,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11498,7 +11498,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11566,12 +11566,12 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L201" s="2" t="inlineStr">
@@ -11586,7 +11586,7 @@
       </c>
       <c r="N201" s="2" t="inlineStr">
         <is>
-          <t>a1f7a561fc8f794ccb444ef66e1031b1c2ae4aa658b30650696e2bc7ec2c7b1e</t>
+          <t>8eab33f6305b65fe1f19eaa8ea7b68e36a0809fc821a1d1994609db876cec98b</t>
         </is>
       </c>
     </row>
@@ -11638,7 +11638,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11706,10 +11706,14 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
-        </is>
-      </c>
-      <c r="K203" s="2" t="inlineStr"/>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="L203" s="2" t="inlineStr">
         <is>
           <t>2026-09-26</t>
@@ -11722,7 +11726,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>2fc01320f3c51a593a2362a8d1325bcac7cdc06f0fc20560cadf39d2334f5d5d</t>
+          <t>7cf156acfa8cf7fd013d37471de6869ee4faa3c303815e72a9863af6079fa69f</t>
         </is>
       </c>
     </row>
@@ -11774,7 +11778,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11846,7 +11850,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11978,12 +11982,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -11998,7 +12002,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>0398a8b2f44e87e35cebc2bc39be0125946115179470248ee01cc1b367a10e6a</t>
+          <t>06087b9e6a42cd27c16a90c9604b634af5ed9e643e26c0d5a61830976615ff5d</t>
         </is>
       </c>
     </row>
@@ -12050,7 +12054,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12118,7 +12122,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12190,7 +12194,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12486,7 +12490,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12734,7 +12738,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12802,7 +12806,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12870,7 +12874,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -17550,12 +17554,12 @@
       </c>
       <c r="J304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K304" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L304" s="2" t="inlineStr">
@@ -17570,7 +17574,7 @@
       </c>
       <c r="N304" s="2" t="inlineStr">
         <is>
-          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
+          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
         </is>
       </c>
     </row>
@@ -17622,7 +17626,7 @@
       </c>
       <c r="J305" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K305" s="2" t="inlineStr"/>
@@ -17686,7 +17690,7 @@
       </c>
       <c r="J306" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K306" s="2" t="inlineStr">
@@ -17758,7 +17762,7 @@
       </c>
       <c r="J307" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K307" s="2" t="inlineStr"/>
@@ -17826,7 +17830,7 @@
       </c>
       <c r="J308" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K308" s="2" t="inlineStr"/>
@@ -17894,7 +17898,7 @@
       </c>
       <c r="J309" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K309" s="2" t="inlineStr"/>
@@ -18018,7 +18022,7 @@
       </c>
       <c r="J311" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K311" s="2" t="inlineStr"/>
@@ -18086,7 +18090,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr"/>
@@ -18318,7 +18322,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18382,7 +18386,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18446,7 +18450,7 @@
       </c>
       <c r="J318" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K318" s="2" t="inlineStr"/>
@@ -18514,7 +18518,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18582,7 +18586,7 @@
       </c>
       <c r="J320" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K320" s="2" t="inlineStr"/>
@@ -18650,12 +18654,12 @@
       </c>
       <c r="J321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K321" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L321" s="2" t="inlineStr">
@@ -18670,7 +18674,7 @@
       </c>
       <c r="N321" s="2" t="inlineStr">
         <is>
-          <t>1eee3f863b2760f35f4fc5caead5f08a4d767cab3af7e02a10d9909950eae00e</t>
+          <t>e551b13659a4f8862b63ed994c9170edce4e4d1ab9e6ac64edff474e7af9c2f6</t>
         </is>
       </c>
     </row>
@@ -18722,12 +18726,12 @@
       </c>
       <c r="J322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K322" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L322" s="2" t="inlineStr">
@@ -18742,7 +18746,7 @@
       </c>
       <c r="N322" s="2" t="inlineStr">
         <is>
-          <t>f65ab4a0614cb236d1659b60b5f9c62d230989a6c1f4046bc5a6beb58a3b202f</t>
+          <t>dede29f8b571b783b3c67925c068a1ff3c309eea041e18fbeaf1d1a1ed23ffe5</t>
         </is>
       </c>
     </row>
@@ -18794,12 +18798,12 @@
       </c>
       <c r="J323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="K323" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="L323" s="2" t="inlineStr">
@@ -18814,7 +18818,7 @@
       </c>
       <c r="N323" s="2" t="inlineStr">
         <is>
-          <t>a5292dfeb2b4ed0478c525575d6049eabe86c183078f49012976a9352c0139ab</t>
+          <t>7a8bd2d9b8a0739c578852b2825509d25db26005c7cd95298de5ba16da3e6d5b</t>
         </is>
       </c>
     </row>
@@ -19228,7 +19232,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -19266,7 +19270,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -19308,7 +19312,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19346,7 +19350,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19384,7 +19388,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19422,7 +19426,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19460,7 +19464,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19502,7 +19506,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19540,7 +19544,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19587,7 +19591,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -19624,7 +19628,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -19666,7 +19670,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -19708,7 +19712,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -19750,7 +19754,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -19792,7 +19796,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -19834,7 +19838,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -19876,7 +19880,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -19918,7 +19922,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -19960,7 +19964,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -20002,7 +20006,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -20044,7 +20048,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -20086,7 +20090,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -20124,7 +20128,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -20166,7 +20170,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -20204,7 +20208,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -20246,7 +20250,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -20288,7 +20292,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -20330,7 +20334,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -20372,7 +20376,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -20414,7 +20418,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -20452,7 +20456,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -20490,7 +20494,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -20528,7 +20532,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -20570,7 +20574,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -20612,7 +20616,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -20650,7 +20654,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -20688,7 +20692,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -20730,7 +20734,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -20768,7 +20772,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -20810,7 +20814,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -20848,7 +20852,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -20886,7 +20890,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -20928,7 +20932,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -20966,7 +20970,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -21004,7 +21008,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -21042,7 +21046,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -21084,7 +21088,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -21122,7 +21126,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -21164,7 +21168,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -21206,7 +21210,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -21248,7 +21252,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -21290,7 +21294,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -21328,7 +21332,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -21366,7 +21370,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -21404,7 +21408,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -21446,7 +21450,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -21484,7 +21488,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -21526,7 +21530,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -21568,7 +21572,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -21606,7 +21610,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -21648,7 +21652,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -21690,7 +21694,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -21728,7 +21732,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -21770,7 +21774,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -21808,7 +21812,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -21850,7 +21854,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -21892,7 +21896,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -21934,7 +21938,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -21972,7 +21976,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -22010,7 +22014,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -22048,7 +22052,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -22086,7 +22090,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -22124,7 +22128,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -22166,7 +22170,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -22204,7 +22208,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -22246,7 +22250,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -22284,7 +22288,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -22326,7 +22330,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -22364,7 +22368,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -22406,7 +22410,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -22444,7 +22448,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -22482,7 +22486,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -22524,7 +22528,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -22756,7 +22760,7 @@
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -22798,7 +22802,7 @@
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr">
@@ -22840,7 +22844,7 @@
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr">
@@ -22882,7 +22886,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -22924,7 +22928,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -22966,7 +22970,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -23008,7 +23012,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -23088,7 +23092,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -23130,7 +23134,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -23177,7 +23181,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -23214,7 +23218,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -23256,7 +23260,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -23298,7 +23302,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -23340,7 +23344,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -23382,7 +23386,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -23424,7 +23428,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -23466,7 +23470,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -23546,7 +23550,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -23588,7 +23592,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -23630,7 +23634,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -23672,7 +23676,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -23714,7 +23718,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -23756,7 +23760,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -23798,7 +23802,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -23840,7 +23844,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -23882,7 +23886,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -23924,7 +23928,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -23966,7 +23970,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -24008,7 +24012,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -24050,7 +24054,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -24092,7 +24096,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -24134,7 +24138,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -24176,7 +24180,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -24214,7 +24218,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -24256,7 +24260,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -24298,7 +24302,7 @@
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G127" s="2" t="inlineStr">
@@ -24340,7 +24344,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -24382,7 +24386,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -24424,7 +24428,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -24466,7 +24470,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -24508,7 +24512,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -24550,7 +24554,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -24592,7 +24596,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -24634,7 +24638,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -24676,7 +24680,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -24718,7 +24722,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -24765,7 +24769,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -24802,7 +24806,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -24844,7 +24848,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -24886,7 +24890,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -24928,7 +24932,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -24970,7 +24974,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -25012,7 +25016,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -25054,7 +25058,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -25096,7 +25100,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -25138,7 +25142,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -25180,7 +25184,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -25222,7 +25226,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -25264,7 +25268,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -25306,7 +25310,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -25348,7 +25352,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -25390,7 +25394,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -25470,7 +25474,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -25512,7 +25516,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -25554,7 +25558,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -25596,7 +25600,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -25638,7 +25642,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -25680,7 +25684,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -25722,7 +25726,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -25764,7 +25768,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -25806,7 +25810,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -25848,7 +25852,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -25890,7 +25894,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -25932,7 +25936,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -25974,7 +25978,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -26016,7 +26020,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -26063,7 +26067,7 @@
       </c>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr">
@@ -26100,7 +26104,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -26142,7 +26146,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -26184,7 +26188,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -26226,7 +26230,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -26268,7 +26272,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -26310,7 +26314,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -26352,7 +26356,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -26394,7 +26398,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -26436,7 +26440,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -26478,7 +26482,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -26520,7 +26524,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -26562,7 +26566,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -26604,7 +26608,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -26646,7 +26650,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -26688,7 +26692,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -26730,7 +26734,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -26772,7 +26776,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -26814,7 +26818,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -26856,7 +26860,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -26898,7 +26902,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -26978,7 +26982,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -27025,7 +27029,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -27062,7 +27066,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -27104,7 +27108,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -27146,7 +27150,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -27188,7 +27192,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -27230,7 +27234,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -27272,7 +27276,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -27314,7 +27318,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -27352,7 +27356,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -27394,7 +27398,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -27432,7 +27436,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -27474,7 +27478,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -27516,7 +27520,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -27554,7 +27558,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -27592,7 +27596,7 @@
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
@@ -27630,7 +27634,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -27668,7 +27672,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -27706,7 +27710,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -27744,7 +27748,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -27782,7 +27786,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -27820,7 +27824,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -27862,7 +27866,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -27904,7 +27908,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -27942,7 +27946,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -27980,7 +27984,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -28018,7 +28022,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -28056,7 +28060,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -28094,7 +28098,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">

</xml_diff>

<commit_message>
docs, xlsx: counts and workbooks after merging the source fixes
Three sources moved to method=manual in the same batch the hackathon
sources were added, so 229 watched sources are 221 fetched and 8 handled
by hand. Both workbooks are rebuilt from the merged CSVs.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -20309,7 +20309,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>aprameyak/2027-tech-jobs</t>
+          <t>aprameyak/2027-tech-jobs/SUMMER.md</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -20324,7 +20324,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Added 2026-10-01. Measured before adding: about 17 in-field US internships on neither Simplify's full list nor the existing watchlist. Links to the employer's own posting, so cross-source dedupe works on it.</t>
+          <t>Added 2026-10-01. Measured before adding: about 17 in-field US internships on neither Simplify's full list nor the existing watchlist. Links to the employer's own posting, so cross-source dedupe works on it. | 2026-10-08: url was aprameyak/2027-tech-jobs (README.md), now aprameyak/2027-tech-jobs/SUMMER.md. On 2026-10-05 the README dropped its newest-75 table for a page of links and parsed to 0 rows; SUMMER.md carries the full Summer 2027 table, 5,452 rows on 2026-10-08.</t>
         </is>
       </c>
     </row>
@@ -23273,7 +23273,7 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>citadel-students</t>
+          <t>berkeley-superb</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -23288,12 +23288,12 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Citadel students</t>
+          <t>Berkeley SUPERB-AI4E REU</t>
         </is>
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>https://www.citadel.com/careers/students/</t>
+          <t>https://eecs.berkeley.edu/resources/undergrads/undergraduate-research/superb/</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr"/>
@@ -23304,14 +23304,14 @@
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>method=manual on purpose. Re-tested 2026-09-11: 403 Forbidden to state.USER_AGENT, HTTP 200 to a spoofed browser User-Agent. The block is deliberate and UA-based, so the only way to automate this page is to lie about who we are - declined. Surfaces as a monthly calendar reminder instead. An earlier note claiming 6,763 chars of text was measured with a browser-presenting fetcher, not with this tool's client.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 8425 characters of visible text, no JavaScript needed. | MANUAL 2026-10-08: never once fetched from the Actions runner (HTTP 403 on all six runs 2026-10-02..07) while answering a laptop HTTP 200 under the same User-Agent on 2026-10-08 (236 lines). The 2026-10-01 verification was made from a laptop, which is why it missed this. eecs.berkeley.edu resolves to WP Engine (141.193.213.10/11, OrgName WPEngine), the same WAF that refused the runner for gtsx.com and twosigma.com. Probed alternatives: www2.eecs.berkeley.edu/Scholarships/SUPERB/ is a 404, and superb.berkeley.edu is an unrelated student-events site. Surfaces as a January calendar reminder instead.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>citadelsecurities-careers</t>
+          <t>caltech-surf</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -23326,12 +23326,12 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Citadel Securities</t>
+          <t>Caltech SURF</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>https://www.citadelsecurities.com/careers</t>
+          <t>https://sfp.caltech.edu/undergraduate-research/programs/surf/application_information</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr"/>
@@ -23342,14 +23342,14 @@
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>method=manual on purpose. Sampled 10x on 2026-09-11: HTTP 200 in 5 of 10 fetches, 403 Cloudflare in the other 5, all with state.USER_AGENT. An earlier note here claimed the page was readable at 10,638 chars - that was a single lucky sample, the same error made on citadel.com the same day. An INTERMITTENT block is worse than a hard one: the source would report a failure on roughly half of all runs and escalate into ACT NOW after three, so it must not be automated. Re-sample repeatedly, never once, before moving any Citadel row off manual.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 9174 characters of visible text, no JavaScript needed. | MANUAL 2026-10-08: never once fetched from the Actions runner (HTTP 403 on all six runs 2026-10-02..07) while answering a laptop HTTP 200 under the same User-Agent on 2026-10-08 (210 lines). The 2026-10-01 verification was made from a laptop, which is why it missed this. sfp.caltech.edu is a CNAME to sites.caltech.edu on Cloudflare, and www.caltech.edu is on Cloudflare too, so no second Caltech host was found. Surfaces as a January calendar reminder instead.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>kaggle-competitions</t>
+          <t>citadel-students</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -23359,17 +23359,17 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Kaggle Competitions (all active)</t>
+          <t>Citadel students</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>https://www.kaggle.com/api/v1/competitions/list</t>
+          <t>https://www.citadel.com/careers/students/</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr"/>
@@ -23380,14 +23380,14 @@
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>MANUAL. Kaggle competitions are always-open and rolling, so a daily diff is noise rather than news; calendar_reminders.ALWAYS already covers them. Dropped from Phase 2 deliberately.</t>
+          <t>method=manual on purpose. Re-tested 2026-09-11: 403 Forbidden to state.USER_AGENT, HTTP 200 to a spoofed browser User-Agent. The block is deliberate and UA-based, so the only way to automate this page is to lie about who we are - declined. Surfaces as a monthly calendar reminder instead. An earlier note claiming 6,763 chars of text was measured with a browser-presenting fetcher, not with this tool's client.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>spcs-jobs</t>
+          <t>citadelsecurities-careers</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -23397,17 +23397,17 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Stanford Pre-Collegiate Studies jobs (SUMaC RC / TA)</t>
+          <t>Citadel Securities</t>
         </is>
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>https://spcs.stanford.edu/residential-program-positions</t>
+          <t>https://www.citadelsecurities.com/careers</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr"/>
@@ -23418,14 +23418,14 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 4,757 chars, ratio 0.128. | MANUAL 2026-09-30: never once fetched from the Actions runner (403 on every run since it was added) while answering a laptop 200 under the same User-Agent. spcs.stanford.edu is on Pantheon (live-spcs.pantheonsite.io), which refuses datacenter IPs. No second route: Stanford's central Oracle HCM board (careersearch.stanford.edu, reachable) carries 0 Pre-Collegiate requisitions, so SPCS posts only on its own site. Re-pointed at the residential page (SUMaC RC/TA), which on 2026-09-30 said Summer 2026 is filled and offers an interest form for the Summer 2027 cycle.</t>
+          <t>method=manual on purpose. Sampled 10x on 2026-09-11: HTTP 200 in 5 of 10 fetches, 403 Cloudflare in the other 5, all with state.USER_AGENT. An earlier note here claimed the page was readable at 10,638 chars - that was a single lucky sample, the same error made on citadel.com the same day. An INTERMITTENT block is worse than a hard one: the source would report a failure on roughly half of all runs and escalate into ACT NOW after three, so it must not be automated. Re-sample repeatedly, never once, before moving any Citadel row off manual.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>thedeckgame</t>
+          <t>kaggle-competitions</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
@@ -23435,17 +23435,17 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>The Deck Game</t>
+          <t>Kaggle Competitions (all active)</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>https://thedeckgame.com/</t>
+          <t>https://www.kaggle.com/api/v1/competitions/list</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr"/>
@@ -23456,41 +23456,37 @@
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>MANUAL. Verified: JS shell yielding ~28 characters; sitemap has only two URLs. Not worth a Playwright run - there is nothing to diff.</t>
+          <t>MANUAL. Kaggle competitions are always-open and rolling, so a daily diff is noise rather than news; calendar_reminders.ALWAYS already covers them. Dropped from Phase 2 deliberately.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>nsf-reu-sites</t>
+          <t>spcs-jobs</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>nsf_awards</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>NSF REU Sites (computing and mathematics)</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>REU Site</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>Stanford Pre-Collegiate Studies jobs (SUMaC RC / TA)</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>https://spcs.stanford.edu/residential-program-positions</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23498,19 +23494,19 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>Added 2026-10-01. NSF's public Award Search API (api.nsf.gov, no robots.txt), keyword "REU Site", awards still funded on 1 August of the coming summer, kept to the CISE divisions (CCF, CNS, IIS, OAC) and DMS. 78 sites measured that day. A new award is a new summer research programme. www.nsf.gov/awardsearch/* is disallowed by robots.txt and is never fetched: the abstract arrives with the award.</t>
+          <t>Verified 2026-09-26: 200, 4,757 chars, ratio 0.128. | MANUAL 2026-09-30: never once fetched from the Actions runner (403 on every run since it was added) while answering a laptop 200 under the same User-Agent. spcs.stanford.edu is on Pantheon (live-spcs.pantheonsite.io), which refuses datacenter IPs. No second route: Stanford's central Oracle HCM board (careersearch.stanford.edu, reachable) carries 0 Pre-Collegiate requisitions, so SPCS posts only on its own site. Re-pointed at the residential page (SUMaC RC/TA), which on 2026-09-30 said Summer 2026 is filled and offers an interest form for the Summer 2027 cycle.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>8vc-portfolio-interns</t>
+          <t>thedeckgame</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>page_text</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
@@ -23520,19 +23516,15 @@
       </c>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>8VC portfolio internships (early-stage US)</t>
+          <t>The Deck Game</t>
         </is>
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.8vc.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://thedeckgame.com/</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23540,19 +23532,19 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>Getro collection 1005. 32 postings (Bedrock Robotics, General Matter, Matician). 12,004 chars, ratio 0.0336.</t>
+          <t>MANUAL. Verified: JS shell yielding ~28 characters; sitemap has only two URLs. Not worth a Playwright run - there is nothing to diff.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>a16z-portfolio-interns</t>
+          <t>usc-ict-summer</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>page_text</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="C92" s="2" t="inlineStr">
@@ -23562,19 +23554,15 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>a16z portfolio internships (seed/venture US)</t>
+          <t>USC ICT Summer Research Program</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.a16z.com/jobs?internshipsOnly=true&amp;stage=seed&amp;stage=venture&amp;location=country:us</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://ict.usc.edu/careers/internships/summer-research-program-application/</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -23582,19 +23570,19 @@
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>a16z's own Next.js board, server-rendered. 40 postings 2026-09-30 (Amca, Cowboy Space, Heron Power, Northwood Space, Ventrilo). 5,456 chars, ratio 0.0279. The size= param is ignored; stage= is honoured.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 762 characters of visible text, no JavaScript needed. | MANUAL 2026-10-08: never once fetched from the Actions runner (HTTP 403 on all six runs 2026-10-02..07) while answering a laptop HTTP 200 under the same User-Agent on 2026-10-08 (33 lines). The 2026-10-01 verification was made from a laptop, which is why it missed this. ict.usc.edu resolves to WP Engine (141.193.213.20/21, OrgName WPEngine), the same WAF that refused the runner for gtsx.com and twosigma.com; www.usc.edu is on Pantheon, which refused it for spcs-jobs, and no vendor-hosted listing was found. Surfaces as a January calendar reminder instead.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>ai2-internships</t>
+          <t>nsf-reu-sites</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>page_text</t>
+          <t>nsf_awards</t>
         </is>
       </c>
       <c r="C93" s="2" t="inlineStr">
@@ -23604,12 +23592,12 @@
       </c>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>Ai2 internships (Allen Institute for AI)</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>https://allenai.org/internships</t>
+          <t>NSF REU Sites (computing and mathematics)</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>REU Site</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -23624,14 +23612,14 @@
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 3659 characters of visible text, no JavaScript needed.</t>
+          <t>Added 2026-10-01. NSF's public Award Search API (api.nsf.gov, no robots.txt), keyword "REU Site", awards still funded on 1 August of the coming summer, kept to the CISE divisions (CCF, CNS, IIS, OAC) and DMS. 78 sites measured that day. A new award is a new summer research programme. www.nsf.gov/awardsearch/* is disallowed by robots.txt and is never fetched: the abstract arrives with the award.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>albatross-labs</t>
+          <t>8vc-portfolio-interns</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -23641,17 +23629,17 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Albatross Labs</t>
+          <t>8VC portfolio internships (early-stage US)</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>https://www.albatrosslabs.io/</t>
+          <t>https://jobs.8vc.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -23666,14 +23654,14 @@
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 2,390 chars, ratio 0.0055 - above the 0.0015 floor but the thinnest ratio on the watchlist. Advertises Software/Quant Developer at internship level.</t>
+          <t>Getro collection 1005. 32 postings (Bedrock Robotics, General Matter, Matician). 12,004 chars, ratio 0.0336.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>aspect-careers</t>
+          <t>a16z-portfolio-interns</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -23683,17 +23671,17 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>Aspect Capital</t>
+          <t>a16z portfolio internships (seed/venture US)</t>
         </is>
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>https://www.aspectcapital.com/careers/</t>
+          <t>https://jobs.a16z.com/jobs?internshipsOnly=true&amp;stage=seed&amp;stage=venture&amp;location=country:us</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -23708,14 +23696,14 @@
       </c>
       <c r="H95" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 8,724 chars of text.</t>
+          <t>a16z's own Next.js board, server-rendered. 40 postings 2026-09-30 (Amca, Cowboy Space, Heron Power, Northwood Space, Ventrilo). 5,456 chars, ratio 0.0279. The size= param is ignored; stage= is honoured.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>bam-internships</t>
+          <t>ai2-internships</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -23730,12 +23718,12 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Balyasny (BAM)</t>
+          <t>Ai2 internships (Allen Institute for AI)</t>
         </is>
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>https://www.bamfunds.com/careers/internships</t>
+          <t>https://allenai.org/internships</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -23750,14 +23738,14 @@
       </c>
       <c r="H96" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 3,394 chars. Programme page only: BAM's Salesforce ATS is a 60-character shell, so individual reqs are not reachable.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 3659 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>berkeley-superb</t>
+          <t>albatross-labs</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -23767,35 +23755,39 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
         <is>
-          <t>Berkeley SUPERB-AI4E REU</t>
+          <t>Albatross Labs</t>
         </is>
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>https://eecs.berkeley.edu/resources/undergrads/undergraduate-research/superb/</t>
-        </is>
-      </c>
-      <c r="F97" s="2" t="inlineStr"/>
+          <t>https://www.albatrosslabs.io/</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 8425 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-11: 2,390 chars, ratio 0.0055 - above the 0.0015 floor but the thinnest ratio on the watchlist. Advertises Software/Quant Developer at internship level.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>berkeley-trading-competition</t>
+          <t>aspect-careers</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
@@ -23805,17 +23797,17 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>Berkeley Trading Competition</t>
+          <t>Aspect Capital</t>
         </is>
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>https://traders.studentorg.berkeley.edu/competition/</t>
+          <t>https://www.aspectcapital.com/careers/</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -23830,14 +23822,14 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 3,041 chars, ratio 0.138. Page says applications 'not open yet'.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 8,724 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>bluefin-careers</t>
+          <t>bam-internships</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
@@ -23847,17 +23839,17 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
         <is>
-          <t>Bluefin Companies</t>
+          <t>Balyasny (BAM)</t>
         </is>
       </c>
       <c r="E99" s="3" t="inlineStr">
         <is>
-          <t>https://www.bfcm.com/careers/</t>
+          <t>https://www.bamfunds.com/careers/internships</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -23872,14 +23864,14 @@
       </c>
       <c r="H99" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 740 chars, close to the 500 floor. Renamed from Bluefin Trading; applications by email.</t>
+          <t>Verified 2026-09-11: 3,394 chars. Programme page only: BAM's Salesforce ATS is a 60-character shell, so individual reqs are not reachable.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>blueshift-careers</t>
+          <t>berkeley-trading-competition</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
@@ -23889,39 +23881,39 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
         <is>
-          <t>Blueshift Asset Management</t>
+          <t>Berkeley Trading Competition</t>
         </is>
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>https://www.blueshift.am/</t>
+          <t>https://traders.studentorg.berkeley.edu/competition/</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 5,636 chars. Quantitative Analyst (MS/PhD) only. Note blueshift.com is marketing SaaS.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 3,041 chars, ratio 0.138. Page says applications 'not open yet'.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>bny-pre-internship</t>
+          <t>bluefin-careers</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -23936,12 +23928,12 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>BNY Freshman Jumpstart</t>
+          <t>Bluefin Companies</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
         <is>
-          <t>https://www.bny.com/corporate/global/en/about-us/careers/students/pre-internship.html</t>
+          <t>https://www.bfcm.com/careers/</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -23956,14 +23948,14 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 200, 194,182 bytes, ~8.7k chars (ratio 0.045). Akamai edgekey; not yet measured from the runner.</t>
+          <t>Verified 2026-09-11: 740 chars, close to the 500 floor. Renamed from Bluefin Trading; applications by email.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>bofa-campus-events</t>
+          <t>blueshift-careers</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
@@ -23973,39 +23965,39 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
         <is>
-          <t>Bank of America campus events (Early Insights)</t>
+          <t>Blueshift Asset Management</t>
         </is>
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>https://bankcampuscareers.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.blueshift.am/</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 23,558 chars, ratio 0.669 (Atom feed).</t>
+          <t>Verified 2026-09-11: 5,636 chars. Quantitative Analyst (MS/PhD) only. Note blueshift.com is marketing SaaS.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>brevanhoward-students</t>
+          <t>bny-pre-internship</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
@@ -24015,17 +24007,17 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>Brevan Howard students</t>
+          <t>BNY Freshman Jumpstart</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
         <is>
-          <t>https://www.brevanhoward.com/students/</t>
+          <t>https://www.bny.com/corporate/global/en/about-us/careers/students/pre-internship.html</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -24040,14 +24032,14 @@
       </c>
       <c r="H103" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 2,375 chars of text.</t>
+          <t>Verified 2026-09-30: 200, 194,182 bytes, ~8.7k chars (ratio 0.045). Akamai edgekey; not yet measured from the runner.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>bridgewater-students</t>
+          <t>bofa-campus-events</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -24062,12 +24054,12 @@
       </c>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>Bridgewater students</t>
+          <t>Bank of America campus events (Early Insights)</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>https://www.bridgewater.com/working-at-bridgewater/students</t>
+          <t>https://bankcampuscareers.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -24082,14 +24074,14 @@
       </c>
       <c r="H104" s="2" t="inlineStr">
         <is>
-          <t>Students page. bridgewater.com/careers yields less (2,326). Verified 2026-09-11: 4,624 chars.</t>
+          <t>Verified 2026-09-26: 200, 23,558 chars, ratio 0.669 (Atom feed).</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>builtin-data-analytics</t>
+          <t>brevanhoward-students</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -24099,17 +24091,17 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>Built In data and analytics internships</t>
+          <t>Brevan Howard students</t>
         </is>
       </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/data-analytics/internship</t>
+          <t>https://www.brevanhoward.com/students/</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -24124,14 +24116,14 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 10785 characters of visible text.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 2,375 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>builtin-dev-engineering</t>
+          <t>bridgewater-students</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -24141,17 +24133,17 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>Built In software engineering internships</t>
+          <t>Bridgewater students</t>
         </is>
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/dev-engineering/internship</t>
+          <t>https://www.bridgewater.com/working-at-bridgewater/students</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -24166,14 +24158,14 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 14296 characters of visible text.</t>
+          <t>Students page. bridgewater.com/careers yields less (2,326). Verified 2026-09-11: 4,624 chars.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>builtin-finance</t>
+          <t>builtin-data-analytics</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -24188,12 +24180,12 @@
       </c>
       <c r="D107" s="2" t="inlineStr">
         <is>
-          <t>Built In finance internships</t>
+          <t>Built In data and analytics internships</t>
         </is>
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>https://builtin.com/jobs/finance/internship</t>
+          <t>https://builtin.com/jobs/data-analytics/internship</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -24208,14 +24200,14 @@
       </c>
       <c r="H107" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 12543 characters of visible text.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 10785 characters of visible text.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>calhacks</t>
+          <t>builtin-dev-engineering</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -24225,20 +24217,24 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
         <is>
-          <t>Cal Hacks</t>
+          <t>Built In software engineering internships</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>https://www.calhacks.io/</t>
-        </is>
-      </c>
-      <c r="F108" s="2" t="inlineStr"/>
+          <t>https://builtin.com/jobs/dev-engineering/internship</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24246,14 +24242,14 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 10,411 chars from 730KB (ratio 0.0142); calhacks.io redirects to www. FAQ states travel stipends for a limited number of hackers.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 14296 characters of visible text.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>caltech-surf</t>
+          <t>builtin-finance</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -24263,35 +24259,39 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
         <is>
-          <t>Caltech SURF</t>
+          <t>Built In finance internships</t>
         </is>
       </c>
       <c r="E109" s="3" t="inlineStr">
         <is>
-          <t>https://sfp.caltech.edu/undergraduate-research/programs/surf/application_information</t>
-        </is>
-      </c>
-      <c r="F109" s="2" t="inlineStr"/>
+          <t>https://builtin.com/jobs/finance/internship</t>
+        </is>
+      </c>
+      <c r="F109" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 9174 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 12543 characters of visible text.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>capitalone-early-career</t>
+          <t>calhacks</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -24301,24 +24301,20 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
         <is>
-          <t>Capital One Analyst / Tech / Product Summits</t>
+          <t>Cal Hacks</t>
         </is>
       </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
-        </is>
-      </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://www.calhacks.io/</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr"/>
       <c r="G110" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24326,14 +24322,14 @@
       </c>
       <c r="H110" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 11,506 chars, ratio 0.152.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 10,411 chars from 730KB (ratio 0.0142); calhacks.io redirects to www. FAQ states travel stipends for a limited number of hackers.</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>capula-workable</t>
+          <t>capitalone-early-career</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -24348,12 +24344,12 @@
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t>Capula Investment Management</t>
+          <t>Capital One Analyst / Tech / Product Summits</t>
         </is>
       </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/api/v1/widget/accounts/capula-investment-management-ltd</t>
+          <t>https://www.capitalonecareers.com/get-ahead-with-early-career-programs-for-students</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -24368,14 +24364,14 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: Workable JSON widget, 8,015 chars, ratio 0.997. Carries '2027 Trading and Research Summer Internship' and 'Technology Graduate Analyst'. Read as page_text because the tracker has no Workable parser; the feed is deterministic so a text diff is stable.</t>
+          <t>Verified 2026-09-26: 200, 11,506 chars, ratio 0.152.</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>cboe-careers</t>
+          <t>capula-workable</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -24385,17 +24381,17 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Cboe Global Markets</t>
+          <t>Capula Investment Management</t>
         </is>
       </c>
       <c r="E112" s="3" t="inlineStr">
         <is>
-          <t>https://careers.cboe.com/us/en</t>
+          <t>https://apply.workable.com/api/v1/widget/accounts/capula-investment-management-ltd</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -24410,14 +24406,14 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 4,717 chars of text.</t>
+          <t>Verified 2026-09-11: Workable JSON widget, 8,015 chars, ratio 0.997. Carries '2027 Trading and Research Summer Internship' and 'Technology Graduate Analyst'. Read as page_text because the tracker has no Workable parser; the feed is deterministic so a text diff is stable.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>cerebralvalley-sf-events</t>
+          <t>cboe-careers</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -24427,20 +24423,24 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t>Cerebral Valley SF &amp; Bay Area AI events calendar</t>
+          <t>Cboe Global Markets</t>
         </is>
       </c>
       <c r="E113" s="3" t="inlineStr">
         <is>
-          <t>https://cerebralvalley.ai/events/san-francisco</t>
-        </is>
-      </c>
-      <c r="F113" s="2" t="inlineStr"/>
+          <t>https://careers.cboe.com/us/en</t>
+        </is>
+      </c>
+      <c r="F113" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G113" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24448,14 +24448,14 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 10,770 chars from 342KB (ratio 0.0315); robots.txt allows /events/. The ?type=hackathon filter is applied client-side (the server returns the same mixed list), so the unfiltered city page is watched. Expect daily churn as past events drop off.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 4,717 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>citi-pre-internships</t>
+          <t>cerebralvalley-sf-events</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -24470,19 +24470,15 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Citi Freshman Discovery</t>
+          <t>Cerebral Valley SF &amp; Bay Area AI events calendar</t>
         </is>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
-        </is>
-      </c>
-      <c r="F114" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://cerebralvalley.ai/events/san-francisco</t>
+        </is>
+      </c>
+      <c r="F114" s="2" t="inlineStr"/>
       <c r="G114" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24490,14 +24486,14 @@
       </c>
       <c r="H114" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 200, 98,648 bytes, ~8.2k chars. TalentBrew vendor host (jobs-citi-com.talentbrew.com). Complements citi-early-careers-workday, which has no Freshman rows today.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 10,987 chars over 143 lines from 342KB (ratio 0.032, measured by run.py --only); robots.txt allows /events/. The ?type=hackathon filter is applied client-side (the server returns the same mixed list), so the unfiltered city page is watched. Expect daily churn as past events drop off.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>cmu-riss</t>
+          <t>citi-pre-internships</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -24507,17 +24503,17 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
         <is>
-          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
+          <t>Citi Freshman Discovery</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
         <is>
-          <t>https://riss.ri.cmu.edu/</t>
+          <t>https://jobs.citi.com/early-career-programs-pre-internships</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -24532,14 +24528,14 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 2556 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-30: 200, 98,648 bytes, ~8.2k chars. TalentBrew vendor host (jobs-citi-com.talentbrew.com). Complements citi-early-careers-workday, which has no Freshman rows today.</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>comap-mcm</t>
+          <t>cmu-riss</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -24549,17 +24545,17 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>COMAP MCM/ICM</t>
+          <t>CMU Robotics Institute Summer Scholars (RISS)</t>
         </is>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/undergraduate/contests/</t>
+          <t>https://riss.ri.cmu.edu/</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -24574,14 +24570,14 @@
       </c>
       <c r="H116" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 7,350 chars, ratio 0.391. robots.txt not determinable.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 2556 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>cornell-trading-competition</t>
+          <t>comap-mcm</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
@@ -24591,17 +24587,17 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>Cornell Trading Competition</t>
+          <t>COMAP MCM/ICM</t>
         </is>
       </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>https://cornellquantfund.org/competition</t>
+          <t>https://www.contest.comap.com/undergraduate/contests/</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -24616,14 +24612,14 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,188 chars, ratio 0.142.</t>
+          <t>Verified 2026-09-26: 200, 7,350 chars, ratio 0.391. robots.txt not determinable.</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>cra-dreu</t>
+          <t>cornell-trading-competition</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -24633,17 +24629,17 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>CRA DREU</t>
+          <t>Cornell Trading Competition</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>https://cra.org/cra-wp/dreu/</t>
+          <t>https://cornellquantfund.org/competition</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -24658,14 +24654,14 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 94,045 chars, ratio 0.249.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,188 chars, ratio 0.142.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>cs-social-good-fellowships</t>
+          <t>cra-dreu</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -24675,17 +24671,17 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
         <is>
-          <t>CS+Social Good Summer Fellowships</t>
+          <t>CRA DREU</t>
         </is>
       </c>
       <c r="E119" s="3" t="inlineStr">
         <is>
-          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
+          <t>https://cra.org/cra-wp/dreu/</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -24700,14 +24696,14 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 200, 37,530 bytes, ~2.8k chars. Stanford Akamai host like the watched curis/surim rows.</t>
+          <t>Verified 2026-09-26: 200, 94,045 chars, ratio 0.249.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>curis</t>
+          <t>cs-social-good-fellowships</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -24722,12 +24718,12 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Stanford CURIS</t>
+          <t>CS+Social Good Summer Fellowships</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
         <is>
-          <t>https://curis.stanford.edu/</t>
+          <t>https://cardinalservice.stanford.edu/opportunities/cssocial-good-summer-fellowships</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -24742,14 +24738,14 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: render_js: 5 chars plain, 1,264 rendered.</t>
+          <t>Verified 2026-09-30: 200, 37,530 bytes, ~2.8k chars. Stanford Akamai host like the watched curis/surim rows.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>datasurf</t>
+          <t>curis</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -24764,12 +24760,12 @@
       </c>
       <c r="D121" s="2" t="inlineStr">
         <is>
-          <t>Stanford DataSURF</t>
+          <t>Stanford CURIS</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
+          <t>https://curis.stanford.edu/</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -24784,14 +24780,14 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 200, 56,385 bytes. Stanford Akamai host.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: render_js: 5 chars plain, 1,264 rendered.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>deshaw-campus</t>
+          <t>datasurf</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -24806,12 +24802,12 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>D. E. Shaw campus site</t>
+          <t>Stanford DataSURF</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
         <is>
-          <t>https://campus.deshaw.com/</t>
+          <t>https://datasciencemajor.stanford.edu/research-impact/data-science-undergraduate-research-focus</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -24826,14 +24822,14 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 10,795 chars, ratio 0.114.</t>
+          <t>Verified 2026-09-30: 200, 56,385 bytes. Stanford Akamai host.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>deshaw-careers</t>
+          <t>deshaw-campus</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -24848,12 +24844,12 @@
       </c>
       <c r="D123" s="2" t="inlineStr">
         <is>
-          <t>D. E. Shaw</t>
+          <t>D. E. Shaw campus site</t>
         </is>
       </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
-          <t>https://www.deshaw.com/careers</t>
+          <t>https://campus.deshaw.com/</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -24868,14 +24864,14 @@
       </c>
       <c r="H123" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 36,840 chars of text. deshaw.com/careers/students renders nothing (0 chars); /careers is the readable one.</t>
+          <t>Verified 2026-09-26: 200, 10,795 chars, ratio 0.114.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>dimacs-reu</t>
+          <t>deshaw-careers</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -24885,17 +24881,17 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>DIMACS REU</t>
+          <t>D. E. Shaw</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>https://dimacs.rutgers.edu/reu-main</t>
+          <t>https://www.deshaw.com/careers</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -24910,14 +24906,14 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 2,928 chars, ratio 0.072.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 36,840 chars of text. deshaw.com/careers/students renders nothing (0 chars); /careers is the readable one.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>dukequant-competition</t>
+          <t>dimacs-reu</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -24927,17 +24923,17 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>Duke FinTech Trading Competition</t>
+          <t>DIMACS REU</t>
         </is>
       </c>
       <c r="E125" s="3" t="inlineStr">
         <is>
-          <t>https://www.dukequant.com/general-7</t>
+          <t>https://dimacs.rutgers.edu/reu-main</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -24952,14 +24948,14 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: render_js: Wix site, 942 chars at ratio 0.001 on every page plain; 965 rendered. 'Applications due January 25, 2026'.</t>
+          <t>Verified 2026-09-26: 200, 2,928 chars, ratio 0.072.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>eagleseven-careers</t>
+          <t>dukequant-competition</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -24969,17 +24965,17 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>Eagle Seven</t>
+          <t>Duke FinTech Trading Competition</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>https://www.eagleseven.com/</t>
+          <t>https://www.dukequant.com/general-7</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -24994,14 +24990,14 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 15,784 chars. 'Junior Trader' is the most junior role today. CORRECTED 2026-09-12: the 'no public ATS' claim above is false -- eagleseven-workable watches the real board, found by a domain-anchored fingerprint probe. This page_text row is kept because the page may still carry programme detail the board rows do not state; retire it if it proves redundant.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: render_js: Wix site, 942 chars at ratio 0.001 on every page plain; 965 rendered. 'Applications due January 25, 2026'.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>eagleseven-workable</t>
+          <t>eagleseven-careers</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -25014,10 +25010,14 @@
           <t>low</t>
         </is>
       </c>
-      <c r="D127" s="2" t="inlineStr"/>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>Eagle Seven</t>
+        </is>
+      </c>
       <c r="E127" s="3" t="inlineStr">
         <is>
-          <t>https://apply.workable.com/api/v1/widget/accounts/eagle-seven</t>
+          <t>https://www.eagleseven.com/</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -25032,14 +25032,14 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>Added 2026-09-12 by the audit that followed a manual finding that watched careers pages were not the real job boards. The eagleseven-careers row's note claimed the firm was on no public ATS; it is not true. 5 postings. Watched as page_text on the Workable widget JSON, the same shape as the existing capula-workable row, because there is no workable method.</t>
+          <t>Verified 2026-09-11: 15,784 chars. 'Junior Trader' is the most junior role today. CORRECTED 2026-09-12: the 'no public ATS' claim above is false -- eagleseven-workable watches the real board, found by a domain-anchored fingerprint probe. This page_text row is kept because the page may still carry programme detail the board rows do not state; retire it if it proves redundant.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>edgehog-rippling</t>
+          <t>eagleseven-workable</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -25049,17 +25049,13 @@
       </c>
       <c r="C128" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="D128" s="2" t="inlineStr">
-        <is>
-          <t>Edgehog Trading</t>
-        </is>
-      </c>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr"/>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>https://api.rippling.com/platform/api/ats/v1/board/edgehog-trading/jobs</t>
+          <t>https://apply.workable.com/api/v1/widget/accounts/eagle-seven</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -25074,14 +25070,14 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: Rippling ATS JSON, 14 jobs, 3,171 chars, ratio 0.79. Graduate Quant Trader, Graduate SWE, Junior FPGA Developer.</t>
+          <t>Added 2026-09-12 by the audit that followed a manual finding that watched careers pages were not the real job boards. The eagleseven-careers row's note claimed the firm was on no public ATS; it is not true. 5 postings. Watched as page_text on the Workable widget JSON, the same shape as the existing capula-workable row, because there is no workable method.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>eschaton-careers</t>
+          <t>edgehog-rippling</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -25096,12 +25092,12 @@
       </c>
       <c r="D129" s="2" t="inlineStr">
         <is>
-          <t>Eschaton Trading</t>
+          <t>Edgehog Trading</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>https://www.eschatontrading.com/careers</t>
+          <t>https://api.rippling.com/platform/api/ats/v1/board/edgehog-trading/jobs</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -25116,14 +25112,14 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 2,184 chars of text.</t>
+          <t>Verified 2026-09-11: Rippling ATS JSON, 14 jobs, 3,171 chars, ratio 0.79. Graduate Quant Trader, Graduate SWE, Junior FPGA Developer.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>evercore-campus</t>
+          <t>eschaton-careers</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -25133,17 +25129,17 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D130" s="2" t="inlineStr">
         <is>
-          <t>Evercore student events</t>
+          <t>Eschaton Trading</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.eschatontrading.com/careers</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -25158,14 +25154,14 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 17,150 chars, ratio 0.40 (Atom feed).</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 2,184 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>felicis-portfolio-interns</t>
+          <t>evercore-campus</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -25175,17 +25171,17 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D131" s="2" t="inlineStr">
         <is>
-          <t>Felicis portfolio internships (&lt;100 staff)</t>
+          <t>Evercore student events</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.felicis.com/jobs?internshipOnly=true&amp;stages=10-100+employees&amp;stages=1-10+employees</t>
+          <t>https://evercore.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -25200,14 +25196,14 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>Consider board 'felicis'. 21 postings via API 2026-09-30. Rendered with the same params as the Lightspeed row, which was verified to honour them.</t>
+          <t>Verified 2026-09-26: 200, 17,150 chars, ratio 0.40 (Atom feed).</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>futureforce-launchpad</t>
+          <t>felicis-portfolio-interns</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -25222,12 +25218,12 @@
       </c>
       <c r="D132" s="2" t="inlineStr">
         <is>
-          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
+          <t>Felicis portfolio internships (&lt;100 staff)</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
+          <t>https://jobs.felicis.com/jobs?internshipOnly=true&amp;stages=10-100+employees&amp;stages=1-10+employees</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -25242,14 +25238,14 @@
       </c>
       <c r="H132" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 7,896 chars, ratio 0.071.</t>
+          <t>Consider board 'felicis'. 21 postings via API 2026-09-30. Rendered with the same params as the Lightspeed row, which was verified to honour them.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>garda-careers</t>
+          <t>futureforce-launchpad</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -25259,17 +25255,17 @@
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D133" s="2" t="inlineStr">
         <is>
-          <t>Garda Capital Partners</t>
+          <t>Salesforce Futureforce Tech Launchpad (CodePath)</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>https://www.gardacp.com/careers/</t>
+          <t>https://info.codepath.org/futureforce-tech-launchpad</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -25284,14 +25280,14 @@
       </c>
       <c r="H133" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 5,287 chars. Six internships live, including SWE Intern (NY) and Trading Analyst Intern across Credit/Mortgages/Rates.</t>
+          <t>Verified 2026-09-26: 200, 7,896 chars, ratio 0.071.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>generalcatalyst-portfolio-interns</t>
+          <t>garda-careers</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
@@ -25306,12 +25302,12 @@
       </c>
       <c r="D134" s="2" t="inlineStr">
         <is>
-          <t>General Catalyst portfolio internships (early-stage US)</t>
+          <t>Garda Capital Partners</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.generalcatalyst.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
+          <t>https://www.gardacp.com/careers/</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -25326,14 +25322,14 @@
       </c>
       <c r="H134" s="2" t="inlineStr">
         <is>
-          <t>Getro collection 222. 35 postings 2026-09-30 (Nominal, Pacific Fusion, Pylon, Eudia, Vital Lyfe, General Intuition). 11,782 chars, ratio 0.0158.</t>
+          <t>Verified 2026-09-11: 5,287 chars. Six internships live, including SWE Intern (NY) and Trading Analyst Intern across Credit/Mortgages/Rates.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>gresearch-careers</t>
+          <t>generalcatalyst-portfolio-interns</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -25348,12 +25344,12 @@
       </c>
       <c r="D135" s="2" t="inlineStr">
         <is>
-          <t>G-Research</t>
+          <t>General Catalyst portfolio internships (early-stage US)</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
         <is>
-          <t>https://www.gresearch.com/careers/</t>
+          <t>https://jobs.generalcatalyst.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -25368,14 +25364,14 @@
       </c>
       <c r="H135" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 1,801 chars of text.</t>
+          <t>Getro collection 222. 35 postings 2026-09-30 (Nominal, Pacific Fusion, Pylon, Eudia, Vital Lyfe, General Intuition). 11,782 chars, ratio 0.0158.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>group1-careers</t>
+          <t>gresearch-careers</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -25390,12 +25386,12 @@
       </c>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>Group One Trading</t>
+          <t>G-Research</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>https://group1.com/careers/</t>
+          <t>https://www.gresearch.com/careers/</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -25410,14 +25406,14 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 3,990 chars. Trading Analyst Intern and Software Developer Intern. Also advertises a STANFORD CAREER FAIR on 6 Oct 2026 - see calendar_reminders.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 1,801 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>gts-careers</t>
+          <t>group1-careers</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
@@ -25432,12 +25428,12 @@
       </c>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>GTS</t>
+          <t>Group One Trading</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
         <is>
-          <t>https://careers-gtsx.icims.com/jobs/search?ss=1&amp;in_iframe=1</t>
+          <t>https://group1.com/careers/</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -25452,14 +25448,14 @@
       </c>
       <c r="H137" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 18,734 chars of text. Correction 2026-09-16: "no public ATS" was false. GTS is on iCIMS at careers-gtsx.icims.com, linked from the careers page as a button; the project does not fingerprint iCIMS, so the discovery probe never saw it. Re-pointed at the board itself, which is vendor-hosted (CNAME wildcard.cloud.icims.tools) and so outside the WAF that was returning 403 to the Actions runner on gtsx.com. The in_iframe=1 parameter is load-bearing: without it the response is the WordPress wrapper, 2,877 chars at ratio 0.017. With it, 10,156 chars at 0.241, including "Quantitative Trader - 2027 Graduates".</t>
+          <t>Verified 2026-09-11: 3,990 chars. Trading Analyst Intern and Software Developer Intern. Also advertises a STANFORD CAREER FAIR on 6 Oct 2026 - see calendar_reminders.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>hackgt</t>
+          <t>gts-careers</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
@@ -25469,20 +25465,24 @@
       </c>
       <c r="C138" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>HackGT</t>
+          <t>GTS</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
         <is>
-          <t>https://hack.gt/</t>
-        </is>
-      </c>
-      <c r="F138" s="2" t="inlineStr"/>
+          <t>https://careers-gtsx.icims.com/jobs/search?ss=1&amp;in_iframe=1</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25490,14 +25490,14 @@
       </c>
       <c r="H138" s="2" t="inlineStr">
         <is>
-          <t>render_js: verified 2026-10-08 through gather.browser, 5,650 chars rendered; plain HTTP yields 9 chars from 1.2KB. States travel reimbursement.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 18,734 chars of text. Correction 2026-09-16: "no public ATS" was false. GTS is on iCIMS at careers-gtsx.icims.com, linked from the careers page as a button; the project does not fingerprint iCIMS, so the discovery probe never saw it. Re-pointed at the board itself, which is vendor-hosted (CNAME wildcard.cloud.icims.tools) and so outside the WAF that was returning 403 to the Actions runner on gtsx.com. The in_iframe=1 parameter is load-bearing: without it the response is the WordPress wrapper, 2,877 chars at ratio 0.017. With it, 10,156 chars at 0.241, including "Quantitative Trader - 2027 Graduates".</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>hackprinceton</t>
+          <t>hackgt</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
@@ -25512,12 +25512,12 @@
       </c>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>HackPrinceton</t>
+          <t>HackGT</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
         <is>
-          <t>https://www.hackprinceton.com/</t>
+          <t>https://hack.gt/</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr"/>
@@ -25528,14 +25528,14 @@
       </c>
       <c r="H139" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,959 chars from 305KB (ratio 0.0130). FAQ states partial travel stipends for some admitted hackers.</t>
+          <t>render_js: verified 2026-10-08 through gather.browser, 5,650 chars rendered; plain HTTP yields 9 chars from 1.2KB. States travel reimbursement.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>hackumass</t>
+          <t>hackprinceton</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
@@ -25550,12 +25550,12 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>HackUMass</t>
+          <t>HackPrinceton</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>https://www.hackumass.com/</t>
+          <t>https://www.hackprinceton.com/</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr"/>
@@ -25566,14 +25566,14 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 9,237 chars from 44KB (ratio 0.21); hackumass.com redirects to www. States travel reimbursement for early applicants.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,959 chars from 305KB (ratio 0.0130). FAQ states partial travel stipends for some admitted hackers.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>harvard-undergraduate-trading</t>
+          <t>hackumass</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
@@ -25583,24 +25583,20 @@
       </c>
       <c r="C141" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
         <is>
-          <t>Harvard Undergraduate Trading Competition</t>
+          <t>HackUMass</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>https://www.huqt.com/</t>
-        </is>
-      </c>
-      <c r="F141" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://www.hackumass.com/</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr"/>
       <c r="G141" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25608,14 +25604,14 @@
       </c>
       <c r="H141" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 1654 chars of text over plain HTTP, no robots.txt. Use huqt.com - the article's harvarduqt.com/competition redirects to a 404.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 9,237 chars from 44KB (ratio 0.21); hackumass.com redirects to www. States travel reimbursement for early applicants.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>hedgewest-sf-meetup-series</t>
+          <t>harvard-undergraduate-trading</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
@@ -25630,12 +25626,12 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>HedgeWest SF Meetup Series</t>
+          <t>Harvard Undergraduate Trading Competition</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>https://hedgewestsf.org/</t>
+          <t>https://www.huqt.com/</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -25650,14 +25646,14 @@
       </c>
       <c r="H142" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 837 chars of text over plain HTTP.</t>
+          <t>Probed 2026-09-06: 200, 1654 chars of text over plain HTTP, no robots.txt. Use huqt.com - the article's harvarduqt.com/competition redirects to a 404.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>hophacks</t>
+          <t>hedgewest-sf-meetup-series</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
@@ -25667,20 +25663,24 @@
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
         <is>
-          <t>HopHacks</t>
+          <t>HedgeWest SF Meetup Series</t>
         </is>
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>https://hophacks.com/</t>
-        </is>
-      </c>
-      <c r="F143" s="2" t="inlineStr"/>
+          <t>https://hedgewestsf.org/</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25688,14 +25688,14 @@
       </c>
       <c r="H143" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 8,684 chars from 159KB (ratio 0.055). No individual travel reimbursement; possible free buses by city.</t>
+          <t>Probed 2026-09-06: 200, 837 chars of text over plain HTTP.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>iaqf-academic-paper-competition</t>
+          <t>hophacks</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -25705,39 +25705,35 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>IAQF Academic Paper Competition</t>
+          <t>HopHacks</t>
         </is>
       </c>
       <c r="E144" s="3" t="inlineStr">
         <is>
-          <t>https://www.iaqf.org/upcoming-events</t>
-        </is>
-      </c>
-      <c r="F144" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-06T14:25:47+00:00</t>
-        </is>
-      </c>
+          <t>https://hophacks.com/</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr"/>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 8194 chars of text over plain HTTP.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 8,684 chars from 159KB (ratio 0.055). No individual travel reimbursement; possible free buses by city.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>icerm-summer</t>
+          <t>iaqf-academic-paper-competition</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
@@ -25752,34 +25748,34 @@
       </c>
       <c r="D145" s="2" t="inlineStr">
         <is>
-          <t>Summer@ICERM</t>
+          <t>IAQF Academic Paper Competition</t>
         </is>
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>https://icerm.brown.edu/summerug/</t>
+          <t>https://www.iaqf.org/upcoming-events</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-06T14:25:47+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 8,350 chars, ratio 0.06.</t>
+          <t>Probed 2026-09-06: 200, 8194 chars of text over plain HTTP.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>icpc-pnw</t>
+          <t>icerm-summer</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -25794,12 +25790,12 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>ICPC</t>
+          <t>Summer@ICERM</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>https://pnw.na.icpc.global/</t>
+          <t>https://icerm.brown.edu/summerug/</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -25814,14 +25810,14 @@
       </c>
       <c r="H146" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 2,213 chars, ratio 0.009. Stanford's region; registration Sep 15 - Nov 5 2026, contest Nov 14.</t>
+          <t>Verified 2026-09-26: 200, 8,350 chars, ratio 0.06.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>imc-launchpad-us</t>
+          <t>icpc-pnw</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -25836,12 +25832,12 @@
       </c>
       <c r="D147" s="2" t="inlineStr">
         <is>
-          <t>IMC Launchpad (US)</t>
+          <t>ICPC</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
         <is>
-          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
+          <t>https://pnw.na.icpc.global/</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -25856,14 +25852,14 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 2450 chars of text over plain HTTP.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 2,213 chars, ratio 0.009. Stanford's region; registration Sep 15 - Nov 5 2026, contest Nov 14.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>imc-prosperity</t>
+          <t>imc-launchpad-us</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -25878,12 +25874,12 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t>IMC Prosperity Trading Competition</t>
+          <t>IMC Launchpad (US)</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>https://prosperity.imc.com/</t>
+          <t>https://www.imc.com/us/careers/students-graduates/programs/launchpad</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
@@ -25898,14 +25894,14 @@
       </c>
       <c r="H148" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 11,458 chars, ratio 0.025.</t>
+          <t>Probed 2026-09-06: 200, 2450 chars of text over plain HTTP.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>ipam-rips</t>
+          <t>imc-prosperity</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
@@ -25920,12 +25916,12 @@
       </c>
       <c r="D149" s="2" t="inlineStr">
         <is>
-          <t>IPAM RIPS (UCLA)</t>
+          <t>IMC Prosperity Trading Competition</t>
         </is>
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
+          <t>https://prosperity.imc.com/</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -25940,14 +25936,14 @@
       </c>
       <c r="H149" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 3609 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 11,458 chars, ratio 0.025.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>janestreet-bridge</t>
+          <t>ipam-rips</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -25962,12 +25958,12 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t>Jane Street Bridge</t>
+          <t>IPAM RIPS (UCLA)</t>
         </is>
       </c>
       <c r="E150" s="3" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/bridge/</t>
+          <t>https://www.ipam.ucla.edu/programs/student-research-programs/</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
@@ -25982,14 +25978,14 @@
       </c>
       <c r="H150" s="2" t="inlineStr">
         <is>
-          <t>Programme page for first- and second-years. Verified 2026-09-11: 4,111 chars.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 3609 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>janestreet-fttp</t>
+          <t>janestreet-bridge</t>
         </is>
       </c>
       <c r="B151" s="2" t="inlineStr">
@@ -26004,12 +26000,12 @@
       </c>
       <c r="D151" s="2" t="inlineStr">
         <is>
-          <t>Jane Street FTTP</t>
+          <t>Jane Street Bridge</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/bridge/</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -26024,14 +26020,14 @@
       </c>
       <c r="H151" s="2" t="inlineStr">
         <is>
-          <t>Programme page, not the board. Jane Street's Greenhouse board has no FTTP listing at all, and this page carries the apply button. Rolling review. Verified 2026-09-11: 3,393 chars.</t>
+          <t>Programme page for first- and second-years. Verified 2026-09-11: 4,111 chars.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>janestreet-insight</t>
+          <t>janestreet-fttp</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
@@ -26046,12 +26042,12 @@
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Jane Street INSIGHT</t>
+          <t>Jane Street FTTP</t>
         </is>
       </c>
       <c r="E152" s="3" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/fttp/</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
@@ -26066,14 +26062,14 @@
       </c>
       <c r="H152" s="2" t="inlineStr">
         <is>
-          <t>Programme page for INSIGHT, Jane Street's first-year programme. Verified 2026-09-11: 4,780 chars.</t>
+          <t>Programme page, not the board. Jane Street's Greenhouse board has no FTTP listing at all, and this page carries the apply button. Rolling review. Verified 2026-09-11: 3,393 chars.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>janestreet-preview</t>
+          <t>janestreet-insight</t>
         </is>
       </c>
       <c r="B153" s="2" t="inlineStr">
@@ -26088,12 +26084,12 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Jane Street Preview</t>
+          <t>Jane Street INSIGHT</t>
         </is>
       </c>
       <c r="E153" s="3" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/insight/</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -26108,14 +26104,14 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 with add_opportunity --probe: 200, 3,079 chars, ratio 0.084.</t>
+          <t>Programme page for INSIGHT, Jane Street's first-year programme. Verified 2026-09-11: 4,780 chars.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
-          <t>janestreet-programs</t>
+          <t>janestreet-preview</t>
         </is>
       </c>
       <c r="B154" s="2" t="inlineStr">
@@ -26130,12 +26126,12 @@
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Jane Street programs and events</t>
+          <t>Jane Street Preview</t>
         </is>
       </c>
       <c r="E154" s="3" t="inlineStr">
         <is>
-          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/preview/</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -26150,14 +26146,14 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>Index of every Jane Street programme; catches a new one appearing. Verified 2026-09-11: 5,997 chars.</t>
+          <t>Verified 2026-09-26 with add_opportunity --probe: 200, 3,079 chars, ratio 0.084.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
         <is>
-          <t>jefferies-campus</t>
+          <t>janestreet-programs</t>
         </is>
       </c>
       <c r="B155" s="2" t="inlineStr">
@@ -26167,17 +26163,17 @@
       </c>
       <c r="C155" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
         <is>
-          <t>Jefferies campus opportunities</t>
+          <t>Jane Street programs and events</t>
         </is>
       </c>
       <c r="E155" s="3" t="inlineStr">
         <is>
-          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
+          <t>https://www.janestreet.com/join-jane-street/programs-and-events/</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -26192,14 +26188,14 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 22,043 chars, ratio 0.369 (Atom feed).</t>
+          <t>Index of every Jane Street programme; catches a new one appearing. Verified 2026-09-11: 5,997 chars.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
         <is>
-          <t>jhuapl-internships</t>
+          <t>jefferies-campus</t>
         </is>
       </c>
       <c r="B156" s="2" t="inlineStr">
@@ -26209,17 +26205,17 @@
       </c>
       <c r="C156" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
         <is>
-          <t>Johns Hopkins APL internships</t>
+          <t>Jefferies campus opportunities</t>
         </is>
       </c>
       <c r="E156" s="3" t="inlineStr">
         <is>
-          <t>https://www.jhuapl.edu/careers/internships</t>
+          <t>https://jefferies.tal.net/vx/mobile-0/candidate/jobboard/vacancy/2/feed</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -26234,14 +26230,14 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 12419 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-26: 200, 22,043 chars, ratio 0.369 (Atom feed).</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
         <is>
-          <t>jpmc-career-edyou</t>
+          <t>jhuapl-internships</t>
         </is>
       </c>
       <c r="B157" s="2" t="inlineStr">
@@ -26251,17 +26247,17 @@
       </c>
       <c r="C157" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
         <is>
-          <t>JPMorganChase Career.edYOU Academy</t>
+          <t>Johns Hopkins APL internships</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
+          <t>https://www.jhuapl.edu/careers/internships</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -26276,14 +26272,14 @@
       </c>
       <c r="H157" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 10,788 chars, ratio 0.089.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 12419 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
         <is>
-          <t>jpmc-fellowship</t>
+          <t>jpmc-career-edyou</t>
         </is>
       </c>
       <c r="B158" s="2" t="inlineStr">
@@ -26298,12 +26294,12 @@
       </c>
       <c r="D158" s="2" t="inlineStr">
         <is>
-          <t>JPMC Fellowship Program</t>
+          <t>JPMorganChase Career.edYOU Academy</t>
         </is>
       </c>
       <c r="E158" s="3" t="inlineStr">
         <is>
-          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/career-edyou</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -26318,14 +26314,14 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 6,062 chars, ratio 0.054.</t>
+          <t>Verified 2026-09-26: 200, 10,788 chars, ratio 0.089.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
         <is>
-          <t>kore-careers</t>
+          <t>jpmc-fellowship</t>
         </is>
       </c>
       <c r="B159" s="2" t="inlineStr">
@@ -26340,12 +26336,12 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>Kore Trading</t>
+          <t>JPMC Fellowship Program</t>
         </is>
       </c>
       <c r="E159" s="3" t="inlineStr">
         <is>
-          <t>https://www.koretrading.com/front-page/careers/</t>
+          <t>https://www.jpmorganchase.com/careers/explore-opportunities/programs/jpmcfellowship</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -26360,14 +26356,14 @@
       </c>
       <c r="H159" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 1,485 chars of text.</t>
+          <t>Verified 2026-09-26: 200, 6,062 chars, ratio 0.054.</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
         <is>
-          <t>lahacks</t>
+          <t>kore-careers</t>
         </is>
       </c>
       <c r="B160" s="2" t="inlineStr">
@@ -26382,15 +26378,19 @@
       </c>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>LA Hacks</t>
+          <t>Kore Trading</t>
         </is>
       </c>
       <c r="E160" s="3" t="inlineStr">
         <is>
-          <t>https://www.lahacks.com/</t>
-        </is>
-      </c>
-      <c r="F160" s="2" t="inlineStr"/>
+          <t>https://www.koretrading.com/front-page/careers/</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26398,14 +26398,14 @@
       </c>
       <c r="H160" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 8,651 chars from 350KB (ratio 0.0247); lahacks.com redirects to www. Has a Travel Reimbursement FAQ tab whose answer is not in the HTML.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 1,485 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>lanl-students</t>
+          <t>lahacks</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -26415,35 +26415,35 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>LANL student internships (Los Alamos National Laboratory)</t>
+          <t>LA Hacks</t>
         </is>
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>https://www.lanl.gov/engage/collaboration/internships</t>
+          <t>https://www.lahacks.com/</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 1572 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 8,651 chars from 350KB (ratio 0.0247); lahacks.com redirects to www. Has a Travel Reimbursement FAQ tab whose answer is not in the HTML.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
         <is>
-          <t>lightspeed-portfolio-interns</t>
+          <t>lanl-students</t>
         </is>
       </c>
       <c r="B162" s="2" t="inlineStr">
@@ -26458,19 +26458,15 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Lightspeed portfolio internships (&lt;100 staff)</t>
+          <t>LANL student internships (Los Alamos National Laboratory)</t>
         </is>
       </c>
       <c r="E162" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.lsvp.com/jobs?internshipOnly=true&amp;stages=10-100+employees&amp;stages=1-10+employees</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://lanl.jobs/search/searchjobs?categoryid=7f2fb73c-b4e4-4644-a234-858a80163473</t>
+        </is>
+      </c>
+      <c r="F162" s="2" t="inlineStr"/>
       <c r="G162" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26478,14 +26474,14 @@
       </c>
       <c r="H162" s="2" t="inlineStr">
         <is>
-          <t>Consider board 'lightspeed'. Plain GET is a 21KB JS shell, so render_js is required. Rendered 2026-09-30: '38 jobs', 6,310 chars, ratio 0.071. Amca, K2 Space, Composio, Periodic Labs, Skild AI.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 1572 characters of visible text, no JavaScript needed. | 2026-10-08: url was https://www.lanl.gov/engage/collaboration/internships, now LANL's Undergraduate Internships category on lanl.jobs, because www.lanl.gov (CloudFront, d24zmp7uf2gm1q.cloudfront.net) answered HTTP 404 to the Actions runner on all six runs 2026-10-02..07 while answering a laptop HTTP 200 under the same User-Agent on 2026-10-08, so the source never once succeeded. lanl.jobs is LANL's own job board (linked from its Students and Postdocs page), on Azure Front Door, robots.txt allows all. The results render in JavaScript (1,534 characters plain), so render_js=true: rendered 2026-10-08 it lists 12 of 19 undergraduate postings, newest first, and two renders were identical. A newest-12 watcher, not a full list. Failure count reset: the six failures were the old URL's.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>llnl-students</t>
+          <t>lightspeed-portfolio-interns</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -26500,12 +26496,12 @@
       </c>
       <c r="D163" s="2" t="inlineStr">
         <is>
-          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
+          <t>Lightspeed portfolio internships (&lt;100 staff)</t>
         </is>
       </c>
       <c r="E163" s="3" t="inlineStr">
         <is>
-          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
+          <t>https://jobs.lsvp.com/jobs?internshipOnly=true&amp;stages=10-100+employees&amp;stages=1-10+employees</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -26520,14 +26516,14 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 13831 characters of visible text, no JavaScript needed.</t>
+          <t>Consider board 'lightspeed'. Plain GET is a 21KB JS shell, so render_js is required. Rendered 2026-09-30: '38 jobs', 6,310 chars, ratio 0.071. Amca, K2 Space, Composio, Periodic Labs, Skild AI.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>lynx-teamtailor</t>
+          <t>llnl-students</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -26537,17 +26533,17 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Lynx Asset Management</t>
+          <t>LLNL student internships (Lawrence Livermore National Laboratory)</t>
         </is>
       </c>
       <c r="E164" s="3" t="inlineStr">
         <is>
-          <t>https://careers.lynxhedge.se/jobs.json</t>
+          <t>https://www.llnl.gov/join-our-team/careers/student-internship-veteran-programs</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -26562,14 +26558,14 @@
       </c>
       <c r="H164" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: Teamtailor JSON feed, 17,592 chars, ratio 0.993. Tags a Hackathon 2026 row as [Student Opportunity].</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 13831 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>marquette-careers</t>
+          <t>lynx-teamtailor</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -26579,17 +26575,17 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
         <is>
-          <t>Marquette Partners</t>
+          <t>Lynx Asset Management</t>
         </is>
       </c>
       <c r="E165" s="3" t="inlineStr">
         <is>
-          <t>https://www.marquettepartnersholdingsllc.com/careers</t>
+          <t>https://careers.lynxhedge.se/jobs.json</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -26604,14 +26600,14 @@
       </c>
       <c r="H165" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 4,406 chars. Experienced only today.</t>
+          <t>Verified 2026-09-11: Teamtailor JSON feed, 17,592 chars, ratio 0.993. Tags a Hackathon 2026 row as [Student Opportunity].</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>mathprograms-listing</t>
+          <t>marquette-careers</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -26621,17 +26617,17 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>MathPrograms.org programme listing</t>
+          <t>Marquette Partners</t>
         </is>
       </c>
       <c r="E166" s="3" t="inlineStr">
         <is>
-          <t>https://www.mathprograms.org/db/program</t>
+          <t>https://www.marquettepartnersholdingsllc.com/careers</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -26646,14 +26642,14 @@
       </c>
       <c r="H166" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 3,585 chars, ratio 0.166.</t>
+          <t>Verified 2026-09-11: 4,406 chars. Experienced only today.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
         <is>
-          <t>meta-hacker-cup</t>
+          <t>mathprograms-listing</t>
         </is>
       </c>
       <c r="B167" s="2" t="inlineStr">
@@ -26663,17 +26659,17 @@
       </c>
       <c r="C167" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
         <is>
-          <t>Meta Hacker Cup</t>
+          <t>MathPrograms.org programme listing</t>
         </is>
       </c>
       <c r="E167" s="3" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
+          <t>https://www.mathprograms.org/db/program</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
@@ -26688,14 +26684,14 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>render_js: verified 2026-09-26 through gather.browser, 1,485 chars rendered.</t>
+          <t>Verified 2026-09-26: 200, 3,585 chars, ratio 0.166.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>mit-battlecode-2027</t>
+          <t>meta-hacker-cup</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -26705,17 +26701,17 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>MIT Battlecode 2027</t>
+          <t>Meta Hacker Cup</t>
         </is>
       </c>
       <c r="E168" s="3" t="inlineStr">
         <is>
-          <t>https://battlecode.org/</t>
+          <t>https://www.facebook.com/codingcompetitions/hacker-cup</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -26730,14 +26726,14 @@
       </c>
       <c r="H168" s="2" t="inlineStr">
         <is>
-          <t>Probed: HTTP 200, 1,627 chars of visible text over plain HTTP, no robots.txt. Home page carries the live season banner ('Battlecode 2026 ended on January 31st, 2026!'), so a text diff should catch the 2027 announcement.</t>
+          <t>render_js: verified 2026-09-26 through gather.browser, 1,485 chars rendered.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
         <is>
-          <t>mit-trading-competition</t>
+          <t>mit-battlecode-2027</t>
         </is>
       </c>
       <c r="B169" s="2" t="inlineStr">
@@ -26752,12 +26748,12 @@
       </c>
       <c r="D169" s="2" t="inlineStr">
         <is>
-          <t>Traders@MIT Trading Competition</t>
+          <t>MIT Battlecode 2027</t>
         </is>
       </c>
       <c r="E169" s="3" t="inlineStr">
         <is>
-          <t>https://traders.mit.edu/competition</t>
+          <t>https://battlecode.org/</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
@@ -26772,14 +26768,14 @@
       </c>
       <c r="H169" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 974 chars, ratio 0.041. 'Applications Closed Spring 2026'.</t>
+          <t>Probed: HTTP 200, 1,627 chars of visible text over plain HTTP, no robots.txt. Home page carries the live season banner ('Battlecode 2026 ended on January 31st, 2026!'), so a text diff should catch the 2027 announcement.</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
         <is>
-          <t>mitll-students</t>
+          <t>mit-trading-competition</t>
         </is>
       </c>
       <c r="B170" s="2" t="inlineStr">
@@ -26794,12 +26790,12 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>MIT Lincoln Laboratory student opportunities</t>
+          <t>Traders@MIT Trading Competition</t>
         </is>
       </c>
       <c r="E170" s="3" t="inlineStr">
         <is>
-          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
+          <t>https://traders.mit.edu/competition</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -26814,14 +26810,14 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 6545 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 974 chars, ratio 0.041. 'Applications Closed Spring 2026'.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
         <is>
-          <t>mlh-season-events</t>
+          <t>mitll-students</t>
         </is>
       </c>
       <c r="B171" s="2" t="inlineStr">
@@ -26831,20 +26827,24 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>MLH hackathon season calendar</t>
+          <t>MIT Lincoln Laboratory student opportunities</t>
         </is>
       </c>
       <c r="E171" s="3" t="inlineStr">
         <is>
-          <t>https://www.mlh.com/seasons/2027/events</t>
-        </is>
-      </c>
-      <c r="F171" s="2" t="inlineStr"/>
+          <t>https://www.ll.mit.edu/careers/student-opportunities</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26852,14 +26852,14 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 7,592 chars from 580KB (ratio 0.0131), allowed by robots.txt. Lists every upcoming MLH member event (~100) with city, dates and tags (DIVERSITY, HARDWARE, HIGH SCHOOL); it does not mark travel reimbursement. mlh.com/events 302s to this season URL, so the season is pinned to avoid a standing redirect warning: re-point when the 2028 season opens (late summer 2027); the upcoming list emptying at season end trips the shrink guard.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 6545 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
         <is>
-          <t>neo-scholars</t>
+          <t>mlh-season-events</t>
         </is>
       </c>
       <c r="B172" s="2" t="inlineStr">
@@ -26869,24 +26869,20 @@
       </c>
       <c r="C172" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>Neo Scholars</t>
+          <t>MLH hackathon season calendar</t>
         </is>
       </c>
       <c r="E172" s="3" t="inlineStr">
         <is>
-          <t>https://neo.com/scholars</t>
-        </is>
-      </c>
-      <c r="F172" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://www.mlh.com/seasons/2027/events</t>
+        </is>
+      </c>
+      <c r="F172" s="2" t="inlineStr"/>
       <c r="G172" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26894,14 +26890,14 @@
       </c>
       <c r="H172" s="2" t="inlineStr">
         <is>
-          <t>Student programme (mentorship, fast-tracked startup interviews, $40k residency grant). Plain GET is 12 chars (JS shell); rendered 61KB, readable. A programme, not a posting list.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 8,090 chars over 499 lines from 580KB (ratio 0.014, measured by run.py --only), allowed by robots.txt. Lists every upcoming MLH member event (~100) with city, dates and tags (DIVERSITY, HARDWARE, HIGH SCHOOL); it does not mark travel reimbursement. mlh.com/events 302s to this season URL, so the season is pinned to avoid a standing redirect warning: re-point when the 2028 season opens (late summer 2027); the upcoming list emptying at season end trips the shrink guard.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
         <is>
-          <t>nist-surf</t>
+          <t>neo-scholars</t>
         </is>
       </c>
       <c r="B173" s="2" t="inlineStr">
@@ -26911,17 +26907,17 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>NIST SURF</t>
+          <t>Neo Scholars</t>
         </is>
       </c>
       <c r="E173" s="3" t="inlineStr">
         <is>
-          <t>https://www.nist.gov/surf</t>
+          <t>https://neo.com/scholars</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
@@ -26936,14 +26932,14 @@
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30: 200, 105,422 bytes, ~8.7k chars. The page carries the 2027 dates line ('expected to open USAjobs mid-October 2026').</t>
+          <t>Student programme (mentorship, fast-tracked startup interviews, $40k residency grant). Plain GET is 12 chars (JS shell); rendered 61KB, readable. A programme, not a posting list.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
         <is>
-          <t>nsa-students</t>
+          <t>nist-surf</t>
         </is>
       </c>
       <c r="B174" s="2" t="inlineStr">
@@ -26958,12 +26954,12 @@
       </c>
       <c r="D174" s="2" t="inlineStr">
         <is>
-          <t>NSA student programs</t>
+          <t>NIST SURF</t>
         </is>
       </c>
       <c r="E174" s="3" t="inlineStr">
         <is>
-          <t>https://www.intelligencecareers.gov/nsa/students</t>
+          <t>https://www.nist.gov/surf</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
@@ -26978,14 +26974,14 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 1479 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-30: 200, 105,422 bytes, ~8.7k chars. The page carries the 2027 dates line ('expected to open USAjobs mid-October 2026').</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
         <is>
-          <t>open-source-quantitative-finance</t>
+          <t>nsa-students</t>
         </is>
       </c>
       <c r="B175" s="2" t="inlineStr">
@@ -27000,12 +26996,12 @@
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>Open Source Quantitative Finance Conference</t>
+          <t>NSA student programs</t>
         </is>
       </c>
       <c r="E175" s="3" t="inlineStr">
         <is>
-          <t>https://osqf.org/</t>
+          <t>https://www.intelligencecareers.gov/nsa/students</t>
         </is>
       </c>
       <c r="F175" s="2" t="inlineStr">
@@ -27020,14 +27016,14 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 1966 chars of text over plain HTTP.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 1479 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
         <is>
-          <t>optiver-futurefocus</t>
+          <t>open-source-quantitative-finance</t>
         </is>
       </c>
       <c r="B176" s="2" t="inlineStr">
@@ -27042,12 +27038,12 @@
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>Optiver FutureFocus</t>
+          <t>Open Source Quantitative Finance Conference</t>
         </is>
       </c>
       <c r="E176" s="3" t="inlineStr">
         <is>
-          <t>https://www.optiver.com/join-us/students/programs/futurefocus/</t>
+          <t>https://osqf.org/</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
@@ -27062,14 +27058,14 @@
       </c>
       <c r="H176" s="2" t="inlineStr">
         <is>
-          <t>Programme page for FutureFocus, Optiver's five-day discovery programme, which the page states is for FIRST and second-year students. Renamed and re-pointed 2026-09-11: the old id and URL (optiver-futurefocus-chicago-2026, /recruitment-events/futurefocus-chicago) baked in a city and a year, and the old URL now 301s here. Verified 2026-09-11: 4,591 chars. Note the page states no graduation-year window, only 'first and second-year', so eligibility cannot be confirmed from it the way Susquehanna's postings can - read the application itself before trusting the label.</t>
+          <t>Probed 2026-09-06: 200, 1966 chars of text over plain HTTP.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
         <is>
-          <t>optiver-ready-trader</t>
+          <t>optiver-futurefocus</t>
         </is>
       </c>
       <c r="B177" s="2" t="inlineStr">
@@ -27084,34 +27080,34 @@
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>Optiver Ready Trader Go</t>
+          <t>Optiver FutureFocus</t>
         </is>
       </c>
       <c r="E177" s="3" t="inlineStr">
         <is>
-          <t>https://readytradergo.optiver.com/</t>
+          <t>https://www.optiver.com/join-us/students/programs/futurefocus/</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-08T14:49:47+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr">
         <is>
-          <t>PHASE 3. Verified: 200, ~1KB of text over plain HTTP, no JS needed.</t>
+          <t>Programme page for FutureFocus, Optiver's five-day discovery programme, which the page states is for FIRST and second-year students. Renamed and re-pointed 2026-09-11: the old id and URL (optiver-futurefocus-chicago-2026, /recruitment-events/futurefocus-chicago) baked in a city and a year, and the old URL now 301s here. Verified 2026-09-11: 4,591 chars. Note the page states no graduation-year window, only 'first and second-year', so eligibility cannot be confirmed from it the way Susquehanna's postings can - read the application itself before trusting the label.</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
         <is>
-          <t>pokerbots</t>
+          <t>optiver-ready-trader</t>
         </is>
       </c>
       <c r="B178" s="2" t="inlineStr">
@@ -27126,34 +27122,34 @@
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>MIT Pokerbots</t>
+          <t>Optiver Ready Trader Go</t>
         </is>
       </c>
       <c r="E178" s="3" t="inlineStr">
         <is>
-          <t>https://pokerbots.org/</t>
+          <t>https://readytradergo.optiver.com/</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-07T14:42:32+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr">
         <is>
-          <t>PHASE 3. Verified: 200, ~6.2KB of text over plain HTTP, no JS needed. Needs a selector - the page retains announcement banners from 2023-2026 in the markup.</t>
+          <t>PHASE 3. Verified: 200, ~1KB of text over plain HTTP, no JS needed.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>purdue-srop</t>
+          <t>pokerbots</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
@@ -27168,12 +27164,12 @@
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>Purdue Summer Research Opportunities Program (SROP)</t>
+          <t>MIT Pokerbots</t>
         </is>
       </c>
       <c r="E179" s="3" t="inlineStr">
         <is>
-          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
+          <t>https://pokerbots.org/</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
@@ -27188,14 +27184,14 @@
       </c>
       <c r="H179" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 16224 characters of visible text, no JavaScript needed.</t>
+          <t>PHASE 3. Verified: 200, ~6.2KB of text over plain HTTP, no JS needed. Needs a selector - the page retains announcement banners from 2023-2026 in the markup.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
         <is>
-          <t>rentec-careers</t>
+          <t>purdue-srop</t>
         </is>
       </c>
       <c r="B180" s="2" t="inlineStr">
@@ -27210,12 +27206,12 @@
       </c>
       <c r="D180" s="2" t="inlineStr">
         <is>
-          <t>Renaissance Technologies</t>
+          <t>Purdue Summer Research Opportunities Program (SROP)</t>
         </is>
       </c>
       <c r="E180" s="3" t="inlineStr">
         <is>
-          <t>https://www.rentec.com/careers</t>
+          <t>https://www.purdue.edu/academics/ogsps/ogrs/summer-research-opportunity-program/</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -27230,14 +27226,14 @@
       </c>
       <c r="H180" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 1,380 chars of text.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 16224 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>reufinder-freshmen</t>
+          <t>rentec-careers</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -27252,12 +27248,12 @@
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>REU Finder - freshman-eligible filter</t>
+          <t>Renaissance Technologies</t>
         </is>
       </c>
       <c r="E181" s="3" t="inlineStr">
         <is>
-          <t>https://reufinder.com/programs-for-freshmen/</t>
+          <t>https://www.rentec.com/careers</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
@@ -27272,14 +27268,14 @@
       </c>
       <c r="H181" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 162,692 chars, ratio 0.31. Already posting 2027 entries.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 1,380 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
         <is>
-          <t>rokos-careers</t>
+          <t>reufinder-freshmen</t>
         </is>
       </c>
       <c r="B182" s="2" t="inlineStr">
@@ -27289,17 +27285,17 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>Rokos Capital</t>
+          <t>REU Finder - freshman-eligible filter</t>
         </is>
       </c>
       <c r="E182" s="3" t="inlineStr">
         <is>
-          <t>https://www.rokoscapital.com/careers</t>
+          <t>https://reufinder.com/programs-for-freshmen/</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -27314,14 +27310,14 @@
       </c>
       <c r="H182" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 620 chars of text. Close to the 500-char floor; a redesign will trip the shrink guard rather than go quiet.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 162,692 chars, ratio 0.31. Already posting 2027 entries.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>sandia-students</t>
+          <t>rokos-careers</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -27331,17 +27327,17 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>Sandia National Laboratories student internships</t>
+          <t>Rokos Capital</t>
         </is>
       </c>
       <c r="E183" s="3" t="inlineStr">
         <is>
-          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
+          <t>https://www.rokoscapital.com/careers</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
@@ -27356,14 +27352,14 @@
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 8504 characters of visible text, no JavaScript needed.</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 620 chars of text. Close to the 500-char floor; a redesign will trip the shrink guard rather than go quiet.</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
         <is>
-          <t>scudem</t>
+          <t>sandia-students</t>
         </is>
       </c>
       <c r="B184" s="2" t="inlineStr">
@@ -27378,12 +27374,12 @@
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>SCUDEM</t>
+          <t>Sandia National Laboratories student internships</t>
         </is>
       </c>
       <c r="E184" s="3" t="inlineStr">
         <is>
-          <t>https://www.contest.comap.com/scudem/index.html</t>
+          <t>https://www.sandia.gov/careers/careers/students-and-postdocs/</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -27398,14 +27394,14 @@
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-30 with opportunity-tracker/1.0: 200, 12,029 bytes, ~1.2k chars text. AWS ELB host, not a marketing-site WAF.</t>
+          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 8504 characters of visible text, no JavaScript needed.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>seo-tech</t>
+          <t>scudem</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
@@ -27420,12 +27416,12 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t>SEO Tech Developer + First-Year Academy</t>
+          <t>SCUDEM</t>
         </is>
       </c>
       <c r="E185" s="3" t="inlineStr">
         <is>
-          <t>https://tech.seo-usa.org/</t>
+          <t>https://www.contest.comap.com/scudem/index.html</t>
         </is>
       </c>
       <c r="F185" s="2" t="inlineStr">
@@ -27440,14 +27436,14 @@
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 6,446 chars, ratio 0.029.</t>
+          <t>Verified 2026-09-30 with opportunity-tracker/1.0: 200, 12,029 bytes, ~1.2k chars text. AWS ELB host, not a marketing-site WAF.</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
         <is>
-          <t>sfhacks</t>
+          <t>seo-tech</t>
         </is>
       </c>
       <c r="B186" s="2" t="inlineStr">
@@ -27457,20 +27453,24 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>SF Hacks</t>
+          <t>SEO Tech Developer + First-Year Academy</t>
         </is>
       </c>
       <c r="E186" s="3" t="inlineStr">
         <is>
-          <t>https://www.sfhacks.io/</t>
-        </is>
-      </c>
-      <c r="F186" s="2" t="inlineStr"/>
+          <t>https://tech.seo-usa.org/</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27478,14 +27478,14 @@
       </c>
       <c r="H186" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,393 chars from 63KB (ratio 0.054); sfhacks.io redirects to www. States no travel reimbursement.</t>
+          <t>Verified 2026-09-26: 200, 6,446 chars, ratio 0.029.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
         <is>
-          <t>sfi-ucr</t>
+          <t>sfhacks</t>
         </is>
       </c>
       <c r="B187" s="2" t="inlineStr">
@@ -27495,24 +27495,20 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>SFI Undergraduate Complexity Research</t>
+          <t>SF Hacks</t>
         </is>
       </c>
       <c r="E187" s="3" t="inlineStr">
         <is>
-          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
-        </is>
-      </c>
-      <c r="F187" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://www.sfhacks.io/</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr"/>
       <c r="G187" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27520,14 +27516,14 @@
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 4,452 chars, ratio 0.01.</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,393 chars from 63KB (ratio 0.054); sfhacks.io redirects to www. States no travel reimbursement.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
         <is>
-          <t>sjhacks</t>
+          <t>sfi-ucr</t>
         </is>
       </c>
       <c r="B188" s="2" t="inlineStr">
@@ -27537,20 +27533,24 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>SJHacks</t>
+          <t>SFI Undergraduate Complexity Research</t>
         </is>
       </c>
       <c r="E188" s="3" t="inlineStr">
         <is>
-          <t>https://www.sjhacks.com/</t>
-        </is>
-      </c>
-      <c r="F188" s="2" t="inlineStr"/>
+          <t>https://www.santafe.edu/engage/learn/programs/undergraduate-complexity-research</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27558,14 +27558,14 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,323 chars from 63KB (ratio 0.053); sjhacks.com redirects to www. No travel statement.</t>
+          <t>Verified 2026-09-26: 200, 4,452 chars, ratio 0.01.</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
         <is>
-          <t>smart-scholarship</t>
+          <t>sjhacks</t>
         </is>
       </c>
       <c r="B189" s="2" t="inlineStr">
@@ -27575,24 +27575,20 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>SMART Scholarship</t>
+          <t>SJHacks</t>
         </is>
       </c>
       <c r="E189" s="3" t="inlineStr">
         <is>
-          <t>https://www.smartscholarship.org/smart</t>
-        </is>
-      </c>
-      <c r="F189" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08T14:49:47+00:00</t>
-        </is>
-      </c>
+          <t>https://www.sjhacks.com/</t>
+        </is>
+      </c>
+      <c r="F189" s="2" t="inlineStr"/>
       <c r="G189" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27600,14 +27596,14 @@
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
-          <t>render_js: verified 2026-09-26, 3,640 chars rendered (120 plain).</t>
+          <t>Verified 2026-10-08 with the tracker's own client: 200, 3,323 chars from 63KB (ratio 0.053); sjhacks.com redirects to www. No travel statement.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
         <is>
-          <t>solayer-careers</t>
+          <t>smart-scholarship</t>
         </is>
       </c>
       <c r="B190" s="2" t="inlineStr">
@@ -27622,12 +27618,12 @@
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>Solayer Labs</t>
+          <t>SMART Scholarship</t>
         </is>
       </c>
       <c r="E190" s="3" t="inlineStr">
         <is>
-          <t>https://solayer.org/careers</t>
+          <t>https://www.smartscholarship.org/smart</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
@@ -27642,14 +27638,14 @@
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>Added 2026-09-21 from a pasted link. Whole careers page, not a programme page: Solayer Labs (Solana/SVM infrastructure and payments, San Mateo CA) is on no public ATS - 226KB of Framer HTML with no greenhouse/lever/ashby/workday/iCIMS fingerprint and no external apply link, so the page itself is the durable target. Probed: HTTP 200, 2,514 characters of visible text, ratio 0.011, roles are server-rendered and clear both content floors; robots.txt allows. One role listed on the day it was added - Marketing Lead, full-time permanent, master's required, apply by posting a resume with code SLML - which is off-field and not applicable; watched for the engineering and internship postings it may carry later.</t>
+          <t>render_js: verified 2026-09-26, 3,640 chars rendered (120 plain).</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
         <is>
-          <t>stevens-high-frequency-trading</t>
+          <t>solayer-careers</t>
         </is>
       </c>
       <c r="B191" s="2" t="inlineStr">
@@ -27659,17 +27655,17 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>Stevens High Frequency Trading Competition 2026</t>
+          <t>Solayer Labs</t>
         </is>
       </c>
       <c r="E191" s="3" t="inlineStr">
         <is>
-          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
+          <t>https://solayer.org/careers</t>
         </is>
       </c>
       <c r="F191" s="2" t="inlineStr">
@@ -27684,14 +27680,14 @@
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
-          <t>Probed 2026-09-06: 200, 10400 chars of text over plain HTTP, robots.txt allows. Cleanly pollable.</t>
+          <t>Added 2026-09-21 from a pasted link. Whole careers page, not a programme page: Solayer Labs (Solana/SVM infrastructure and payments, San Mateo CA) is on no public ATS - 226KB of Framer HTML with no greenhouse/lever/ashby/workday/iCIMS fingerprint and no external apply link, so the page itself is the durable target. Probed: HTTP 200, 2,514 characters of visible text, ratio 0.011, roles are server-rendered and clear both content floors; robots.txt allows. One role listed on the day it was added - Marketing Lead, full-time permanent, master's required, apply by posting a resume with code SLML - which is off-field and not applicable; watched for the engineering and internship postings it may carry later.</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
         <is>
-          <t>surim-apply</t>
+          <t>stevens-high-frequency-trading</t>
         </is>
       </c>
       <c r="B192" s="2" t="inlineStr">
@@ -27706,12 +27702,12 @@
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>Stanford SURIM</t>
+          <t>Stevens High Frequency Trading Competition 2026</t>
         </is>
       </c>
       <c r="E192" s="3" t="inlineStr">
         <is>
-          <t>https://surim.stanford.edu/apply-surim</t>
+          <t>https://www.stevens.edu/page-basic/2026-stevens-high-frequency-trading-competition</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
@@ -27726,14 +27722,14 @@
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,986 chars, ratio 0.098.</t>
+          <t>Probed 2026-09-06: 200, 10400 chars of text over plain HTTP, robots.txt allows. Cleanly pollable.</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
         <is>
-          <t>tgs-join-our-team</t>
+          <t>surim-apply</t>
         </is>
       </c>
       <c r="B193" s="2" t="inlineStr">
@@ -27743,17 +27739,17 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>TGS Management</t>
+          <t>Stanford SURIM</t>
         </is>
       </c>
       <c r="E193" s="3" t="inlineStr">
         <is>
-          <t>https://www.tgsmc.com/join-our-team/</t>
+          <t>https://surim.stanford.edu/apply-surim</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
@@ -27768,14 +27764,14 @@
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-11: 1,977 chars. The Lever slug `tgsmc` resolves but returns an empty list, so the page is the only non-alerting surface.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,986 chars, ratio 0.098.</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
         <is>
-          <t>thrive-portfolio-interns</t>
+          <t>tgs-join-our-team</t>
         </is>
       </c>
       <c r="B194" s="2" t="inlineStr">
@@ -27785,17 +27781,17 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>low</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>Thrive Capital portfolio internships (early-stage US)</t>
+          <t>TGS Management</t>
         </is>
       </c>
       <c r="E194" s="3" t="inlineStr">
         <is>
-          <t>https://jobs.thrivecap.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
+          <t>https://www.tgsmc.com/join-our-team/</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -27810,14 +27806,14 @@
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>Getro board (collection 2105), server-rendered. filter= is base64 of {seniority:[internship], organization.stage:[pre_seed,seed,series_a,series_b], searchable_locations:[United States]}. 57 postings 2026-09-30; page shows first 20, newest first. 9,958 chars, ratio 0.0375.</t>
+          <t>Verified 2026-09-11: 1,977 chars. The Lever slug `tgsmc` resolves but returns an empty list, so the page is the only non-alerting surface.</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
         <is>
-          <t>tradebot-students</t>
+          <t>thrive-portfolio-interns</t>
         </is>
       </c>
       <c r="B195" s="2" t="inlineStr">
@@ -27827,17 +27823,17 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>high</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>Tradebot Systems</t>
+          <t>Thrive Capital portfolio internships (early-stage US)</t>
         </is>
       </c>
       <c r="E195" s="3" t="inlineStr">
         <is>
-          <t>https://www.tradebot.com/careers/students</t>
+          <t>https://jobs.thrivecap.com/jobs?filter=eyJzZW5pb3JpdHkiOlsiaW50ZXJuc2hpcCJdLCJvcmdhbml6YXRpb24uc3RhZ2UiOlsicHJlX3NlZWQiLCJzZWVkIiwic2VyaWVzX2EiLCJzZXJpZXNfYiJdLCJzZWFyY2hhYmxlX2xvY2F0aW9ucyI6WyJVbml0ZWQgU3RhdGVzIl19</t>
         </is>
       </c>
       <c r="F195" s="2" t="inlineStr">
@@ -27852,14 +27848,14 @@
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 1,253 chars of text.</t>
+          <t>Getro board (collection 2105), server-rendered. filter= is base64 of {seniority:[internship], organization.stage:[pre_seed,seed,series_a,series_b], searchable_locations:[United States]}. 57 postings 2026-09-30; page shows first 20, newest first. 9,958 chars, ratio 0.0375.</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
         <is>
-          <t>treehacks</t>
+          <t>tradebot-students</t>
         </is>
       </c>
       <c r="B196" s="2" t="inlineStr">
@@ -27874,12 +27870,12 @@
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>TreeHacks</t>
+          <t>Tradebot Systems</t>
         </is>
       </c>
       <c r="E196" s="3" t="inlineStr">
         <is>
-          <t>https://treehacks.com/</t>
+          <t>https://www.tradebot.com/careers/students</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -27894,14 +27890,14 @@
       </c>
       <c r="H196" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26: 200, 3,519 chars, ratio 0.024 (www redirects to the bare domain).</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 1,253 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
         <is>
-          <t>trexquant-students</t>
+          <t>treehacks</t>
         </is>
       </c>
       <c r="B197" s="2" t="inlineStr">
@@ -27916,12 +27912,12 @@
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>Trexquant</t>
+          <t>TreeHacks</t>
         </is>
       </c>
       <c r="E197" s="3" t="inlineStr">
         <is>
-          <t>https://trexquant.com/careers/students</t>
+          <t>https://treehacks.com/</t>
         </is>
       </c>
       <c r="F197" s="2" t="inlineStr">
@@ -27936,14 +27932,14 @@
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
-          <t>Firm is on no public ATS. Verified 2026-09-11: 891 chars of text.</t>
+          <t>Verified 2026-09-26: 200, 3,519 chars, ratio 0.024 (www redirects to the bare domain).</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
         <is>
-          <t>twosigma-campus</t>
+          <t>trexquant-students</t>
         </is>
       </c>
       <c r="B198" s="2" t="inlineStr">
@@ -27953,17 +27949,17 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>Two Sigma</t>
+          <t>Trexquant</t>
         </is>
       </c>
       <c r="E198" s="3" t="inlineStr">
         <is>
-          <t>https://careers.twosigma.com/careers/OpenRoles/</t>
+          <t>https://trexquant.com/careers/students</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
@@ -27978,14 +27974,14 @@
       </c>
       <c r="H198" s="2" t="inlineStr">
         <is>
-          <t>Re-pointed 2026-09-12: the old /careers/students/ url 301'd to the generic /careers/ page and had been reporting success from it. The internships page is the real replacement (9,509 chars, 29 'intern' mentions). No public vendor ATS -- careers.twosigma.com is a custom board with no Greenhouse/Lever/Ashby fingerprint. Correction 2026-09-16: "no public vendor ATS" was wrong in its conclusion though right that there is no Greenhouse/Lever/Ashby fingerprint -- careers.twosigma.com is Avature (CNAME portaltwosigma.avature.net), a vendor ATS this project does not fingerprint. Re-pointed to its OpenRoles listing: 2,676 chars at ratio 0.024, including "AI Research Scientist - Intern [2027 Summer]". Vendor-hosted, so outside the WAF that 403s the runner on www.twosigma.com (WP Engine).</t>
+          <t>Firm is on no public ATS. Verified 2026-09-11: 891 chars of text.</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
         <is>
-          <t>uchicago-trading-competition</t>
+          <t>twosigma-campus</t>
         </is>
       </c>
       <c r="B199" s="2" t="inlineStr">
@@ -28000,12 +27996,12 @@
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>UChicago Trading Competition</t>
+          <t>Two Sigma</t>
         </is>
       </c>
       <c r="E199" s="3" t="inlineStr">
         <is>
-          <t>https://tradingcompetition.uchicago.edu/</t>
+          <t>https://careers.twosigma.com/careers/OpenRoles/</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
@@ -28020,14 +28016,14 @@
       </c>
       <c r="H199" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,144 chars, ratio 0.206. Still shows the 2026 event.</t>
+          <t>Re-pointed 2026-09-12: the old /careers/students/ url 301'd to the generic /careers/ page and had been reporting success from it. The internships page is the real replacement (9,509 chars, 29 'intern' mentions). No public vendor ATS -- careers.twosigma.com is a custom board with no Greenhouse/Lever/Ashby fingerprint. Correction 2026-09-16: "no public vendor ATS" was wrong in its conclusion though right that there is no Greenhouse/Lever/Ashby fingerprint -- careers.twosigma.com is Avature (CNAME portaltwosigma.avature.net), a vendor ATS this project does not fingerprint. Re-pointed to its OpenRoles listing: 2,676 chars at ratio 0.024, including "AI Research Scientist - Intern [2027 Summer]". Vendor-hosted, so outside the WAF that 403s the runner on www.twosigma.com (WP Engine).</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
         <is>
-          <t>usc-ict-summer</t>
+          <t>uchicago-trading-competition</t>
         </is>
       </c>
       <c r="B200" s="2" t="inlineStr">
@@ -28042,23 +28038,27 @@
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>USC ICT Summer Research Program</t>
+          <t>UChicago Trading Competition</t>
         </is>
       </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>https://ict.usc.edu/careers/internships/summer-research-program-application/</t>
-        </is>
-      </c>
-      <c r="F200" s="2" t="inlineStr"/>
+          <t>https://tradingcompetition.uchicago.edu/</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08T14:49:47+00:00</t>
+        </is>
+      </c>
       <c r="G200" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>Verified 2026-10-01 with the tracker's own client: HTTP 200, allowed by robots.txt, 762 characters of visible text, no JavaScript needed.</t>
+          <t>Verified 2026-09-26 (source research) with the tracker's own client: 200, 1,144 chars, ratio 0.206. Still shows the 2026 event.</t>
         </is>
       </c>
     </row>
@@ -29267,9 +29267,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E87" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E88" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E89" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E93" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E90" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E91" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E92" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E94" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E95" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E96" r:id="rId12"/>

</xml_diff>

<commit_message>
state: 2026-10-09 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6506,7 +6506,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6804,7 +6804,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J119" s="2" t="inlineStr"/>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K119" s="2" t="inlineStr"/>
       <c r="L119" s="2" t="inlineStr"/>
       <c r="M119" s="2" t="inlineStr">
@@ -6812,7 +6816,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N119" s="2" t="inlineStr"/>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>3b7bcf43a0172952aa50d25c1337ab7318ffbda8b58b9d37169116c38b5e08a4</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7016,7 +7024,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K123" s="2" t="inlineStr"/>
       <c r="L123" s="2" t="inlineStr"/>
       <c r="M123" s="2" t="inlineStr">
@@ -7024,7 +7036,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N123" s="2" t="inlineStr"/>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>a05d036dfccf9c6912b038cc1bced7f3e404d115cb9a862e595f79492dc87f5c</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7224,7 +7240,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J127" s="2" t="inlineStr"/>
+      <c r="J127" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K127" s="2" t="inlineStr"/>
       <c r="L127" s="2" t="inlineStr"/>
       <c r="M127" s="2" t="inlineStr">
@@ -7990,7 +8010,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8054,12 +8074,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8070,7 +8090,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>bfdd2e277c2c12081d4935c0396b97768545901235ccd3b5d52a70b6c940ff94</t>
+          <t>fa93f8d76ea09413cc7c718ed451b26c26ad2d228c00e765d59475f203efec16</t>
         </is>
       </c>
     </row>
@@ -8122,7 +8142,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8190,7 +8210,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8254,7 +8274,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8590,7 +8610,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8658,7 +8678,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8730,7 +8750,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8858,7 +8878,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8926,12 +8946,12 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T00:52:12+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
@@ -8946,7 +8966,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>0a65a7d54ecc562352de4dfca24a192526334f0c374fa2839c7c3dcc19d1c4f2</t>
+          <t>2fc8ac2223271ae6acdb0190db9faae5c00a54a8c4e19384fe8d05ea732ea516</t>
         </is>
       </c>
     </row>
@@ -8998,7 +9018,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10690,7 +10710,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10870,7 +10890,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10938,12 +10958,12 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:00:53+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L192" s="2" t="inlineStr">
@@ -10958,7 +10978,7 @@
       </c>
       <c r="N192" s="2" t="inlineStr">
         <is>
-          <t>5849cd1f0a1d2fe399642c5beec06f20d5e3f29b3f5e385731ecd95949e16c1b</t>
+          <t>650a293414a2ed55794add852584991215842908be7f45aa94b52cc7616e798a</t>
         </is>
       </c>
     </row>
@@ -11010,12 +11030,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11030,7 +11050,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>55aa3c3b411138dba0e0c12558b43e7e4e74fecce5f11007874d8206b922daa3</t>
+          <t>ba5c2a7269bd068d12484a0639e74d3481f622b69c856afc6f3d79d402dfd31e</t>
         </is>
       </c>
     </row>
@@ -11082,12 +11102,12 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L194" s="2" t="inlineStr">
@@ -11102,7 +11122,7 @@
       </c>
       <c r="N194" s="2" t="inlineStr">
         <is>
-          <t>c52b57cce9eb161c21a787804f715604ea4b9b4451a07f4c154df106687dae71</t>
+          <t>eb6c71808c83546daa05541541be631063ae1c3125608d710c8796264c76afae</t>
         </is>
       </c>
     </row>
@@ -11154,7 +11174,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11226,12 +11246,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11246,7 +11266,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>4a26ade2f69607e364c3af2b4ec186ffb3cf4ae890c4df9033aee06cab95819d</t>
+          <t>c738a28ca945b73ae10dbac861a04080b088fd5f46f7f61fd249e436264ab5fb</t>
         </is>
       </c>
     </row>
@@ -11298,7 +11318,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11370,7 +11390,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11438,7 +11458,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11506,7 +11526,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11574,7 +11594,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11646,7 +11666,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11714,7 +11734,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11786,12 +11806,12 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L204" s="2" t="inlineStr">
@@ -11806,7 +11826,7 @@
       </c>
       <c r="N204" s="2" t="inlineStr">
         <is>
-          <t>fe407a1f970cb6774a68730ac78b1812bb948b211b14501b52cdc9c3a22dbccf</t>
+          <t>e386a49fc405e8f0578ce0070f1916df213f95355fa7210de1fe27beac7d0f97</t>
         </is>
       </c>
     </row>
@@ -11858,7 +11878,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -11990,7 +12010,7 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
@@ -12062,7 +12082,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12130,7 +12150,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12202,7 +12222,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12498,7 +12518,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12746,7 +12766,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12814,7 +12834,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12882,7 +12902,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13072,7 +13092,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J224" s="2" t="inlineStr"/>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K224" s="2" t="inlineStr"/>
       <c r="L224" s="2" t="inlineStr">
         <is>
@@ -13084,7 +13108,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N224" s="2" t="inlineStr"/>
+      <c r="N224" s="2" t="inlineStr">
+        <is>
+          <t>86c7e948b3264fe37a0c5409975f8fec1eea4f0ff8f9c01b11bb08ebada1876d</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="inlineStr">
@@ -13132,7 +13160,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J225" s="2" t="inlineStr"/>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K225" s="2" t="inlineStr"/>
       <c r="L225" s="2" t="inlineStr">
         <is>
@@ -13144,7 +13176,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N225" s="2" t="inlineStr"/>
+      <c r="N225" s="2" t="inlineStr">
+        <is>
+          <t>66a0661a0966c676dd7d1d601a9d41ac34dadac9991081817d728bef6a5ab33e</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -13192,7 +13228,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J226" s="2" t="inlineStr"/>
+      <c r="J226" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K226" s="2" t="inlineStr"/>
       <c r="L226" s="2" t="inlineStr">
         <is>
@@ -13204,7 +13244,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N226" s="2" t="inlineStr"/>
+      <c r="N226" s="2" t="inlineStr">
+        <is>
+          <t>81a8cc3894d31d1c48ec96e11198fcb9bc26f93e549242b13ab98d9048060022</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -13252,7 +13296,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J227" s="2" t="inlineStr"/>
+      <c r="J227" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K227" s="2" t="inlineStr"/>
       <c r="L227" s="2" t="inlineStr">
         <is>
@@ -13264,7 +13312,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N227" s="2" t="inlineStr"/>
+      <c r="N227" s="2" t="inlineStr">
+        <is>
+          <t>72d03b08d589492cd60f3d2986f1260cea965b3cfe6de216375d328caf7c6aea</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -13312,7 +13364,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J228" s="2" t="inlineStr"/>
+      <c r="J228" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K228" s="2" t="inlineStr"/>
       <c r="L228" s="2" t="inlineStr">
         <is>
@@ -13324,7 +13380,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N228" s="2" t="inlineStr"/>
+      <c r="N228" s="2" t="inlineStr">
+        <is>
+          <t>9ad1b81208e9662d9d0b011457b245be0df7486d3a66e613119d2e03034a8099</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -13372,7 +13432,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J229" s="2" t="inlineStr"/>
+      <c r="J229" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K229" s="2" t="inlineStr"/>
       <c r="L229" s="2" t="inlineStr">
         <is>
@@ -13384,7 +13448,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N229" s="2" t="inlineStr"/>
+      <c r="N229" s="2" t="inlineStr">
+        <is>
+          <t>9bb41627f314ac00faea49ef02e861785d54dfbbd8be435221640cf6c998e7f5</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -13488,7 +13556,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J231" s="2" t="inlineStr"/>
+      <c r="J231" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K231" s="2" t="inlineStr"/>
       <c r="L231" s="2" t="inlineStr">
         <is>
@@ -13500,7 +13572,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N231" s="2" t="inlineStr"/>
+      <c r="N231" s="2" t="inlineStr">
+        <is>
+          <t>7aac9d9c52a684d194f84c75ea15e8b14fb3a13a5f54f735261a8d39b6d4af67</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="inlineStr">
@@ -13548,7 +13624,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J232" s="2" t="inlineStr"/>
+      <c r="J232" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K232" s="2" t="inlineStr"/>
       <c r="L232" s="2" t="inlineStr">
         <is>
@@ -13784,7 +13864,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J236" s="2" t="inlineStr"/>
+      <c r="J236" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K236" s="2" t="inlineStr"/>
       <c r="L236" s="2" t="inlineStr">
         <is>
@@ -13796,7 +13880,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N236" s="2" t="inlineStr"/>
+      <c r="N236" s="2" t="inlineStr">
+        <is>
+          <t>dcdb120dbe3f7a669c69db40787e656451bfafc441a9b3e2b65cd88b960058d8</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="inlineStr">
@@ -18046,12 +18134,12 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L312" s="2" t="inlineStr">
@@ -18066,7 +18154,7 @@
       </c>
       <c r="N312" s="2" t="inlineStr">
         <is>
-          <t>54f57f8f73ad40662374dbfec960a34fd4666e285a941647a51880f38dd2f712</t>
+          <t>35faef9fae846e990fab57f24c2da1aa1dbbaca7cd66ec0c677871c020c6d346</t>
         </is>
       </c>
     </row>
@@ -18118,7 +18206,7 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K313" s="2" t="inlineStr"/>
@@ -18132,7 +18220,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N313" s="2" t="inlineStr"/>
+      <c r="N313" s="2" t="inlineStr">
+        <is>
+          <t>760fd1e652f7d1a0967c79c08ce0ec746ef0663e9352d0491c7bf0b00e2688a6</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="2" t="inlineStr">
@@ -18182,7 +18274,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18254,7 +18346,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18322,7 +18414,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18390,7 +18482,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18514,7 +18606,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -18942,7 +19034,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19010,7 +19102,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19078,7 +19170,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19146,12 +19238,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19166,7 +19258,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>e551b13659a4f8862b63ed994c9170edce4e4d1ab9e6ac64edff474e7af9c2f6</t>
+          <t>e7d3380f7da6ba01188e2a946c522701b458faccfe24f80bf9ee0779fb949048</t>
         </is>
       </c>
     </row>
@@ -19218,12 +19310,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19238,7 +19330,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>dede29f8b571b783b3c67925c068a1ff3c309eea041e18fbeaf1d1a1ed23ffe5</t>
+          <t>3364770d8ef21d5b502b30b49d73d867654fa68a942a212dbde11eaeb01b3b2d</t>
         </is>
       </c>
     </row>
@@ -19290,12 +19382,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19310,7 +19402,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>7a8bd2d9b8a0739c578852b2825509d25db26005c7cd95298de5ba16da3e6d5b</t>
+          <t>c831be1f7e407c8962f45bd4f14f4398a8d8fc22fba3472377c75ffedbfbec77</t>
         </is>
       </c>
     </row>
@@ -19360,7 +19452,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J332" s="2" t="inlineStr"/>
+      <c r="J332" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K332" s="2" t="inlineStr"/>
       <c r="L332" s="2" t="inlineStr">
         <is>
@@ -19372,7 +19468,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N332" s="2" t="inlineStr"/>
+      <c r="N332" s="2" t="inlineStr">
+        <is>
+          <t>7ab22c25100b1653e811fd08ea7b898d5db6f3ff74bb599e2c0a92951160a597</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="2" t="inlineStr">
@@ -19476,7 +19576,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J334" s="2" t="inlineStr"/>
+      <c r="J334" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K334" s="2" t="inlineStr"/>
       <c r="L334" s="2" t="inlineStr">
         <is>
@@ -19488,7 +19592,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N334" s="2" t="inlineStr"/>
+      <c r="N334" s="2" t="inlineStr">
+        <is>
+          <t>1e606554cb1fb3233faad3f328b540d49ed508c91d00a0f43d4a661e0a0455d6</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="2" t="inlineStr">
@@ -19536,7 +19644,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J335" s="2" t="inlineStr"/>
+      <c r="J335" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K335" s="2" t="inlineStr"/>
       <c r="L335" s="2" t="inlineStr">
         <is>
@@ -19548,7 +19660,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N335" s="2" t="inlineStr"/>
+      <c r="N335" s="2" t="inlineStr">
+        <is>
+          <t>c82ad6e396a494c1d28812732826d280080ea860925c28c7c9631f0698c0ce63</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="2" t="inlineStr">
@@ -19596,7 +19712,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J336" s="2" t="inlineStr"/>
+      <c r="J336" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K336" s="2" t="inlineStr"/>
       <c r="L336" s="2" t="inlineStr">
         <is>
@@ -19608,7 +19728,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N336" s="2" t="inlineStr"/>
+      <c r="N336" s="2" t="inlineStr">
+        <is>
+          <t>60a00bf44ee65fc9a6885579a3d1b8db86c815e4955f959203554379397a67d5</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -19656,7 +19780,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J337" s="2" t="inlineStr"/>
+      <c r="J337" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K337" s="2" t="inlineStr"/>
       <c r="L337" s="2" t="inlineStr">
         <is>
@@ -19668,7 +19796,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N337" s="2" t="inlineStr"/>
+      <c r="N337" s="2" t="inlineStr">
+        <is>
+          <t>b974bde6fb9765f483d9acb34135a5d37f925aecea5037ec34a676b0394c30e9</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -19716,7 +19848,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J338" s="2" t="inlineStr"/>
+      <c r="J338" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K338" s="2" t="inlineStr"/>
       <c r="L338" s="2" t="inlineStr">
         <is>
@@ -19728,7 +19864,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N338" s="2" t="inlineStr"/>
+      <c r="N338" s="2" t="inlineStr">
+        <is>
+          <t>ea06a46b11320bd57b751172369cfcc31f17024123cbd88ddcaf6a325a9e091c</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -19776,7 +19916,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J339" s="2" t="inlineStr"/>
+      <c r="J339" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K339" s="2" t="inlineStr"/>
       <c r="L339" s="2" t="inlineStr">
         <is>
@@ -19788,7 +19932,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N339" s="2" t="inlineStr"/>
+      <c r="N339" s="2" t="inlineStr">
+        <is>
+          <t>918a52f94a4c7373e0ca6ebb8b3e5af6910735ca0080fe12b93c03d30cbbc367</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
@@ -19836,7 +19984,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J340" s="2" t="inlineStr"/>
+      <c r="J340" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K340" s="2" t="inlineStr"/>
       <c r="L340" s="2" t="inlineStr">
         <is>
@@ -19848,7 +20000,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N340" s="2" t="inlineStr"/>
+      <c r="N340" s="2" t="inlineStr">
+        <is>
+          <t>7cbee8e9e69bade2441a703f668b47db0bed730ace44335f07c9397f2224e921</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" s="2" t="inlineStr">
@@ -19896,7 +20052,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J341" s="2" t="inlineStr"/>
+      <c r="J341" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K341" s="2" t="inlineStr"/>
       <c r="L341" s="2" t="inlineStr">
         <is>
@@ -19908,7 +20068,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N341" s="2" t="inlineStr"/>
+      <c r="N341" s="2" t="inlineStr">
+        <is>
+          <t>18d18e171afae3acff81839588ce5b4630c393b4040cc728474ab2269a54d251</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="2" t="inlineStr">
@@ -19956,7 +20120,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J342" s="2" t="inlineStr"/>
+      <c r="J342" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K342" s="2" t="inlineStr"/>
       <c r="L342" s="2" t="inlineStr">
         <is>
@@ -19968,7 +20136,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N342" s="2" t="inlineStr"/>
+      <c r="N342" s="2" t="inlineStr">
+        <is>
+          <t>6f3864cfea788dfa8383a47e55d90a3a1a684cd1949baf8f248c58b7d54de7b3</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -20132,7 +20304,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J345" s="2" t="inlineStr"/>
+      <c r="J345" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K345" s="2" t="inlineStr"/>
       <c r="L345" s="2" t="inlineStr">
         <is>
@@ -20144,7 +20320,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N345" s="2" t="inlineStr"/>
+      <c r="N345" s="2" t="inlineStr">
+        <is>
+          <t>c31211e6e78496e706641583348f9e7896ed2e9deced3e7afead68283d64a796</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -20192,7 +20372,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J346" s="2" t="inlineStr"/>
+      <c r="J346" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K346" s="2" t="inlineStr"/>
       <c r="L346" s="2" t="inlineStr">
         <is>
@@ -20204,7 +20388,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N346" s="2" t="inlineStr"/>
+      <c r="N346" s="2" t="inlineStr">
+        <is>
+          <t>62cf2b1e8233f3210e3811388cba703ad037160950fed45ead309ddf75501a12</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -20252,7 +20440,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J347" s="2" t="inlineStr"/>
+      <c r="J347" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K347" s="2" t="inlineStr"/>
       <c r="L347" s="2" t="inlineStr">
         <is>
@@ -20264,7 +20456,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N347" s="2" t="inlineStr"/>
+      <c r="N347" s="2" t="inlineStr">
+        <is>
+          <t>a99f4492af7218450a406851894cfca0769c5478fffc760eb7fefd5656e32715</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -20312,7 +20508,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J348" s="2" t="inlineStr"/>
+      <c r="J348" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K348" s="2" t="inlineStr"/>
       <c r="L348" s="2" t="inlineStr">
         <is>
@@ -20324,7 +20524,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N348" s="2" t="inlineStr"/>
+      <c r="N348" s="2" t="inlineStr">
+        <is>
+          <t>af6aae976a11f28c0bd8b5465e224b6f7b51e64b20224821c597cb9cc63aa3a5</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="inlineStr">
@@ -20372,7 +20576,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J349" s="2" t="inlineStr"/>
+      <c r="J349" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K349" s="2" t="inlineStr"/>
       <c r="L349" s="2" t="inlineStr">
         <is>
@@ -20384,7 +20592,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N349" s="2" t="inlineStr"/>
+      <c r="N349" s="2" t="inlineStr">
+        <is>
+          <t>4bedd057012c58ee5ef8ed7a919564f4b6a35835113213fd5e0411d5177a7151</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -20432,7 +20644,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J350" s="2" t="inlineStr"/>
+      <c r="J350" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K350" s="2" t="inlineStr"/>
       <c r="L350" s="2" t="inlineStr">
         <is>
@@ -20444,7 +20660,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N350" s="2" t="inlineStr"/>
+      <c r="N350" s="2" t="inlineStr">
+        <is>
+          <t>c4f4377b426d0f61d44992fd52d46220ac4354378b16a6c17649e17b1791e969</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -20492,7 +20712,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J351" s="2" t="inlineStr"/>
+      <c r="J351" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K351" s="2" t="inlineStr"/>
       <c r="L351" s="2" t="inlineStr">
         <is>
@@ -20504,7 +20728,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N351" s="2" t="inlineStr"/>
+      <c r="N351" s="2" t="inlineStr">
+        <is>
+          <t>1ba8a44c736a68d0a7d0767bb9b205351a6d3db419b838e9db1f939f34ed7a41</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="inlineStr">
@@ -20552,7 +20780,11 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="J352" s="2" t="inlineStr"/>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="K352" s="2" t="inlineStr"/>
       <c r="L352" s="2" t="inlineStr">
         <is>
@@ -20564,7 +20796,11 @@
           <t>false</t>
         </is>
       </c>
-      <c r="N352" s="2" t="inlineStr"/>
+      <c r="N352" s="2" t="inlineStr">
+        <is>
+          <t>693b069427ebe89db381f243613080d22fa9e9f832f9ce651ff7f887c07140d6</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:N352"/>
@@ -21005,7 +21241,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -21043,7 +21279,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -21085,7 +21321,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -21123,7 +21359,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -21161,7 +21397,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -21199,7 +21435,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -21237,7 +21473,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -21279,7 +21515,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -21317,7 +21553,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -21359,12 +21595,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T16:09:03+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -21401,7 +21637,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -21443,7 +21679,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -21485,7 +21721,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -21527,7 +21763,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -21569,7 +21805,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -21611,7 +21847,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -21653,7 +21889,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -21695,7 +21931,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -21737,7 +21973,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -21779,7 +22015,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -21821,7 +22057,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -21863,7 +22099,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -21901,7 +22137,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -21943,7 +22179,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -21981,7 +22217,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -22023,7 +22259,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -22065,7 +22301,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -22107,7 +22343,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -22149,7 +22385,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -22191,7 +22427,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -22229,7 +22465,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -22267,7 +22503,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -22305,7 +22541,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -22347,7 +22583,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -22389,7 +22625,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -22427,7 +22663,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -22465,7 +22701,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -22507,7 +22743,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -22545,7 +22781,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -22587,7 +22823,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -22625,7 +22861,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -22663,7 +22899,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -22705,7 +22941,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -22743,7 +22979,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -22781,7 +23017,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -22819,7 +23055,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -22861,7 +23097,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -22899,7 +23135,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -22941,7 +23177,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -22983,7 +23219,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -23025,7 +23261,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -23067,7 +23303,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -23105,7 +23341,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -23143,7 +23379,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -23181,7 +23417,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -23223,7 +23459,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -23261,7 +23497,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -23303,7 +23539,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -23345,7 +23581,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -23383,7 +23619,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -23425,7 +23661,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -23467,7 +23703,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -23505,7 +23741,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -23547,7 +23783,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -23585,7 +23821,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -23627,7 +23863,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -23669,7 +23905,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -23711,7 +23947,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -23749,7 +23985,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -23787,7 +24023,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -23825,7 +24061,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -23863,7 +24099,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -23901,7 +24137,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -23943,7 +24179,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -23981,7 +24217,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -24017,7 +24253,11 @@
           <t>weissassetmanagement</t>
         </is>
       </c>
-      <c r="F77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -24057,7 +24297,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -24095,7 +24335,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -24137,7 +24377,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -24175,7 +24415,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -24217,7 +24457,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -24255,7 +24495,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -24293,7 +24533,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -24335,7 +24575,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -24681,7 +24921,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -24723,7 +24963,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -24765,7 +25005,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -24807,7 +25047,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -24849,7 +25089,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -24891,7 +25131,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -24933,7 +25173,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -24975,7 +25215,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -25015,7 +25255,11 @@
           <t>https://www.blvdinvestmentgroup.org/thebigpitchcomp</t>
         </is>
       </c>
-      <c r="F102" s="2" t="inlineStr"/>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25055,7 +25299,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -25097,12 +25341,12 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -25139,7 +25383,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -25181,7 +25425,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -25223,7 +25467,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -25265,7 +25509,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -25307,7 +25551,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -25349,7 +25593,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -25391,7 +25635,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -25431,7 +25675,11 @@
           <t>https://www.calhacks.io/</t>
         </is>
       </c>
-      <c r="F112" s="2" t="inlineStr"/>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G112" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25471,7 +25719,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -25513,7 +25761,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -25555,7 +25803,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -25595,7 +25843,11 @@
           <t>https://cerebralvalley.ai/events/san-francisco</t>
         </is>
       </c>
-      <c r="F116" s="2" t="inlineStr"/>
+      <c r="F116" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -25635,7 +25887,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -25677,7 +25929,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -25719,7 +25971,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -25761,7 +26013,7 @@
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G120" s="2" t="inlineStr">
@@ -25803,7 +26055,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -25845,7 +26097,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -25887,7 +26139,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -25929,7 +26181,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -25971,7 +26223,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -26013,7 +26265,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -26056,7 +26308,7 @@
       <c r="F127" s="2" t="inlineStr"/>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -26093,7 +26345,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -26135,7 +26387,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -26177,7 +26429,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -26215,7 +26467,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -26257,7 +26509,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -26299,7 +26551,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -26341,7 +26593,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -26383,7 +26635,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -26425,7 +26677,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -26467,7 +26719,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -26509,7 +26761,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -26551,7 +26803,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -26593,7 +26845,7 @@
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G140" s="2" t="inlineStr">
@@ -26635,7 +26887,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -26675,7 +26927,11 @@
           <t>https://hack.gt/</t>
         </is>
       </c>
-      <c r="F142" s="2" t="inlineStr"/>
+      <c r="F142" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G142" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26713,7 +26969,11 @@
           <t>https://www.hackprinceton.com/</t>
         </is>
       </c>
-      <c r="F143" s="2" t="inlineStr"/>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G143" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26751,7 +27011,11 @@
           <t>https://www.hackumass.com/</t>
         </is>
       </c>
-      <c r="F144" s="2" t="inlineStr"/>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26789,7 +27053,11 @@
           <t>https://hai.stanford.edu/research/research-opportunities</t>
         </is>
       </c>
-      <c r="F145" s="2" t="inlineStr"/>
+      <c r="F145" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26829,7 +27097,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -26871,7 +27139,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -26911,7 +27179,11 @@
           <t>https://www.harvardfac.org/hfac-citadel-pitch-comp</t>
         </is>
       </c>
-      <c r="F148" s="2" t="inlineStr"/>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G148" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26949,7 +27221,11 @@
           <t>https://hophacks.com/</t>
         </is>
       </c>
-      <c r="F149" s="2" t="inlineStr"/>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -26989,12 +27265,12 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -27031,7 +27307,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -27073,7 +27349,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -27115,7 +27391,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -27157,7 +27433,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -27199,7 +27475,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -27241,7 +27517,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -27283,7 +27559,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -27325,7 +27601,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -27367,7 +27643,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -27409,7 +27685,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -27451,7 +27727,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -27493,7 +27769,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -27535,7 +27811,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -27577,7 +27853,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -27617,7 +27893,11 @@
           <t>https://kingcenter.stanford.edu/opportunities/undergraduate-students/summer-full-time-undergraduate-research-fellow-program</t>
         </is>
       </c>
-      <c r="F165" s="2" t="inlineStr"/>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27657,7 +27937,7 @@
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G166" s="2" t="inlineStr">
@@ -27697,7 +27977,11 @@
           <t>https://www.lahacks.com/</t>
         </is>
       </c>
-      <c r="F167" s="2" t="inlineStr"/>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G167" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27735,7 +28019,11 @@
           <t>https://lanl.jobs/search/searchjobs?categoryid=7f2fb73c-b4e4-4644-a234-858a80163473</t>
         </is>
       </c>
-      <c r="F168" s="2" t="inlineStr"/>
+      <c r="F168" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27775,7 +28063,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -27817,7 +28105,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -27859,7 +28147,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -27901,7 +28189,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -27941,7 +28229,11 @@
           <t>https://mathdrp.stanford.edu/</t>
         </is>
       </c>
-      <c r="F173" s="2" t="inlineStr"/>
+      <c r="F173" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -27981,7 +28273,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -28023,7 +28315,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -28063,7 +28355,11 @@
           <t>https://miamioh.edu/fsb/departments/finance/stock-pitch.html</t>
         </is>
       </c>
-      <c r="F176" s="2" t="inlineStr"/>
+      <c r="F176" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G176" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28103,7 +28399,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -28145,7 +28441,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -28187,7 +28483,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -28227,7 +28523,11 @@
           <t>https://www.mlh.com/seasons/2027/events</t>
         </is>
       </c>
-      <c r="F180" s="2" t="inlineStr"/>
+      <c r="F180" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28265,7 +28565,11 @@
           <t>https://msandepro.stanford.edu/academic-year-research-experience-undergraduates</t>
         </is>
       </c>
-      <c r="F181" s="2" t="inlineStr"/>
+      <c r="F181" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G181" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28303,7 +28607,11 @@
           <t>https://msande.stanford.edu/research-impact/mse-student-research/research-experience-undergraduates</t>
         </is>
       </c>
-      <c r="F182" s="2" t="inlineStr"/>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G182" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28343,7 +28651,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -28385,7 +28693,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -28427,7 +28735,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -28469,7 +28777,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -28511,7 +28819,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -28553,12 +28861,12 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
@@ -28593,7 +28901,11 @@
           <t>https://physics.stanford.edu/undergraduate/undergraduate-research</t>
         </is>
       </c>
-      <c r="F189" s="2" t="inlineStr"/>
+      <c r="F189" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28633,7 +28945,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -28673,7 +28985,11 @@
           <t>https://princetonstockpitch.vercel.app/</t>
         </is>
       </c>
-      <c r="F191" s="2" t="inlineStr"/>
+      <c r="F191" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -28713,7 +29029,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -28755,7 +29071,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -28797,7 +29113,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -28839,7 +29155,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -28881,7 +29197,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -28923,7 +29239,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -28965,7 +29281,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -29005,7 +29321,11 @@
           <t>https://www.sfhacks.io/</t>
         </is>
       </c>
-      <c r="F199" s="2" t="inlineStr"/>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G199" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29045,7 +29365,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -29085,7 +29405,11 @@
           <t>https://siepr.stanford.edu/programs/undergraduate-student-opportunities/undergraduate-research-fellows-program/academic-year</t>
         </is>
       </c>
-      <c r="F201" s="2" t="inlineStr"/>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G201" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29123,7 +29447,11 @@
           <t>https://siepr.stanford.edu/programs/undergraduate-student-opportunities/undergraduate-research-fellows-program/siepr-summer</t>
         </is>
       </c>
-      <c r="F202" s="2" t="inlineStr"/>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29161,7 +29489,11 @@
           <t>https://www.sjhacks.com/</t>
         </is>
       </c>
-      <c r="F203" s="2" t="inlineStr"/>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29201,7 +29533,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -29243,7 +29575,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -29286,7 +29618,7 @@
       <c r="F206" s="2" t="inlineStr"/>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -29323,7 +29655,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -29365,7 +29697,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -29405,7 +29737,11 @@
           <t>https://symsys.stanford.edu/opportunities/research/summer-undergraduate-research-symbolic-systems</t>
         </is>
       </c>
-      <c r="F209" s="2" t="inlineStr"/>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29443,7 +29779,11 @@
           <t>https://www.texasusit.org/competitions-overviews</t>
         </is>
       </c>
-      <c r="F210" s="2" t="inlineStr"/>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29483,7 +29823,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -29525,7 +29865,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -29567,7 +29907,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -29609,7 +29949,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -29651,7 +29991,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -29693,7 +30033,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -29733,7 +30073,11 @@
           <t>https://www.tbc.uchicago.edu/pitch-competition</t>
         </is>
       </c>
-      <c r="F217" s="2" t="inlineStr"/>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G217" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29773,7 +30117,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -29813,7 +30157,11 @@
           <t>https://www.umichuic.com/</t>
         </is>
       </c>
-      <c r="F219" s="2" t="inlineStr"/>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G219" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29853,7 +30201,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -29895,12 +30243,12 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:42:32+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr">
@@ -29935,7 +30283,11 @@
           <t>https://undergradresearch.stanford.edu/fund-your-project/explore-departmental-funding</t>
         </is>
       </c>
-      <c r="F222" s="2" t="inlineStr"/>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G222" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -29975,7 +30327,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -30017,7 +30369,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -30057,7 +30409,11 @@
           <t>https://www.pennwitg.com/competition</t>
         </is>
       </c>
-      <c r="F225" s="2" t="inlineStr"/>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G225" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -30097,7 +30453,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -30139,7 +30495,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -30179,7 +30535,11 @@
           <t>https://www.yhack.org/</t>
         </is>
       </c>
-      <c r="F228" s="2" t="inlineStr"/>
+      <c r="F228" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09T14:37:00+00:00</t>
+        </is>
+      </c>
       <c r="G228" s="2" t="inlineStr">
         <is>
           <t>0</t>
@@ -30219,7 +30579,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -30261,7 +30621,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -30303,7 +30663,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -30341,7 +30701,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -30383,7 +30743,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -30421,7 +30781,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -30463,7 +30823,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -30505,7 +30865,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -30543,7 +30903,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -30581,7 +30941,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -30619,7 +30979,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -30657,7 +31017,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -30695,7 +31055,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -30733,7 +31093,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -30776,7 +31136,7 @@
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr">
@@ -30814,7 +31174,7 @@
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
@@ -30851,7 +31211,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -30893,7 +31253,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -30931,7 +31291,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -30969,7 +31329,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -31007,7 +31367,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -31045,7 +31405,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -31083,7 +31443,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-09T14:37:00+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">

</xml_diff>

<commit_message>
state: 2026-10-10 upstream changes detected
</commit_message>
<xml_diff>
--- a/out/tracked.xlsx
+++ b/out/tracked.xlsx
@@ -1006,7 +1006,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -1170,7 +1170,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
@@ -3794,7 +3794,7 @@
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="J69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr"/>
@@ -4234,7 +4234,7 @@
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
@@ -4298,7 +4298,7 @@
       </c>
       <c r="J72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -4366,7 +4366,7 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
@@ -4430,7 +4430,7 @@
       </c>
       <c r="J74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
@@ -4598,7 +4598,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
@@ -5122,7 +5122,7 @@
       </c>
       <c r="J87" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr"/>
@@ -6501,17 +6501,17 @@
       </c>
       <c r="I114" s="2" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>open</t>
         </is>
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:25:47+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L114" s="2" t="inlineStr"/>
@@ -6522,7 +6522,7 @@
       </c>
       <c r="N114" s="2" t="inlineStr">
         <is>
-          <t>6b57b6d45119bce4b9c57e0b98d5f324efd8b16950e41e2d4023b2da03de8a0e</t>
+          <t>c9eeeca6895d5ef3de5570fe0f5140c10370d30499177d7fd68d450803b44d05</t>
         </is>
       </c>
     </row>
@@ -6678,7 +6678,7 @@
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
@@ -6742,7 +6742,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="J119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
@@ -7026,7 +7026,7 @@
       </c>
       <c r="J123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K123" s="2" t="inlineStr"/>
@@ -7242,7 +7242,7 @@
       </c>
       <c r="J127" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr"/>
@@ -8010,7 +8010,7 @@
       </c>
       <c r="J142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
@@ -8074,12 +8074,12 @@
       </c>
       <c r="J143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L143" s="2" t="inlineStr"/>
@@ -8090,7 +8090,7 @@
       </c>
       <c r="N143" s="2" t="inlineStr">
         <is>
-          <t>fa93f8d76ea09413cc7c718ed451b26c26ad2d228c00e765d59475f203efec16</t>
+          <t>826b577fecaf22bbf65c9544168d1dd82dd44e910b60182e7014015b6c62f6e3</t>
         </is>
       </c>
     </row>
@@ -8142,7 +8142,7 @@
       </c>
       <c r="J144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr">
@@ -8210,7 +8210,7 @@
       </c>
       <c r="J145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="J146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K146" s="2" t="inlineStr"/>
@@ -8610,7 +8610,7 @@
       </c>
       <c r="J152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="J153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K153" s="2" t="inlineStr">
@@ -8750,7 +8750,7 @@
       </c>
       <c r="J154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
@@ -8878,7 +8878,7 @@
       </c>
       <c r="J156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K156" s="2" t="inlineStr"/>
@@ -8946,12 +8946,12 @@
       </c>
       <c r="J157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L157" s="2" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="N157" s="2" t="inlineStr">
         <is>
-          <t>2fc8ac2223271ae6acdb0190db9faae5c00a54a8c4e19384fe8d05ea732ea516</t>
+          <t>77ba24c4ad1d8b1fa0465ee32d5ff183763e6a2684ad829796c59ca1a20eebcf</t>
         </is>
       </c>
     </row>
@@ -9018,7 +9018,7 @@
       </c>
       <c r="J158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K158" s="2" t="inlineStr"/>
@@ -10710,7 +10710,7 @@
       </c>
       <c r="J188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K188" s="2" t="inlineStr"/>
@@ -10890,7 +10890,7 @@
       </c>
       <c r="J191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K191" s="2" t="inlineStr"/>
@@ -10958,7 +10958,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -11030,12 +11030,12 @@
       </c>
       <c r="J193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L193" s="2" t="inlineStr">
@@ -11050,7 +11050,7 @@
       </c>
       <c r="N193" s="2" t="inlineStr">
         <is>
-          <t>ba5c2a7269bd068d12484a0639e74d3481f622b69c856afc6f3d79d402dfd31e</t>
+          <t>c6428ad2e363473f019e0d99586e6f8557f8e6aa31b3ab110f475e98f64e9fea</t>
         </is>
       </c>
     </row>
@@ -11102,7 +11102,7 @@
       </c>
       <c r="J194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K194" s="2" t="inlineStr">
@@ -11174,7 +11174,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">
@@ -11246,12 +11246,12 @@
       </c>
       <c r="J196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L196" s="2" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="N196" s="2" t="inlineStr">
         <is>
-          <t>c738a28ca945b73ae10dbac861a04080b088fd5f46f7f61fd249e436264ab5fb</t>
+          <t>5d3931b51d7fb11073b8907fc7cfa1e20083c39adf7a2ed8ff67d00713e6ba95</t>
         </is>
       </c>
     </row>
@@ -11318,7 +11318,7 @@
       </c>
       <c r="J197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K197" s="2" t="inlineStr">
@@ -11390,7 +11390,7 @@
       </c>
       <c r="J198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K198" s="2" t="inlineStr"/>
@@ -11458,7 +11458,7 @@
       </c>
       <c r="J199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K199" s="2" t="inlineStr"/>
@@ -11526,7 +11526,7 @@
       </c>
       <c r="J200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K200" s="2" t="inlineStr"/>
@@ -11594,7 +11594,7 @@
       </c>
       <c r="J201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K201" s="2" t="inlineStr">
@@ -11666,7 +11666,7 @@
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr"/>
@@ -11734,7 +11734,7 @@
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
@@ -11806,7 +11806,7 @@
       </c>
       <c r="J204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K204" s="2" t="inlineStr">
@@ -11878,7 +11878,7 @@
       </c>
       <c r="J205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K205" s="2" t="inlineStr"/>
@@ -12010,12 +12010,12 @@
       </c>
       <c r="J207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L207" s="2" t="inlineStr">
@@ -12030,7 +12030,7 @@
       </c>
       <c r="N207" s="2" t="inlineStr">
         <is>
-          <t>06087b9e6a42cd27c16a90c9604b634af5ed9e643e26c0d5a61830976615ff5d</t>
+          <t>abdcb5c9c9ba2fec3bbc78a104a53261117b2fc19cc2510708187da1cc60737f</t>
         </is>
       </c>
     </row>
@@ -12082,7 +12082,7 @@
       </c>
       <c r="J208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K208" s="2" t="inlineStr"/>
@@ -12150,7 +12150,7 @@
       </c>
       <c r="J209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K209" s="2" t="inlineStr">
@@ -12222,7 +12222,7 @@
       </c>
       <c r="J210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K210" s="2" t="inlineStr"/>
@@ -12518,7 +12518,7 @@
       </c>
       <c r="J215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K215" s="2" t="inlineStr"/>
@@ -12766,7 +12766,7 @@
       </c>
       <c r="J219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K219" s="2" t="inlineStr"/>
@@ -12834,7 +12834,7 @@
       </c>
       <c r="J220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K220" s="2" t="inlineStr"/>
@@ -12902,7 +12902,7 @@
       </c>
       <c r="J221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K221" s="2" t="inlineStr">
@@ -13094,7 +13094,7 @@
       </c>
       <c r="J224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K224" s="2" t="inlineStr"/>
@@ -13162,7 +13162,7 @@
       </c>
       <c r="J225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K225" s="2" t="inlineStr"/>
@@ -13230,7 +13230,7 @@
       </c>
       <c r="J226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K226" s="2" t="inlineStr"/>
@@ -13298,7 +13298,7 @@
       </c>
       <c r="J227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K227" s="2" t="inlineStr"/>
@@ -13366,7 +13366,7 @@
       </c>
       <c r="J228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K228" s="2" t="inlineStr"/>
@@ -13434,7 +13434,7 @@
       </c>
       <c r="J229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K229" s="2" t="inlineStr"/>
@@ -13558,10 +13558,14 @@
       </c>
       <c r="J231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
-        </is>
-      </c>
-      <c r="K231" s="2" t="inlineStr"/>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
+      <c r="K231" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
       <c r="L231" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -13574,7 +13578,7 @@
       </c>
       <c r="N231" s="2" t="inlineStr">
         <is>
-          <t>7aac9d9c52a684d194f84c75ea15e8b14fb3a13a5f54f735261a8d39b6d4af67</t>
+          <t>a55a21f9c39028df1294608bfa4eea59bcb8dbf9cd3fc8ac33b197e038e27e34</t>
         </is>
       </c>
     </row>
@@ -13626,7 +13630,7 @@
       </c>
       <c r="J232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K232" s="2" t="inlineStr"/>
@@ -13866,7 +13870,7 @@
       </c>
       <c r="J236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K236" s="2" t="inlineStr"/>
@@ -18134,7 +18138,7 @@
       </c>
       <c r="J312" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K312" s="2" t="inlineStr">
@@ -18206,10 +18210,14 @@
       </c>
       <c r="J313" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
-        </is>
-      </c>
-      <c r="K313" s="2" t="inlineStr"/>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
+      <c r="K313" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
       <c r="L313" s="2" t="inlineStr">
         <is>
           <t>2026-10-01</t>
@@ -18222,7 +18230,7 @@
       </c>
       <c r="N313" s="2" t="inlineStr">
         <is>
-          <t>760fd1e652f7d1a0967c79c08ce0ec746ef0663e9352d0491c7bf0b00e2688a6</t>
+          <t>13ddb9df9d2cc52fea3f018ba916c3df659388776543d7a21e93141cc8810e77</t>
         </is>
       </c>
     </row>
@@ -18274,7 +18282,7 @@
       </c>
       <c r="J314" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K314" s="2" t="inlineStr">
@@ -18346,7 +18354,7 @@
       </c>
       <c r="J315" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K315" s="2" t="inlineStr"/>
@@ -18414,7 +18422,7 @@
       </c>
       <c r="J316" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K316" s="2" t="inlineStr"/>
@@ -18482,7 +18490,7 @@
       </c>
       <c r="J317" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K317" s="2" t="inlineStr"/>
@@ -18606,7 +18614,7 @@
       </c>
       <c r="J319" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K319" s="2" t="inlineStr"/>
@@ -19034,7 +19042,7 @@
       </c>
       <c r="J326" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K326" s="2" t="inlineStr"/>
@@ -19102,7 +19110,7 @@
       </c>
       <c r="J327" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K327" s="2" t="inlineStr"/>
@@ -19170,7 +19178,7 @@
       </c>
       <c r="J328" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K328" s="2" t="inlineStr"/>
@@ -19238,12 +19246,12 @@
       </c>
       <c r="J329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K329" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L329" s="2" t="inlineStr">
@@ -19258,7 +19266,7 @@
       </c>
       <c r="N329" s="2" t="inlineStr">
         <is>
-          <t>e7d3380f7da6ba01188e2a946c522701b458faccfe24f80bf9ee0779fb949048</t>
+          <t>689ff0a10ae8a53468c66dd085c3c06b3e1b65ddcbafd123f1d16236198a2d97</t>
         </is>
       </c>
     </row>
@@ -19310,12 +19318,12 @@
       </c>
       <c r="J330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K330" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L330" s="2" t="inlineStr">
@@ -19330,7 +19338,7 @@
       </c>
       <c r="N330" s="2" t="inlineStr">
         <is>
-          <t>3364770d8ef21d5b502b30b49d73d867654fa68a942a212dbde11eaeb01b3b2d</t>
+          <t>65ecd7c7d703437fcf068b759971925488a3d670b656c1377a2a8bb6da1e33f6</t>
         </is>
       </c>
     </row>
@@ -19382,12 +19390,12 @@
       </c>
       <c r="J331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K331" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="L331" s="2" t="inlineStr">
@@ -19402,7 +19410,7 @@
       </c>
       <c r="N331" s="2" t="inlineStr">
         <is>
-          <t>c831be1f7e407c8962f45bd4f14f4398a8d8fc22fba3472377c75ffedbfbec77</t>
+          <t>37efc8c16173ea0352bc660d406f5c88a1553f458978f2f841e0d7e647eff8c8</t>
         </is>
       </c>
     </row>
@@ -19454,7 +19462,7 @@
       </c>
       <c r="J332" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K332" s="2" t="inlineStr"/>
@@ -19578,7 +19586,7 @@
       </c>
       <c r="J334" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K334" s="2" t="inlineStr"/>
@@ -19646,7 +19654,7 @@
       </c>
       <c r="J335" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K335" s="2" t="inlineStr"/>
@@ -19714,7 +19722,7 @@
       </c>
       <c r="J336" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K336" s="2" t="inlineStr"/>
@@ -19782,7 +19790,7 @@
       </c>
       <c r="J337" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K337" s="2" t="inlineStr"/>
@@ -19850,7 +19858,7 @@
       </c>
       <c r="J338" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K338" s="2" t="inlineStr"/>
@@ -19918,7 +19926,7 @@
       </c>
       <c r="J339" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K339" s="2" t="inlineStr"/>
@@ -19986,7 +19994,7 @@
       </c>
       <c r="J340" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K340" s="2" t="inlineStr"/>
@@ -20054,7 +20062,7 @@
       </c>
       <c r="J341" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K341" s="2" t="inlineStr"/>
@@ -20122,10 +20130,14 @@
       </c>
       <c r="J342" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
-        </is>
-      </c>
-      <c r="K342" s="2" t="inlineStr"/>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
+      <c r="K342" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-10T13:51:10+00:00</t>
+        </is>
+      </c>
       <c r="L342" s="2" t="inlineStr">
         <is>
           <t>2026-10-08</t>
@@ -20138,7 +20150,7 @@
       </c>
       <c r="N342" s="2" t="inlineStr">
         <is>
-          <t>6f3864cfea788dfa8383a47e55d90a3a1a684cd1949baf8f248c58b7d54de7b3</t>
+          <t>9b6c8fad2b0c95f685bac8bf6d888e13b5d47c583146a86af8b847c5d3f17d6a</t>
         </is>
       </c>
     </row>
@@ -20306,7 +20318,7 @@
       </c>
       <c r="J345" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K345" s="2" t="inlineStr"/>
@@ -20374,7 +20386,7 @@
       </c>
       <c r="J346" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K346" s="2" t="inlineStr"/>
@@ -20442,7 +20454,7 @@
       </c>
       <c r="J347" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K347" s="2" t="inlineStr"/>
@@ -20510,7 +20522,7 @@
       </c>
       <c r="J348" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K348" s="2" t="inlineStr"/>
@@ -20578,7 +20590,7 @@
       </c>
       <c r="J349" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K349" s="2" t="inlineStr"/>
@@ -20646,7 +20658,7 @@
       </c>
       <c r="J350" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K350" s="2" t="inlineStr"/>
@@ -20714,7 +20726,7 @@
       </c>
       <c r="J351" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K351" s="2" t="inlineStr"/>
@@ -20782,7 +20794,7 @@
       </c>
       <c r="J352" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="K352" s="2" t="inlineStr"/>
@@ -21241,7 +21253,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -21279,7 +21291,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -21321,7 +21333,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -21359,7 +21371,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -21397,7 +21409,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -21435,7 +21447,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -21473,7 +21485,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -21515,7 +21527,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -21553,7 +21565,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -21595,7 +21607,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -21637,7 +21649,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -21679,7 +21691,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -21721,7 +21733,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -21763,7 +21775,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -21805,7 +21817,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -21847,7 +21859,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -21889,7 +21901,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -21931,7 +21943,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -21973,7 +21985,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -22015,7 +22027,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -22057,7 +22069,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -22099,7 +22111,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -22137,7 +22149,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -22179,7 +22191,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
@@ -22217,7 +22229,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -22259,7 +22271,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
@@ -22301,7 +22313,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -22343,7 +22355,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -22385,7 +22397,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
@@ -22427,7 +22439,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -22465,7 +22477,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
@@ -22503,7 +22515,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
@@ -22541,7 +22553,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -22583,7 +22595,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -22625,7 +22637,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -22663,7 +22675,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -22701,7 +22713,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -22743,7 +22755,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -22781,7 +22793,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -22823,7 +22835,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -22861,7 +22873,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -22899,7 +22911,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -22941,7 +22953,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -22979,7 +22991,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
@@ -23017,7 +23029,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
@@ -23055,7 +23067,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -23097,7 +23109,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -23135,7 +23147,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -23177,7 +23189,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -23219,7 +23231,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -23261,7 +23273,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -23303,7 +23315,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -23341,7 +23353,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -23379,7 +23391,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
@@ -23417,7 +23429,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -23459,7 +23471,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
@@ -23497,7 +23509,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -23539,7 +23551,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr">
@@ -23581,7 +23593,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -23619,7 +23631,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -23661,7 +23673,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
@@ -23703,7 +23715,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr">
@@ -23741,7 +23753,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
@@ -23783,7 +23795,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -23821,7 +23833,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
@@ -23863,7 +23875,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
@@ -23905,7 +23917,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
@@ -23947,7 +23959,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
@@ -23985,7 +23997,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -24023,7 +24035,7 @@
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr">
@@ -24061,7 +24073,7 @@
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
@@ -24099,7 +24111,7 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
@@ -24137,7 +24149,7 @@
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr">
@@ -24179,7 +24191,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -24217,7 +24229,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -24255,7 +24267,7 @@
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -24297,7 +24309,7 @@
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr">
@@ -24335,7 +24347,7 @@
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -24377,7 +24389,7 @@
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr">
@@ -24415,7 +24427,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr">
@@ -24457,7 +24469,7 @@
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
@@ -24495,7 +24507,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -24533,7 +24545,7 @@
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr">
@@ -24575,7 +24587,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -24921,7 +24933,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -24963,7 +24975,7 @@
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr">
@@ -25005,7 +25017,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -25047,7 +25059,7 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
@@ -25089,7 +25101,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -25131,7 +25143,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -25173,7 +25185,7 @@
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G100" s="2" t="inlineStr">
@@ -25215,7 +25227,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -25257,7 +25269,7 @@
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G102" s="2" t="inlineStr">
@@ -25299,7 +25311,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -25341,7 +25353,7 @@
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G104" s="2" t="inlineStr">
@@ -25383,7 +25395,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -25425,7 +25437,7 @@
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G106" s="2" t="inlineStr">
@@ -25467,7 +25479,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -25509,7 +25521,7 @@
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G108" s="2" t="inlineStr">
@@ -25551,7 +25563,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -25593,7 +25605,7 @@
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G110" s="2" t="inlineStr">
@@ -25635,7 +25647,7 @@
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G111" s="2" t="inlineStr">
@@ -25677,7 +25689,7 @@
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G112" s="2" t="inlineStr">
@@ -25719,7 +25731,7 @@
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G113" s="2" t="inlineStr">
@@ -25761,7 +25773,7 @@
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G114" s="2" t="inlineStr">
@@ -25803,7 +25815,7 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
@@ -25845,7 +25857,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -25887,7 +25899,7 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
@@ -25929,7 +25941,7 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
@@ -25971,7 +25983,7 @@
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G119" s="2" t="inlineStr">
@@ -26018,7 +26030,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -26055,7 +26067,7 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
@@ -26097,7 +26109,7 @@
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G122" s="2" t="inlineStr">
@@ -26139,7 +26151,7 @@
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G123" s="2" t="inlineStr">
@@ -26181,7 +26193,7 @@
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G124" s="2" t="inlineStr">
@@ -26223,7 +26235,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -26265,7 +26277,7 @@
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G126" s="2" t="inlineStr">
@@ -26308,7 +26320,7 @@
       <c r="F127" s="2" t="inlineStr"/>
       <c r="G127" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H127" s="2" t="inlineStr">
@@ -26345,7 +26357,7 @@
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G128" s="2" t="inlineStr">
@@ -26387,7 +26399,7 @@
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G129" s="2" t="inlineStr">
@@ -26429,7 +26441,7 @@
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G130" s="2" t="inlineStr">
@@ -26467,7 +26479,7 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
@@ -26509,7 +26521,7 @@
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G132" s="2" t="inlineStr">
@@ -26551,7 +26563,7 @@
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G133" s="2" t="inlineStr">
@@ -26593,7 +26605,7 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
@@ -26635,7 +26647,7 @@
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
@@ -26677,7 +26689,7 @@
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G136" s="2" t="inlineStr">
@@ -26719,7 +26731,7 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
@@ -26761,7 +26773,7 @@
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G138" s="2" t="inlineStr">
@@ -26803,7 +26815,7 @@
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G139" s="2" t="inlineStr">
@@ -26850,7 +26862,7 @@
       </c>
       <c r="G140" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H140" s="2" t="inlineStr">
@@ -26887,7 +26899,7 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
@@ -26929,7 +26941,7 @@
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G142" s="2" t="inlineStr">
@@ -26971,7 +26983,7 @@
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G143" s="2" t="inlineStr">
@@ -27013,7 +27025,7 @@
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G144" s="2" t="inlineStr">
@@ -27055,7 +27067,7 @@
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G145" s="2" t="inlineStr">
@@ -27097,7 +27109,7 @@
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G146" s="2" t="inlineStr">
@@ -27139,7 +27151,7 @@
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G147" s="2" t="inlineStr">
@@ -27181,7 +27193,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -27223,7 +27235,7 @@
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G149" s="2" t="inlineStr">
@@ -27265,7 +27277,7 @@
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G150" s="2" t="inlineStr">
@@ -27307,7 +27319,7 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
@@ -27349,7 +27361,7 @@
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G152" s="2" t="inlineStr">
@@ -27391,7 +27403,7 @@
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G153" s="2" t="inlineStr">
@@ -27433,7 +27445,7 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
@@ -27475,7 +27487,7 @@
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G155" s="2" t="inlineStr">
@@ -27517,7 +27529,7 @@
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G156" s="2" t="inlineStr">
@@ -27559,7 +27571,7 @@
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
@@ -27601,7 +27613,7 @@
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G158" s="2" t="inlineStr">
@@ -27643,7 +27655,7 @@
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G159" s="2" t="inlineStr">
@@ -27685,7 +27697,7 @@
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G160" s="2" t="inlineStr">
@@ -27727,7 +27739,7 @@
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G161" s="2" t="inlineStr">
@@ -27769,7 +27781,7 @@
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G162" s="2" t="inlineStr">
@@ -27811,7 +27823,7 @@
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G163" s="2" t="inlineStr">
@@ -27853,7 +27865,7 @@
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G164" s="2" t="inlineStr">
@@ -27895,7 +27907,7 @@
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G165" s="2" t="inlineStr">
@@ -27942,7 +27954,7 @@
       </c>
       <c r="G166" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H166" s="2" t="inlineStr">
@@ -27979,7 +27991,7 @@
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G167" s="2" t="inlineStr">
@@ -28021,7 +28033,7 @@
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G168" s="2" t="inlineStr">
@@ -28063,7 +28075,7 @@
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G169" s="2" t="inlineStr">
@@ -28105,7 +28117,7 @@
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G170" s="2" t="inlineStr">
@@ -28147,7 +28159,7 @@
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G171" s="2" t="inlineStr">
@@ -28189,7 +28201,7 @@
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G172" s="2" t="inlineStr">
@@ -28231,7 +28243,7 @@
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G173" s="2" t="inlineStr">
@@ -28273,7 +28285,7 @@
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G174" s="2" t="inlineStr">
@@ -28315,7 +28327,7 @@
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G175" s="2" t="inlineStr">
@@ -28357,7 +28369,7 @@
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G176" s="2" t="inlineStr">
@@ -28399,7 +28411,7 @@
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G177" s="2" t="inlineStr">
@@ -28441,7 +28453,7 @@
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G178" s="2" t="inlineStr">
@@ -28483,7 +28495,7 @@
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G179" s="2" t="inlineStr">
@@ -28525,7 +28537,7 @@
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G180" s="2" t="inlineStr">
@@ -28567,7 +28579,7 @@
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G181" s="2" t="inlineStr">
@@ -28609,7 +28621,7 @@
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G182" s="2" t="inlineStr">
@@ -28651,7 +28663,7 @@
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G183" s="2" t="inlineStr">
@@ -28693,7 +28705,7 @@
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G184" s="2" t="inlineStr">
@@ -28735,7 +28747,7 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
@@ -28777,7 +28789,7 @@
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G186" s="2" t="inlineStr">
@@ -28819,7 +28831,7 @@
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G187" s="2" t="inlineStr">
@@ -28861,7 +28873,7 @@
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G188" s="2" t="inlineStr">
@@ -28903,7 +28915,7 @@
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G189" s="2" t="inlineStr">
@@ -28945,7 +28957,7 @@
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G190" s="2" t="inlineStr">
@@ -28987,7 +28999,7 @@
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G191" s="2" t="inlineStr">
@@ -29029,7 +29041,7 @@
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G192" s="2" t="inlineStr">
@@ -29071,7 +29083,7 @@
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G193" s="2" t="inlineStr">
@@ -29113,7 +29125,7 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
@@ -29155,7 +29167,7 @@
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G195" s="2" t="inlineStr">
@@ -29197,7 +29209,7 @@
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G196" s="2" t="inlineStr">
@@ -29239,7 +29251,7 @@
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G197" s="2" t="inlineStr">
@@ -29281,7 +29293,7 @@
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G198" s="2" t="inlineStr">
@@ -29323,7 +29335,7 @@
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G199" s="2" t="inlineStr">
@@ -29365,7 +29377,7 @@
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G200" s="2" t="inlineStr">
@@ -29407,7 +29419,7 @@
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G201" s="2" t="inlineStr">
@@ -29449,7 +29461,7 @@
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
@@ -29491,7 +29503,7 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
@@ -29533,7 +29545,7 @@
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
@@ -29575,7 +29587,7 @@
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
@@ -29618,7 +29630,7 @@
       <c r="F206" s="2" t="inlineStr"/>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
@@ -29655,7 +29667,7 @@
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
@@ -29697,7 +29709,7 @@
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
@@ -29739,7 +29751,7 @@
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
@@ -29781,7 +29793,7 @@
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
@@ -29823,7 +29835,7 @@
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G211" s="2" t="inlineStr">
@@ -29865,7 +29877,7 @@
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G212" s="2" t="inlineStr">
@@ -29907,7 +29919,7 @@
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G213" s="2" t="inlineStr">
@@ -29949,7 +29961,7 @@
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G214" s="2" t="inlineStr">
@@ -29991,7 +30003,7 @@
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G215" s="2" t="inlineStr">
@@ -30033,7 +30045,7 @@
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G216" s="2" t="inlineStr">
@@ -30075,7 +30087,7 @@
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G217" s="2" t="inlineStr">
@@ -30117,7 +30129,7 @@
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G218" s="2" t="inlineStr">
@@ -30159,7 +30171,7 @@
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G219" s="2" t="inlineStr">
@@ -30201,7 +30213,7 @@
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G220" s="2" t="inlineStr">
@@ -30243,7 +30255,7 @@
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G221" s="2" t="inlineStr">
@@ -30285,7 +30297,7 @@
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G222" s="2" t="inlineStr">
@@ -30327,7 +30339,7 @@
       </c>
       <c r="F223" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G223" s="2" t="inlineStr">
@@ -30369,7 +30381,7 @@
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G224" s="2" t="inlineStr">
@@ -30411,7 +30423,7 @@
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G225" s="2" t="inlineStr">
@@ -30453,7 +30465,7 @@
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G226" s="2" t="inlineStr">
@@ -30495,7 +30507,7 @@
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G227" s="2" t="inlineStr">
@@ -30537,7 +30549,7 @@
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G228" s="2" t="inlineStr">
@@ -30579,7 +30591,7 @@
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G229" s="2" t="inlineStr">
@@ -30621,7 +30633,7 @@
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G230" s="2" t="inlineStr">
@@ -30663,7 +30675,7 @@
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G231" s="2" t="inlineStr">
@@ -30701,7 +30713,7 @@
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G232" s="2" t="inlineStr">
@@ -30743,7 +30755,7 @@
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G233" s="2" t="inlineStr">
@@ -30781,7 +30793,7 @@
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G234" s="2" t="inlineStr">
@@ -30823,7 +30835,7 @@
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G235" s="2" t="inlineStr">
@@ -30865,7 +30877,7 @@
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G236" s="2" t="inlineStr">
@@ -30903,7 +30915,7 @@
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G237" s="2" t="inlineStr">
@@ -30941,7 +30953,7 @@
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G238" s="2" t="inlineStr">
@@ -30979,7 +30991,7 @@
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G239" s="2" t="inlineStr">
@@ -31017,7 +31029,7 @@
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G240" s="2" t="inlineStr">
@@ -31055,7 +31067,7 @@
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G241" s="2" t="inlineStr">
@@ -31093,7 +31105,7 @@
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G242" s="2" t="inlineStr">
@@ -31131,12 +31143,12 @@
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G243" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H243" s="2" t="inlineStr">
@@ -31169,12 +31181,12 @@
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
-          <t>2026-10-08T14:49:47+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G244" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H244" s="2" t="inlineStr">
@@ -31211,7 +31223,7 @@
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G245" s="2" t="inlineStr">
@@ -31253,7 +31265,7 @@
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G246" s="2" t="inlineStr">
@@ -31291,7 +31303,7 @@
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G247" s="2" t="inlineStr">
@@ -31329,7 +31341,7 @@
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G248" s="2" t="inlineStr">
@@ -31367,7 +31379,7 @@
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G249" s="2" t="inlineStr">
@@ -31405,7 +31417,7 @@
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G250" s="2" t="inlineStr">
@@ -31443,7 +31455,7 @@
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09T14:37:00+00:00</t>
+          <t>2026-10-10T13:51:10+00:00</t>
         </is>
       </c>
       <c r="G251" s="2" t="inlineStr">

</xml_diff>